<commit_message>
Updated Indicator calculations and added additional indicators
</commit_message>
<xml_diff>
--- a/Skupna tabela občine.xlsx
+++ b/Skupna tabela občine.xlsx
@@ -5,17 +5,17 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Desktop/Slovenija/Razširjeni kazalniki/streamlit_turisticne_regije_app_v4/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Desktop/Slovenija/Razširjeni kazalniki/streamlit app/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{976BB245-1900-1E49-B335-CCBCFD866476}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A94DDDA7-DAEF-3947-BF50-F00B1B973273}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="38700" yWindow="5240" windowWidth="33320" windowHeight="21620" xr2:uid="{855CFD84-EAB2-0A43-A92D-394EE615CEA5}"/>
+    <workbookView xWindow="21480" yWindow="14380" windowWidth="49940" windowHeight="34980" xr2:uid="{855CFD84-EAB2-0A43-A92D-394EE615CEA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Skupna Tabela" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1427" uniqueCount="315">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1429" uniqueCount="317">
   <si>
     <t>Občine</t>
   </si>
@@ -725,9 +725,6 @@
     <t>Povprečna starost prebivalcev</t>
   </si>
   <si>
-    <t>Število prebivalcev H2/2024)</t>
-  </si>
-  <si>
     <t>Površina območja (km2)</t>
   </si>
   <si>
@@ -743,25 +740,13 @@
     <t>Ocenjena povp. Letna zased. sob (nedeljivih enot)</t>
   </si>
   <si>
-    <t>Pritisk turizma na družbeni prostor</t>
-  </si>
-  <si>
     <t>Gostota turizma</t>
-  </si>
-  <si>
-    <t>Intenzivnost turizma</t>
   </si>
   <si>
     <t>Delovno aktivni v  turizmu (OECD/WTO)</t>
   </si>
   <si>
-    <t>Število zaposl. in samozaposl. V aktivnih podjetjih v Gostinstvu (I)</t>
-  </si>
-  <si>
     <t>Zaposleni v Gostinstvu (I) v registr.podjetjih in s.p.</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Zaposleni v nastan.dejav. (I55) v registr.podjetjih in s.p.</t>
   </si>
   <si>
     <t>Vsi delovni aktivni na območju</t>
@@ -821,9 +806,6 @@
     <t>Donosnost kapitala v reg. podjetjih in s.p. v Gostinstvu (I)</t>
   </si>
   <si>
-    <t>Dobičkovnost prihodkov v podjetjih in s.p. v Gostinstvu (I)21</t>
-  </si>
-  <si>
     <t>Število reg. podjetij in s.p. v nastanitveni dejav. (I 55)</t>
   </si>
   <si>
@@ -843,9 +825,6 @@
   </si>
   <si>
     <t>Delež stroškov dela v prihodkih v reg. podj. v nast.gost.dej. (I 55)</t>
-  </si>
-  <si>
-    <t>Delež stroškov dela v dod vredn. v reg. podj. v nast.gost.dej. (I)</t>
   </si>
   <si>
     <t>EBITDA v reg.podjetjih in s.p. v nastanitveni dejav. (I 55)</t>
@@ -870,15 +849,6 @@
   </si>
   <si>
     <t>Dobičkovnost prihodkov v nastanitveni dejav. (I 55)</t>
-  </si>
-  <si>
-    <t>Cel.prihodki v nastan. dejav. na prenočitev</t>
-  </si>
-  <si>
-    <t>Ocenjeni.prihodki iz nast. dejav. na prenočitev</t>
-  </si>
-  <si>
-    <t>Ocenj.prihodki iz nastan. dej. na razpoložljivo sobo (enoto)</t>
   </si>
   <si>
     <t>Ocenjeni prihodki iz nast.dej. na prodano sobo (ned.enoto)</t>
@@ -911,13 +881,7 @@
     <t>Povprečna neto plača izplačana na zaposl. osebo v Gostinstvu (I)</t>
   </si>
   <si>
-    <t xml:space="preserve"> Indeks neto plača v Gostinstvu (I) /pvp. plača v vseh dejavnostih</t>
-  </si>
-  <si>
     <t>Število izdanih gradbenih dovoljenj/1000 prebivalcev</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> Število počitniških stanovanj</t>
   </si>
   <si>
     <t>Delež naseljenih stanovanj od vseh razp.</t>
@@ -941,16 +905,10 @@
     <t>Prihodi turistov SKUPAJ</t>
   </si>
   <si>
-    <t>Prihodi turistov Domaći</t>
-  </si>
-  <si>
     <t>Prihodi turistov Tuji</t>
   </si>
   <si>
     <t>PDB turistov	SKUPAJ</t>
-  </si>
-  <si>
-    <t>PDB turistov	Domaći</t>
   </si>
   <si>
     <t>PDB turistov	Tuji</t>
@@ -981,6 +939,54 @@
   </si>
   <si>
     <t>Struktura nastanitvenih kapacitet - Stalna ležišča - Druge vrste kapacitet</t>
+  </si>
+  <si>
+    <t>Število prebivalcev (H2/2024)</t>
+  </si>
+  <si>
+    <t>Prihodi turistov Domači</t>
+  </si>
+  <si>
+    <t>PDB turistov	Domači</t>
+  </si>
+  <si>
+    <t>Število zaposl. in samozaposl. v aktivnih podjetjih v Gostinstvu (I)</t>
+  </si>
+  <si>
+    <t>Dobičkovnost prihodkov v podjetjih in s.p. v Gostinstvu (I)</t>
+  </si>
+  <si>
+    <t>Delež stroškov dela v dod vredn. v reg. podj. v nast.gost.dej. (I 55)</t>
+  </si>
+  <si>
+    <t>Pritisk turizma na družbeni prostor (število stalnih ležišč / 100 prebivalcev)</t>
+  </si>
+  <si>
+    <t>Intenzivnost turizma (število nočitev na dan / 100 prebivalcev)</t>
+  </si>
+  <si>
+    <t>Zaposleni v nastan.dejav. (I55) v registr.podjetjih in s.p.</t>
+  </si>
+  <si>
+    <t>Celotni prihodki v nastan. dejav. na prenočitev</t>
+  </si>
+  <si>
+    <t>Ocenjeni prihodki iz nastan. dej. na razpoložljivo sobo (enoto)</t>
+  </si>
+  <si>
+    <t>Ocenjeni prihodki iz nast. dejav. na prenočitev</t>
+  </si>
+  <si>
+    <t>Indeks neto plača v Gostinstvu (I) /pvp. plača v vseh dejavnostih</t>
+  </si>
+  <si>
+    <t>Število počitniških stanovanj</t>
+  </si>
+  <si>
+    <t>Delež naseljenih stanovanj</t>
+  </si>
+  <si>
+    <t>Število vseh stanovanj</t>
   </si>
 </sst>
 </file>
@@ -1041,13 +1047,13 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B15064BA-5E36-434F-9555-4D01A0E03380}" name="Table1" displayName="Table1" ref="A1:CL214" totalsRowShown="0">
-  <autoFilter ref="A1:CL214" xr:uid="{B15064BA-5E36-434F-9555-4D01A0E03380}"/>
-  <tableColumns count="90">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{B15064BA-5E36-434F-9555-4D01A0E03380}" name="Table1" displayName="Table1" ref="A1:CN214" totalsRowShown="0">
+  <autoFilter ref="A1:CN214" xr:uid="{B15064BA-5E36-434F-9555-4D01A0E03380}"/>
+  <tableColumns count="92">
     <tableColumn id="1" xr3:uid="{C7C32248-C834-9C44-AFE7-AB13CDAAE424}" name="Občine"/>
     <tableColumn id="2" xr3:uid="{C4443C77-0C1D-3441-8686-6D6A33F6AF30}" name="Turistična regija"/>
     <tableColumn id="3" xr3:uid="{9C93C5AB-E721-1A4A-90F2-B3397080611D}" name="Površina območja (km2)"/>
-    <tableColumn id="4" xr3:uid="{6A516117-D02C-9042-BED8-A834718FD32E}" name="Število prebivalcev H2/2024)"/>
+    <tableColumn id="4" xr3:uid="{6A516117-D02C-9042-BED8-A834718FD32E}" name="Število prebivalcev (H2/2024)"/>
     <tableColumn id="5" xr3:uid="{91CEC2B5-9950-E340-9265-15A390DF7689}" name="Povprečna starost prebivalcev"/>
     <tableColumn id="6" xr3:uid="{FB5CAD11-15F3-A24F-9CAF-8E64EAD3A48D}" name="Naravni prirast /1000 prebival."/>
     <tableColumn id="7" xr3:uid="{E209E213-8FD4-4C47-B297-1F887AE8D7A7}" name="Prenočitve turistov SKUPAJ" dataDxfId="0"/>
@@ -1055,10 +1061,10 @@
     <tableColumn id="9" xr3:uid="{F2E07E25-D318-EF4C-9D58-4F9D024FA8A8}" name="Prenočitve turistov_x0009_Tuji"/>
     <tableColumn id="10" xr3:uid="{AE7EC853-0402-A44C-9F12-18D82AF38827}" name="Delež tujih prenočitev"/>
     <tableColumn id="11" xr3:uid="{5CF30DCA-BA0F-D047-9308-6222A89F2E07}" name="Prihodi turistov SKUPAJ"/>
-    <tableColumn id="12" xr3:uid="{2608AA17-F184-2D44-B158-EC683F751D56}" name="Prihodi turistov Domaći"/>
+    <tableColumn id="12" xr3:uid="{2608AA17-F184-2D44-B158-EC683F751D56}" name="Prihodi turistov Domači"/>
     <tableColumn id="13" xr3:uid="{D040950F-FE38-AF40-AC39-E818CABE1FE1}" name="Prihodi turistov Tuji"/>
     <tableColumn id="14" xr3:uid="{494C63A2-19AC-0544-861F-B7FA12714240}" name="PDB turistov_x0009_SKUPAJ"/>
-    <tableColumn id="15" xr3:uid="{A743FB1C-E3E3-8340-BA42-61AD9082C50D}" name="PDB turistov_x0009_Domaći"/>
+    <tableColumn id="15" xr3:uid="{A743FB1C-E3E3-8340-BA42-61AD9082C50D}" name="PDB turistov_x0009_Domači"/>
     <tableColumn id="16" xr3:uid="{D6397E34-AE62-1B40-8641-B68E90F526C0}" name="PDB turistov_x0009_Tuji"/>
     <tableColumn id="17" xr3:uid="{FF46E309-259F-F74C-B4E3-7DF480EC498E}" name="Nastanitvene kapacitete - Nedeljive enote"/>
     <tableColumn id="18" xr3:uid="{DFA7A743-7B9B-AC4B-B555-AB008106AD20}" name="Nastanitvene kapacitete - vsa ležišča"/>
@@ -1072,13 +1078,13 @@
     <tableColumn id="26" xr3:uid="{6B98A6DD-4A64-EE45-AE54-458C05388214}" name="Delež stalnih ležišč v Hotelih ipd."/>
     <tableColumn id="27" xr3:uid="{CC3F87E6-B3CD-E841-BCED-E5C77DFA385B}" name="Povprečna letna zasedenost staln. ležišč"/>
     <tableColumn id="28" xr3:uid="{36E12EEC-F431-7640-B38F-3F28A52A27A2}" name="Ocenjena povp. Letna zased. sob (nedeljivih enot)"/>
-    <tableColumn id="29" xr3:uid="{E32E1653-4218-8144-AE1B-7DA0234BDD6B}" name="Pritisk turizma na družbeni prostor"/>
+    <tableColumn id="29" xr3:uid="{E32E1653-4218-8144-AE1B-7DA0234BDD6B}" name="Pritisk turizma na družbeni prostor (število stalnih ležišč / 100 prebivalcev)"/>
     <tableColumn id="30" xr3:uid="{6235832E-2F71-6247-9BC2-BB497EF940F1}" name="Gostota turizma"/>
-    <tableColumn id="31" xr3:uid="{6059D037-013F-3443-92BE-556256221BB9}" name="Intenzivnost turizma"/>
+    <tableColumn id="31" xr3:uid="{6059D037-013F-3443-92BE-556256221BB9}" name="Intenzivnost turizma (število nočitev na dan / 100 prebivalcev)"/>
     <tableColumn id="32" xr3:uid="{0EC9E9BB-E7DF-8F40-8DAC-C329014153B6}" name="Delovno aktivni v  turizmu (OECD/WTO)"/>
-    <tableColumn id="33" xr3:uid="{70783B5E-3FC1-DD44-9C4B-F29ABE2F730A}" name="Število zaposl. in samozaposl. V aktivnih podjetjih v Gostinstvu (I)"/>
+    <tableColumn id="33" xr3:uid="{70783B5E-3FC1-DD44-9C4B-F29ABE2F730A}" name="Število zaposl. in samozaposl. v aktivnih podjetjih v Gostinstvu (I)"/>
     <tableColumn id="34" xr3:uid="{55BC080C-8A66-C04E-A1E9-A6D4133CCFE0}" name="Zaposleni v Gostinstvu (I) v registr.podjetjih in s.p."/>
-    <tableColumn id="35" xr3:uid="{88DF1418-F448-F64B-AB10-E2E30ADD50CE}" name=" Zaposleni v nastan.dejav. (I55) v registr.podjetjih in s.p."/>
+    <tableColumn id="35" xr3:uid="{88DF1418-F448-F64B-AB10-E2E30ADD50CE}" name="Zaposleni v nastan.dejav. (I55) v registr.podjetjih in s.p."/>
     <tableColumn id="36" xr3:uid="{135A837A-5EB5-2546-AB5F-35C76A605B6C}" name="Vsi delovni aktivni na območju"/>
     <tableColumn id="37" xr3:uid="{52A7F38A-5C90-964D-B065-B17C7BA263D5}" name="Delež delovno aktivnih v turizmu (OECD/WTO)"/>
     <tableColumn id="38" xr3:uid="{C0F240E5-648C-7342-B26C-C8B4E0C3F6B4}" name="Število vseh vrst podjetij na območju"/>
@@ -1098,7 +1104,7 @@
     <tableColumn id="52" xr3:uid="{52578512-2D9B-3042-ABA7-4979793AD721}" name="Kapital v reg. Podjetjih in s.p. v Gostinstvu (I)"/>
     <tableColumn id="53" xr3:uid="{0B4E2348-7F98-4A4E-853F-4ACB891509F5}" name="Donosnost sredstev v reg. podjetjih in s.p. v Gostinstvu (I)"/>
     <tableColumn id="54" xr3:uid="{AF0EB5FE-DC22-5A48-BE37-FDD50761F05E}" name="Donosnost kapitala v reg. podjetjih in s.p. v Gostinstvu (I)"/>
-    <tableColumn id="55" xr3:uid="{128A26A4-FAEE-BC4A-B6EE-1A08B8D44E9B}" name="Dobičkovnost prihodkov v podjetjih in s.p. v Gostinstvu (I)21"/>
+    <tableColumn id="55" xr3:uid="{128A26A4-FAEE-BC4A-B6EE-1A08B8D44E9B}" name="Dobičkovnost prihodkov v podjetjih in s.p. v Gostinstvu (I)"/>
     <tableColumn id="56" xr3:uid="{F3FBED48-E964-884C-83EF-540A4CB997DE}" name="Število reg. podjetij in s.p. v nastanitveni dejav. (I 55)"/>
     <tableColumn id="57" xr3:uid="{7E9C06A6-EE05-5A4B-BFC4-1470DA5C6480}" name="Prihodki reg.podjetij in s.p. v nastanitveni dejav. (I 55)"/>
     <tableColumn id="58" xr3:uid="{594A7048-030B-7641-B062-ED36E3B0A3D9}" name="Dodana vrednost reg.podjetij v nastanitveni dejav. (I 55)"/>
@@ -1106,7 +1112,7 @@
     <tableColumn id="60" xr3:uid="{DB8C5AB7-2761-3A43-9547-30F272D35A19}" name="Ocenjeni stroški dela v reg. podj. v nastan.gost. (I 55) dejavnosti"/>
     <tableColumn id="61" xr3:uid="{C40A32FF-D555-5543-9E84-A6DEFFEAA3D9}" name="Stroški dela na zaposl. na leto v reg. podj. v nast.gost. (I 55) dejavnosti"/>
     <tableColumn id="62" xr3:uid="{D0F52755-EE67-9D44-8FB1-80277D4514B0}" name="Delež stroškov dela v prihodkih v reg. podj. v nast.gost.dej. (I 55)"/>
-    <tableColumn id="63" xr3:uid="{901DFC53-DFEE-1A4A-8CD7-EE7638EC34CF}" name="Delež stroškov dela v dod vredn. v reg. podj. v nast.gost.dej. (I)"/>
+    <tableColumn id="63" xr3:uid="{901DFC53-DFEE-1A4A-8CD7-EE7638EC34CF}" name="Delež stroškov dela v dod vredn. v reg. podj. v nast.gost.dej. (I 55)"/>
     <tableColumn id="64" xr3:uid="{8B14609D-EBDD-BD49-B52D-3A5DF542F21A}" name="EBITDA v reg.podjetjih in s.p. v nastanitveni dejav. (I 55)"/>
     <tableColumn id="65" xr3:uid="{F940FDC4-628D-364F-BF83-D4D71F989F3F}" name="EBITDA marža v reg.podjetjih v nastanitveni dejav. (I 55)"/>
     <tableColumn id="66" xr3:uid="{BBFA76B5-9A49-2E42-988A-3ED0E2C22836}" name="Čisti dobiček/izguba v reg. podj. v nastanitveni dejav. (I 55)"/>
@@ -1115,9 +1121,9 @@
     <tableColumn id="69" xr3:uid="{6E81CF29-3AC5-C946-B039-485FA0709B48}" name="Donosnost sredstev v nastanitveni dejav. (I 55)"/>
     <tableColumn id="70" xr3:uid="{8EC89FA0-B734-AB47-8230-A8F5756399A3}" name="Donosnost kapitala v nastanitveni dejav. (I 55)"/>
     <tableColumn id="71" xr3:uid="{BECD681F-4DC8-514B-AC4E-61683DFC409E}" name="Dobičkovnost prihodkov v nastanitveni dejav. (I 55)"/>
-    <tableColumn id="72" xr3:uid="{42865412-C344-4447-BA19-C224FF882D0F}" name="Cel.prihodki v nastan. dejav. na prenočitev"/>
-    <tableColumn id="73" xr3:uid="{C0A55036-7621-FF4E-B008-BD37F9C1DCB0}" name="Ocenjeni.prihodki iz nast. dejav. na prenočitev"/>
-    <tableColumn id="74" xr3:uid="{E97D5474-CD02-7942-9804-B61A028DC811}" name="Ocenj.prihodki iz nastan. dej. na razpoložljivo sobo (enoto)"/>
+    <tableColumn id="72" xr3:uid="{42865412-C344-4447-BA19-C224FF882D0F}" name="Celotni prihodki v nastan. dejav. na prenočitev"/>
+    <tableColumn id="73" xr3:uid="{C0A55036-7621-FF4E-B008-BD37F9C1DCB0}" name="Ocenjeni prihodki iz nast. dejav. na prenočitev"/>
+    <tableColumn id="74" xr3:uid="{E97D5474-CD02-7942-9804-B61A028DC811}" name="Ocenjeni prihodki iz nastan. dej. na razpoložljivo sobo (enoto)"/>
     <tableColumn id="75" xr3:uid="{2E828850-84D9-2047-A9B6-FCFA99B11C13}" name="Ocenjeni prihodki iz nast.dej. na prodano sobo (ned.enoto)"/>
     <tableColumn id="76" xr3:uid="{00135647-AE9B-654D-B4EF-EE54DDE5B2F9}" name="Poraba el.energije (MWh) Dejavnost Gostinstvo (I)"/>
     <tableColumn id="77" xr3:uid="{EB369050-8294-2D49-B9A4-DCA87CEA6142}" name="Poraba el.energ. v kWh na realiz. 1000 EUR prihodka v Gostinstvu (I)"/>
@@ -1128,12 +1134,14 @@
     <tableColumn id="82" xr3:uid="{12B8BC13-DF99-C743-95EC-792C5DC3DBFE}" name="Neto prejeti dohodek iz premoženja, kapitala, idr.povp. na preb."/>
     <tableColumn id="83" xr3:uid="{61271605-FB16-634F-A8C8-C46971209CAE}" name="Povprečna mesečna neto  plača/zaposl. osebo (EUR)"/>
     <tableColumn id="84" xr3:uid="{B839E3AE-E1FB-E546-BD00-FFE1920EB8E0}" name="Povprečna neto plača izplačana na zaposl. osebo v Gostinstvu (I)"/>
-    <tableColumn id="85" xr3:uid="{3DEB35FE-64B9-0843-A98D-1CA12FC3FA2D}" name=" Indeks neto plača v Gostinstvu (I) /pvp. plača v vseh dejavnostih"/>
+    <tableColumn id="85" xr3:uid="{3DEB35FE-64B9-0843-A98D-1CA12FC3FA2D}" name="Indeks neto plača v Gostinstvu (I) /pvp. plača v vseh dejavnostih"/>
     <tableColumn id="86" xr3:uid="{C9E1D9B1-1C78-B646-8ABF-40838C839C1A}" name="Število izdanih gradbenih dovoljenj/1000 prebivalcev"/>
-    <tableColumn id="87" xr3:uid="{4D5B6348-89BA-3242-A0DA-760B9847698D}" name=" Število počitniških stanovanj"/>
+    <tableColumn id="87" xr3:uid="{4D5B6348-89BA-3242-A0DA-760B9847698D}" name="Število počitniških stanovanj"/>
     <tableColumn id="88" xr3:uid="{76D8799C-B5BC-1944-B3D8-EFC1B6DE222D}" name="Delež naseljenih stanovanj od vseh razp."/>
     <tableColumn id="89" xr3:uid="{4A8C349E-38AA-514D-BDE6-DEB9AD9CC3E3}" name="Komunalni odpadki, zbrani  z javnim odvozom (kg/prebivalca)"/>
     <tableColumn id="90" xr3:uid="{1078F758-38E2-CE4E-AA92-AFDF93546914}" name="Štev.dijakov in študentov višjih strok. in visokošolsk.progr./1000 preb."/>
+    <tableColumn id="93" xr3:uid="{94D6BDF5-8A68-FD4A-8B32-B6C002FD5FD7}" name="Število vseh stanovanj"/>
+    <tableColumn id="91" xr3:uid="{C03597A0-F33A-DD4C-91CA-1B1BDC8046EA}" name="Delež naseljenih stanovanj"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -1456,7 +1464,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{96B947C3-A9C5-6843-B1A9-C8C5050E73E5}">
-  <dimension ref="A1:CL214"/>
+  <dimension ref="A1:CN214"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5" bestFit="1" customWidth="1"/>
@@ -1492,8 +1500,9 @@
     <col min="38" max="38" width="15" customWidth="1"/>
     <col min="39" max="39" width="23.6640625" customWidth="1"/>
     <col min="40" max="40" width="15.83203125" customWidth="1"/>
-    <col min="41" max="42" width="17.83203125" customWidth="1"/>
-    <col min="43" max="43" width="24.33203125" customWidth="1"/>
+    <col min="41" max="41" width="17.83203125" customWidth="1"/>
+    <col min="42" max="42" width="33.1640625" customWidth="1"/>
+    <col min="43" max="43" width="63.5" customWidth="1"/>
     <col min="44" max="44" width="23.6640625" customWidth="1"/>
     <col min="45" max="45" width="32.6640625" customWidth="1"/>
     <col min="46" max="46" width="24.83203125" customWidth="1"/>
@@ -1529,10 +1538,10 @@
     <col min="87" max="87" width="11.83203125" customWidth="1"/>
     <col min="88" max="88" width="22.33203125" customWidth="1"/>
     <col min="89" max="89" width="30.6640625" customWidth="1"/>
-    <col min="90" max="90" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="90" max="90" width="63" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1540,271 +1549,277 @@
         <v>214</v>
       </c>
       <c r="C1" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="D1" t="s">
-        <v>229</v>
+        <v>301</v>
       </c>
       <c r="E1" t="s">
         <v>228</v>
       </c>
       <c r="F1" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>297</v>
+        <v>285</v>
       </c>
       <c r="H1" t="s">
-        <v>298</v>
+        <v>286</v>
       </c>
       <c r="I1" t="s">
-        <v>299</v>
+        <v>287</v>
       </c>
       <c r="J1" t="s">
         <v>227</v>
       </c>
       <c r="K1" t="s">
+        <v>288</v>
+      </c>
+      <c r="L1" t="s">
+        <v>302</v>
+      </c>
+      <c r="M1" t="s">
+        <v>289</v>
+      </c>
+      <c r="N1" t="s">
+        <v>290</v>
+      </c>
+      <c r="O1" t="s">
+        <v>303</v>
+      </c>
+      <c r="P1" t="s">
+        <v>291</v>
+      </c>
+      <c r="Q1" t="s">
+        <v>292</v>
+      </c>
+      <c r="R1" t="s">
+        <v>293</v>
+      </c>
+      <c r="S1" t="s">
+        <v>294</v>
+      </c>
+      <c r="T1" t="s">
+        <v>295</v>
+      </c>
+      <c r="U1" t="s">
+        <v>296</v>
+      </c>
+      <c r="V1" t="s">
+        <v>297</v>
+      </c>
+      <c r="W1" t="s">
+        <v>298</v>
+      </c>
+      <c r="X1" t="s">
+        <v>299</v>
+      </c>
+      <c r="Y1" t="s">
         <v>300</v>
       </c>
-      <c r="L1" t="s">
-        <v>301</v>
-      </c>
-      <c r="M1" t="s">
-        <v>302</v>
-      </c>
-      <c r="N1" t="s">
-        <v>303</v>
-      </c>
-      <c r="O1" t="s">
+      <c r="Z1" t="s">
+        <v>231</v>
+      </c>
+      <c r="AA1" t="s">
+        <v>232</v>
+      </c>
+      <c r="AB1" t="s">
+        <v>233</v>
+      </c>
+      <c r="AC1" t="s">
+        <v>307</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>234</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>308</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>235</v>
+      </c>
+      <c r="AG1" t="s">
         <v>304</v>
       </c>
-      <c r="P1" t="s">
+      <c r="AH1" t="s">
+        <v>236</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>309</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>237</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>238</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>239</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>240</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>241</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>242</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>243</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>244</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>245</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>246</v>
+      </c>
+      <c r="AT1" t="s">
+        <v>247</v>
+      </c>
+      <c r="AU1" t="s">
+        <v>248</v>
+      </c>
+      <c r="AV1" t="s">
+        <v>249</v>
+      </c>
+      <c r="AW1" t="s">
+        <v>250</v>
+      </c>
+      <c r="AX1" t="s">
+        <v>251</v>
+      </c>
+      <c r="AY1" t="s">
+        <v>252</v>
+      </c>
+      <c r="AZ1" t="s">
+        <v>253</v>
+      </c>
+      <c r="BA1" t="s">
+        <v>254</v>
+      </c>
+      <c r="BB1" t="s">
+        <v>255</v>
+      </c>
+      <c r="BC1" t="s">
         <v>305</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="BD1" t="s">
+        <v>256</v>
+      </c>
+      <c r="BE1" t="s">
+        <v>257</v>
+      </c>
+      <c r="BF1" t="s">
+        <v>258</v>
+      </c>
+      <c r="BG1" t="s">
+        <v>259</v>
+      </c>
+      <c r="BH1" t="s">
+        <v>260</v>
+      </c>
+      <c r="BI1" t="s">
+        <v>261</v>
+      </c>
+      <c r="BJ1" t="s">
+        <v>262</v>
+      </c>
+      <c r="BK1" t="s">
         <v>306</v>
       </c>
-      <c r="R1" t="s">
-        <v>307</v>
-      </c>
-      <c r="S1" t="s">
-        <v>308</v>
-      </c>
-      <c r="T1" t="s">
-        <v>309</v>
-      </c>
-      <c r="U1" t="s">
+      <c r="BL1" t="s">
+        <v>263</v>
+      </c>
+      <c r="BM1" t="s">
+        <v>264</v>
+      </c>
+      <c r="BN1" t="s">
+        <v>265</v>
+      </c>
+      <c r="BO1" t="s">
+        <v>266</v>
+      </c>
+      <c r="BP1" t="s">
+        <v>267</v>
+      </c>
+      <c r="BQ1" t="s">
+        <v>268</v>
+      </c>
+      <c r="BR1" t="s">
+        <v>269</v>
+      </c>
+      <c r="BS1" t="s">
+        <v>270</v>
+      </c>
+      <c r="BT1" t="s">
         <v>310</v>
       </c>
-      <c r="V1" t="s">
+      <c r="BU1" t="s">
+        <v>312</v>
+      </c>
+      <c r="BV1" t="s">
         <v>311</v>
       </c>
-      <c r="W1" t="s">
-        <v>312</v>
-      </c>
-      <c r="X1" t="s">
+      <c r="BW1" t="s">
+        <v>271</v>
+      </c>
+      <c r="BX1" t="s">
+        <v>272</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>273</v>
+      </c>
+      <c r="BZ1" t="s">
+        <v>274</v>
+      </c>
+      <c r="CA1" t="s">
+        <v>275</v>
+      </c>
+      <c r="CB1" t="s">
+        <v>276</v>
+      </c>
+      <c r="CC1" t="s">
+        <v>277</v>
+      </c>
+      <c r="CD1" t="s">
+        <v>278</v>
+      </c>
+      <c r="CE1" t="s">
+        <v>279</v>
+      </c>
+      <c r="CF1" t="s">
+        <v>280</v>
+      </c>
+      <c r="CG1" t="s">
         <v>313</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="CH1" t="s">
+        <v>281</v>
+      </c>
+      <c r="CI1" t="s">
         <v>314</v>
       </c>
-      <c r="Z1" t="s">
-        <v>232</v>
-      </c>
-      <c r="AA1" t="s">
-        <v>233</v>
-      </c>
-      <c r="AB1" t="s">
-        <v>234</v>
-      </c>
-      <c r="AC1" t="s">
-        <v>235</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>236</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>237</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>238</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>239</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>240</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>241</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>242</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>243</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>244</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>245</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>246</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>247</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>248</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>249</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>250</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>251</v>
-      </c>
-      <c r="AT1" t="s">
-        <v>252</v>
-      </c>
-      <c r="AU1" t="s">
-        <v>253</v>
-      </c>
-      <c r="AV1" t="s">
-        <v>254</v>
-      </c>
-      <c r="AW1" t="s">
-        <v>255</v>
-      </c>
-      <c r="AX1" t="s">
-        <v>256</v>
-      </c>
-      <c r="AY1" t="s">
-        <v>257</v>
-      </c>
-      <c r="AZ1" t="s">
-        <v>258</v>
-      </c>
-      <c r="BA1" t="s">
-        <v>259</v>
-      </c>
-      <c r="BB1" t="s">
-        <v>260</v>
-      </c>
-      <c r="BC1" t="s">
-        <v>261</v>
-      </c>
-      <c r="BD1" t="s">
-        <v>262</v>
-      </c>
-      <c r="BE1" t="s">
-        <v>263</v>
-      </c>
-      <c r="BF1" t="s">
-        <v>264</v>
-      </c>
-      <c r="BG1" t="s">
-        <v>265</v>
-      </c>
-      <c r="BH1" t="s">
-        <v>266</v>
-      </c>
-      <c r="BI1" t="s">
-        <v>267</v>
-      </c>
-      <c r="BJ1" t="s">
-        <v>268</v>
-      </c>
-      <c r="BK1" t="s">
-        <v>269</v>
-      </c>
-      <c r="BL1" t="s">
-        <v>270</v>
-      </c>
-      <c r="BM1" t="s">
-        <v>271</v>
-      </c>
-      <c r="BN1" t="s">
-        <v>272</v>
-      </c>
-      <c r="BO1" t="s">
-        <v>273</v>
-      </c>
-      <c r="BP1" t="s">
-        <v>274</v>
-      </c>
-      <c r="BQ1" t="s">
-        <v>275</v>
-      </c>
-      <c r="BR1" t="s">
-        <v>276</v>
-      </c>
-      <c r="BS1" t="s">
-        <v>277</v>
-      </c>
-      <c r="BT1" t="s">
-        <v>278</v>
-      </c>
-      <c r="BU1" t="s">
-        <v>279</v>
-      </c>
-      <c r="BV1" t="s">
-        <v>280</v>
-      </c>
-      <c r="BW1" t="s">
-        <v>281</v>
-      </c>
-      <c r="BX1" t="s">
+      <c r="CJ1" t="s">
         <v>282</v>
       </c>
-      <c r="BY1" t="s">
+      <c r="CK1" t="s">
         <v>283</v>
       </c>
-      <c r="BZ1" t="s">
+      <c r="CL1" t="s">
         <v>284</v>
       </c>
-      <c r="CA1" t="s">
-        <v>285</v>
-      </c>
-      <c r="CB1" t="s">
-        <v>286</v>
-      </c>
-      <c r="CC1" t="s">
-        <v>287</v>
-      </c>
-      <c r="CD1" t="s">
-        <v>288</v>
-      </c>
-      <c r="CE1" t="s">
-        <v>289</v>
-      </c>
-      <c r="CF1" t="s">
-        <v>290</v>
-      </c>
-      <c r="CG1" t="s">
-        <v>291</v>
-      </c>
-      <c r="CH1" t="s">
-        <v>292</v>
-      </c>
-      <c r="CI1" t="s">
-        <v>293</v>
-      </c>
-      <c r="CJ1" t="s">
-        <v>294</v>
-      </c>
-      <c r="CK1" t="s">
-        <v>295</v>
-      </c>
-      <c r="CL1" t="s">
-        <v>296</v>
+      <c r="CM1" t="s">
+        <v>316</v>
+      </c>
+      <c r="CN1" t="s">
+        <v>315</v>
       </c>
     </row>
-    <row r="2" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>1</v>
       </c>
@@ -2072,8 +2087,14 @@
       <c r="CL2">
         <v>78.3</v>
       </c>
+      <c r="CM2">
+        <v>7322</v>
+      </c>
+      <c r="CN2">
+        <v>0.81876536465446603</v>
+      </c>
     </row>
-    <row r="3" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>2</v>
       </c>
@@ -2344,8 +2365,14 @@
       <c r="CL3">
         <v>81.099999999999994</v>
       </c>
+      <c r="CM3">
+        <v>1891</v>
+      </c>
+      <c r="CN3">
+        <v>0.68746694870438918</v>
+      </c>
     </row>
-    <row r="4" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>3</v>
       </c>
@@ -2616,8 +2643,14 @@
       <c r="CL4">
         <v>67.7</v>
       </c>
+      <c r="CM4">
+        <v>1464</v>
+      </c>
+      <c r="CN4">
+        <v>0.80259562841530052</v>
+      </c>
     </row>
-    <row r="5" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -2888,8 +2921,14 @@
       <c r="CL5">
         <v>61.3</v>
       </c>
+      <c r="CM5">
+        <v>2866</v>
+      </c>
+      <c r="CN5">
+        <v>0.85729239357990228</v>
+      </c>
     </row>
-    <row r="6" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
         <v>5</v>
       </c>
@@ -3160,8 +3199,14 @@
       <c r="CL6">
         <v>68.8</v>
       </c>
+      <c r="CM6">
+        <v>1041</v>
+      </c>
+      <c r="CN6">
+        <v>0.78770413064361189</v>
+      </c>
     </row>
-    <row r="7" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
         <v>6</v>
       </c>
@@ -3432,8 +3477,14 @@
       <c r="CL7">
         <v>78.099999999999994</v>
       </c>
+      <c r="CM7">
+        <v>620</v>
+      </c>
+      <c r="CN7">
+        <v>0.7129032258064516</v>
+      </c>
     </row>
-    <row r="8" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
         <v>7</v>
       </c>
@@ -3704,8 +3755,14 @@
       <c r="CL8">
         <v>72.7</v>
       </c>
+      <c r="CM8">
+        <v>3799</v>
+      </c>
+      <c r="CN8">
+        <v>0.7341405633061332</v>
+      </c>
     </row>
-    <row r="9" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
         <v>8</v>
       </c>
@@ -3976,8 +4033,14 @@
       <c r="CL9">
         <v>65.400000000000006</v>
       </c>
+      <c r="CM9">
+        <v>805</v>
+      </c>
+      <c r="CN9">
+        <v>0.67577639751552798</v>
+      </c>
     </row>
-    <row r="10" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
         <v>9</v>
       </c>
@@ -4248,8 +4311,14 @@
       <c r="CL10">
         <v>66.7</v>
       </c>
+      <c r="CM10">
+        <v>3387</v>
+      </c>
+      <c r="CN10">
+        <v>0.55683495718925302</v>
+      </c>
     </row>
-    <row r="11" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
         <v>10</v>
       </c>
@@ -4520,8 +4589,14 @@
       <c r="CL11">
         <v>65.8</v>
       </c>
+      <c r="CM11">
+        <v>1572</v>
+      </c>
+      <c r="CN11">
+        <v>0.87786259541984735</v>
+      </c>
     </row>
-    <row r="12" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
         <v>11</v>
       </c>
@@ -4792,8 +4867,14 @@
       <c r="CL12">
         <v>72.2</v>
       </c>
+      <c r="CM12">
+        <v>2666</v>
+      </c>
+      <c r="CN12">
+        <v>0.49699924981245314</v>
+      </c>
     </row>
-    <row r="13" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
         <v>12</v>
       </c>
@@ -5064,8 +5145,14 @@
       <c r="CL13">
         <v>57</v>
       </c>
+      <c r="CM13">
+        <v>2167</v>
+      </c>
+      <c r="CN13">
+        <v>0.82418089524688509</v>
+      </c>
     </row>
-    <row r="14" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
         <v>13</v>
       </c>
@@ -5336,8 +5423,14 @@
       <c r="CL14">
         <v>80.400000000000006</v>
       </c>
+      <c r="CM14">
+        <v>2339</v>
+      </c>
+      <c r="CN14">
+        <v>0.74476271911073111</v>
+      </c>
     </row>
-    <row r="15" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
         <v>14</v>
       </c>
@@ -5608,8 +5701,14 @@
       <c r="CL15">
         <v>71.099999999999994</v>
       </c>
+      <c r="CM15">
+        <v>4316</v>
+      </c>
+      <c r="CN15">
+        <v>0.84708063021316038</v>
+      </c>
     </row>
-    <row r="16" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
         <v>15</v>
       </c>
@@ -5880,8 +5979,14 @@
       <c r="CL16">
         <v>92.7</v>
       </c>
+      <c r="CM16">
+        <v>10515</v>
+      </c>
+      <c r="CN16">
+        <v>0.76966238706609602</v>
+      </c>
     </row>
-    <row r="17" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>16</v>
       </c>
@@ -6152,8 +6257,14 @@
       <c r="CL17">
         <v>65.400000000000006</v>
       </c>
+      <c r="CM17">
+        <v>786</v>
+      </c>
+      <c r="CN17">
+        <v>0.71755725190839692</v>
+      </c>
     </row>
-    <row r="18" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>17</v>
       </c>
@@ -6424,8 +6535,14 @@
       <c r="CL18">
         <v>54.1</v>
       </c>
+      <c r="CM18">
+        <v>21321</v>
+      </c>
+      <c r="CN18">
+        <v>0.84967872051029503</v>
+      </c>
     </row>
-    <row r="19" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -6696,8 +6813,14 @@
       <c r="CL19">
         <v>69.900000000000006</v>
       </c>
+      <c r="CM19">
+        <v>2721</v>
+      </c>
+      <c r="CN19">
+        <v>0.78868063212054396</v>
+      </c>
     </row>
-    <row r="20" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>19</v>
       </c>
@@ -6968,8 +7091,14 @@
       <c r="CL20">
         <v>86.7</v>
       </c>
+      <c r="CM20">
+        <v>4541</v>
+      </c>
+      <c r="CN20">
+        <v>0.82426778242677823</v>
+      </c>
     </row>
-    <row r="21" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>20</v>
       </c>
@@ -7240,8 +7369,14 @@
       <c r="CL21">
         <v>77.900000000000006</v>
       </c>
+      <c r="CM21">
+        <v>1997</v>
+      </c>
+      <c r="CN21">
+        <v>0.74211316975463193</v>
+      </c>
     </row>
-    <row r="22" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>21</v>
       </c>
@@ -7512,8 +7647,14 @@
       <c r="CL22">
         <v>78.900000000000006</v>
       </c>
+      <c r="CM22">
+        <v>866</v>
+      </c>
+      <c r="CN22">
+        <v>0.74018475750577373</v>
+      </c>
     </row>
-    <row r="23" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>22</v>
       </c>
@@ -7784,8 +7925,14 @@
       <c r="CL23">
         <v>54.2</v>
       </c>
+      <c r="CM23">
+        <v>1527</v>
+      </c>
+      <c r="CN23">
+        <v>0.53176162409954153</v>
+      </c>
     </row>
-    <row r="24" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>23</v>
       </c>
@@ -8056,8 +8203,14 @@
       <c r="CL24">
         <v>61.9</v>
       </c>
+      <c r="CM24">
+        <v>1483</v>
+      </c>
+      <c r="CN24">
+        <v>0.78624409979770737</v>
+      </c>
     </row>
-    <row r="25" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>24</v>
       </c>
@@ -8328,8 +8481,14 @@
       <c r="CL25">
         <v>70.3</v>
       </c>
+      <c r="CM25">
+        <v>1420</v>
+      </c>
+      <c r="CN25">
+        <v>0.78169014084507038</v>
+      </c>
     </row>
-    <row r="26" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>25</v>
       </c>
@@ -8600,8 +8759,14 @@
       <c r="CL26">
         <v>65.5</v>
       </c>
+      <c r="CM26">
+        <v>5950</v>
+      </c>
+      <c r="CN26">
+        <v>0.75344537815126056</v>
+      </c>
     </row>
-    <row r="27" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>26</v>
       </c>
@@ -8872,8 +9037,14 @@
       <c r="CL27">
         <v>66</v>
       </c>
+      <c r="CM27">
+        <v>1076</v>
+      </c>
+      <c r="CN27">
+        <v>0.79182156133828996</v>
+      </c>
     </row>
-    <row r="28" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>27</v>
       </c>
@@ -9144,8 +9315,14 @@
       <c r="CL28">
         <v>70.400000000000006</v>
       </c>
+      <c r="CM28">
+        <v>1942</v>
+      </c>
+      <c r="CN28">
+        <v>0.7646755921730175</v>
+      </c>
     </row>
-    <row r="29" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>28</v>
       </c>
@@ -9416,8 +9593,14 @@
       <c r="CL29">
         <v>56.8</v>
       </c>
+      <c r="CM29">
+        <v>402</v>
+      </c>
+      <c r="CN29">
+        <v>0.70646766169154229</v>
+      </c>
     </row>
-    <row r="30" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>29</v>
       </c>
@@ -9688,8 +9871,14 @@
       <c r="CL30">
         <v>86.6</v>
       </c>
+      <c r="CM30">
+        <v>1449</v>
+      </c>
+      <c r="CN30">
+        <v>0.77639751552795033</v>
+      </c>
     </row>
-    <row r="31" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>30</v>
       </c>
@@ -9960,8 +10149,14 @@
       <c r="CL31">
         <v>78.400000000000006</v>
       </c>
+      <c r="CM31">
+        <v>890</v>
+      </c>
+      <c r="CN31">
+        <v>0.77078651685393262</v>
+      </c>
     </row>
-    <row r="32" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>31</v>
       </c>
@@ -10232,8 +10427,14 @@
       <c r="CL32">
         <v>63.1</v>
       </c>
+      <c r="CM32">
+        <v>2714</v>
+      </c>
+      <c r="CN32">
+        <v>0.79624170965364771</v>
+      </c>
     </row>
-    <row r="33" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A33" t="s">
         <v>32</v>
       </c>
@@ -10504,8 +10705,14 @@
       <c r="CL33">
         <v>95.4</v>
       </c>
+      <c r="CM33">
+        <v>585</v>
+      </c>
+      <c r="CN33">
+        <v>0.74358974358974361</v>
+      </c>
     </row>
-    <row r="34" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A34" t="s">
         <v>33</v>
       </c>
@@ -10776,8 +10983,14 @@
       <c r="CL34">
         <v>65.2</v>
       </c>
+      <c r="CM34">
+        <v>2186</v>
+      </c>
+      <c r="CN34">
+        <v>0.86276303751143646</v>
+      </c>
     </row>
-    <row r="35" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A35" t="s">
         <v>34</v>
       </c>
@@ -11048,8 +11261,14 @@
       <c r="CL35">
         <v>89.4</v>
       </c>
+      <c r="CM35">
+        <v>1468</v>
+      </c>
+      <c r="CN35">
+        <v>0.75544959128065392</v>
+      </c>
     </row>
-    <row r="36" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A36" t="s">
         <v>35</v>
       </c>
@@ -11320,8 +11539,14 @@
       <c r="CL36">
         <v>83.4</v>
       </c>
+      <c r="CM36">
+        <v>12824</v>
+      </c>
+      <c r="CN36">
+        <v>0.8792108546475359</v>
+      </c>
     </row>
-    <row r="37" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A37" t="s">
         <v>36</v>
       </c>
@@ -11592,8 +11817,14 @@
       <c r="CL37">
         <v>83</v>
       </c>
+      <c r="CM37">
+        <v>1063</v>
+      </c>
+      <c r="CN37">
+        <v>0.78833490122295391</v>
+      </c>
     </row>
-    <row r="38" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A38" t="s">
         <v>37</v>
       </c>
@@ -11864,8 +12095,14 @@
       <c r="CL38">
         <v>64.099999999999994</v>
       </c>
+      <c r="CM38">
+        <v>3116</v>
+      </c>
+      <c r="CN38">
+        <v>0.85654685494223359</v>
+      </c>
     </row>
-    <row r="39" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A39" t="s">
         <v>38</v>
       </c>
@@ -12136,8 +12373,14 @@
       <c r="CL39">
         <v>71.400000000000006</v>
       </c>
+      <c r="CM39">
+        <v>2605</v>
+      </c>
+      <c r="CN39">
+        <v>0.83685220729366605</v>
+      </c>
     </row>
-    <row r="40" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A40" t="s">
         <v>39</v>
       </c>
@@ -12408,8 +12651,14 @@
       <c r="CL40">
         <v>68.7</v>
       </c>
+      <c r="CM40">
+        <v>2599</v>
+      </c>
+      <c r="CN40">
+        <v>0.75836860330896494</v>
+      </c>
     </row>
-    <row r="41" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A41" t="s">
         <v>40</v>
       </c>
@@ -12680,8 +12929,14 @@
       <c r="CL41">
         <v>96.6</v>
       </c>
+      <c r="CM41">
+        <v>1435</v>
+      </c>
+      <c r="CN41">
+        <v>0.83344947735191632</v>
+      </c>
     </row>
-    <row r="42" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>41</v>
       </c>
@@ -12952,8 +13207,14 @@
       <c r="CL42">
         <v>72.5</v>
       </c>
+      <c r="CM42">
+        <v>1151</v>
+      </c>
+      <c r="CN42">
+        <v>0.77584708948740222</v>
+      </c>
     </row>
-    <row r="43" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>42</v>
       </c>
@@ -13224,8 +13485,14 @@
       <c r="CL43">
         <v>74.099999999999994</v>
       </c>
+      <c r="CM43">
+        <v>3745</v>
+      </c>
+      <c r="CN43">
+        <v>0.7965287049399199</v>
+      </c>
     </row>
-    <row r="44" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A44" t="s">
         <v>43</v>
       </c>
@@ -13496,8 +13763,14 @@
       <c r="CL44">
         <v>60.9</v>
       </c>
+      <c r="CM44">
+        <v>953</v>
+      </c>
+      <c r="CN44">
+        <v>0.77334732423924446</v>
+      </c>
     </row>
-    <row r="45" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>44</v>
       </c>
@@ -13768,8 +14041,14 @@
       <c r="CL45">
         <v>69.7</v>
       </c>
+      <c r="CM45">
+        <v>1104</v>
+      </c>
+      <c r="CN45">
+        <v>0.65489130434782605</v>
+      </c>
     </row>
-    <row r="46" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>45</v>
       </c>
@@ -14040,8 +14319,14 @@
       <c r="CL46">
         <v>44.4</v>
       </c>
+      <c r="CM46">
+        <v>897</v>
+      </c>
+      <c r="CN46">
+        <v>0.75027870680044595</v>
+      </c>
     </row>
-    <row r="47" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>46</v>
       </c>
@@ -14312,8 +14597,14 @@
       <c r="CL47">
         <v>51.9</v>
       </c>
+      <c r="CM47">
+        <v>6916</v>
+      </c>
+      <c r="CN47">
+        <v>0.86871023713128981</v>
+      </c>
     </row>
-    <row r="48" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>47</v>
       </c>
@@ -14584,8 +14875,14 @@
       <c r="CL48">
         <v>88</v>
       </c>
+      <c r="CM48">
+        <v>1374</v>
+      </c>
+      <c r="CN48">
+        <v>0.86171761280931591</v>
+      </c>
     </row>
-    <row r="49" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>48</v>
       </c>
@@ -14856,8 +15153,14 @@
       <c r="CL49">
         <v>69.900000000000006</v>
       </c>
+      <c r="CM49">
+        <v>4617</v>
+      </c>
+      <c r="CN49">
+        <v>0.80051981806367767</v>
+      </c>
     </row>
-    <row r="50" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A50" t="s">
         <v>49</v>
       </c>
@@ -15128,8 +15431,14 @@
       <c r="CL50">
         <v>73.5</v>
       </c>
+      <c r="CM50">
+        <v>131</v>
+      </c>
+      <c r="CN50">
+        <v>0.74045801526717558</v>
+      </c>
     </row>
-    <row r="51" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A51" t="s">
         <v>50</v>
       </c>
@@ -15400,8 +15709,14 @@
       <c r="CL51">
         <v>29.9</v>
       </c>
+      <c r="CM51">
+        <v>954</v>
+      </c>
+      <c r="CN51">
+        <v>0.80922431865828093</v>
+      </c>
     </row>
-    <row r="52" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A52" t="s">
         <v>51</v>
       </c>
@@ -15672,8 +15987,14 @@
       <c r="CL52">
         <v>83.9</v>
       </c>
+      <c r="CM52">
+        <v>4162</v>
+      </c>
+      <c r="CN52">
+        <v>0.82316194137433929</v>
+      </c>
     </row>
-    <row r="53" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A53" t="s">
         <v>52</v>
       </c>
@@ -15944,8 +16265,14 @@
       <c r="CL53">
         <v>63.9</v>
       </c>
+      <c r="CM53">
+        <v>2337</v>
+      </c>
+      <c r="CN53">
+        <v>0.7227214377406932</v>
+      </c>
     </row>
-    <row r="54" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>53</v>
       </c>
@@ -16216,8 +16543,14 @@
       <c r="CL54">
         <v>57.6</v>
       </c>
+      <c r="CM54">
+        <v>4967</v>
+      </c>
+      <c r="CN54">
+        <v>0.80893899738272601</v>
+      </c>
     </row>
-    <row r="55" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>54</v>
       </c>
@@ -16488,8 +16821,14 @@
       <c r="CL55">
         <v>75.7</v>
       </c>
+      <c r="CM55">
+        <v>2771</v>
+      </c>
+      <c r="CN55">
+        <v>0.80476362324070727</v>
+      </c>
     </row>
-    <row r="56" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>55</v>
       </c>
@@ -16760,8 +17099,14 @@
       <c r="CL56">
         <v>80.7</v>
       </c>
+      <c r="CM56">
+        <v>6154</v>
+      </c>
+      <c r="CN56">
+        <v>0.75885602859928503</v>
+      </c>
     </row>
-    <row r="57" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>56</v>
       </c>
@@ -17032,8 +17377,14 @@
       <c r="CL57">
         <v>66.900000000000006</v>
       </c>
+      <c r="CM57">
+        <v>6479</v>
+      </c>
+      <c r="CN57">
+        <v>0.77959561660750121</v>
+      </c>
     </row>
-    <row r="58" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>57</v>
       </c>
@@ -17304,8 +17655,14 @@
       <c r="CL58">
         <v>79.599999999999994</v>
       </c>
+      <c r="CM58">
+        <v>8407</v>
+      </c>
+      <c r="CN58">
+        <v>0.72451528488164629</v>
+      </c>
     </row>
-    <row r="59" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>58</v>
       </c>
@@ -17576,8 +17933,14 @@
       <c r="CL59">
         <v>62.6</v>
       </c>
+      <c r="CM59">
+        <v>8575</v>
+      </c>
+      <c r="CN59">
+        <v>0.88746355685131195</v>
+      </c>
     </row>
-    <row r="60" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>59</v>
       </c>
@@ -17848,8 +18211,14 @@
       <c r="CL60">
         <v>58.8</v>
       </c>
+      <c r="CM60">
+        <v>364</v>
+      </c>
+      <c r="CN60">
+        <v>0.63461538461538458</v>
+      </c>
     </row>
-    <row r="61" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>60</v>
       </c>
@@ -18120,8 +18489,14 @@
       <c r="CL61">
         <v>64.2</v>
       </c>
+      <c r="CM61">
+        <v>1069</v>
+      </c>
+      <c r="CN61">
+        <v>0.70439663236669781</v>
+      </c>
     </row>
-    <row r="62" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>61</v>
       </c>
@@ -18392,8 +18767,14 @@
       <c r="CL62">
         <v>69</v>
       </c>
+      <c r="CM62">
+        <v>10679</v>
+      </c>
+      <c r="CN62">
+        <v>0.85663451634048127</v>
+      </c>
     </row>
-    <row r="63" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>62</v>
       </c>
@@ -18664,8 +19045,14 @@
       <c r="CL63">
         <v>78.7</v>
       </c>
+      <c r="CM63">
+        <v>2598</v>
+      </c>
+      <c r="CN63">
+        <v>0.73672055427251737</v>
+      </c>
     </row>
-    <row r="64" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A64" t="s">
         <v>63</v>
       </c>
@@ -18936,8 +19323,14 @@
       <c r="CL64">
         <v>73.8</v>
       </c>
+      <c r="CM64">
+        <v>2459</v>
+      </c>
+      <c r="CN64">
+        <v>0.84993899959333064</v>
+      </c>
     </row>
-    <row r="65" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A65" t="s">
         <v>64</v>
       </c>
@@ -19208,8 +19601,14 @@
       <c r="CL65">
         <v>74.8</v>
       </c>
+      <c r="CM65">
+        <v>2077</v>
+      </c>
+      <c r="CN65">
+        <v>0.70582571015888296</v>
+      </c>
     </row>
-    <row r="66" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>65</v>
       </c>
@@ -19480,8 +19879,14 @@
       <c r="CL66">
         <v>73</v>
       </c>
+      <c r="CM66">
+        <v>238</v>
+      </c>
+      <c r="CN66">
+        <v>0.75630252100840334</v>
+      </c>
     </row>
-    <row r="67" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>66</v>
       </c>
@@ -19752,8 +20157,14 @@
       <c r="CL67">
         <v>55.6</v>
       </c>
+      <c r="CM67">
+        <v>6369</v>
+      </c>
+      <c r="CN67">
+        <v>0.81362851311037843</v>
+      </c>
     </row>
-    <row r="68" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A68" t="s">
         <v>67</v>
       </c>
@@ -20024,8 +20435,14 @@
       <c r="CL68">
         <v>63</v>
       </c>
+      <c r="CM68">
+        <v>1810</v>
+      </c>
+      <c r="CN68">
+        <v>0.69171270718232047</v>
+      </c>
     </row>
-    <row r="69" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>68</v>
       </c>
@@ -20296,8 +20713,14 @@
       <c r="CL69">
         <v>70.400000000000006</v>
       </c>
+      <c r="CM69">
+        <v>2057</v>
+      </c>
+      <c r="CN69">
+        <v>0.87506076810889644</v>
+      </c>
     </row>
-    <row r="70" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>69</v>
       </c>
@@ -20568,8 +20991,14 @@
       <c r="CL70">
         <v>94.8</v>
       </c>
+      <c r="CM70">
+        <v>23097</v>
+      </c>
+      <c r="CN70">
+        <v>0.78707191410139843</v>
+      </c>
     </row>
-    <row r="71" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>70</v>
       </c>
@@ -20840,8 +21269,14 @@
       <c r="CL71">
         <v>68.3</v>
       </c>
+      <c r="CM71">
+        <v>1036</v>
+      </c>
+      <c r="CN71">
+        <v>0.76930501930501927</v>
+      </c>
     </row>
-    <row r="72" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>71</v>
       </c>
@@ -21112,8 +21547,14 @@
       <c r="CL72">
         <v>83.4</v>
       </c>
+      <c r="CM72">
+        <v>632</v>
+      </c>
+      <c r="CN72">
+        <v>0.48101265822784811</v>
+      </c>
     </row>
-    <row r="73" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>72</v>
       </c>
@@ -21384,8 +21825,14 @@
       <c r="CL73">
         <v>63.6</v>
       </c>
+      <c r="CM73">
+        <v>1402</v>
+      </c>
+      <c r="CN73">
+        <v>0.7168330955777461</v>
+      </c>
     </row>
-    <row r="74" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A74" t="s">
         <v>73</v>
       </c>
@@ -21656,8 +22103,14 @@
       <c r="CL74">
         <v>74.599999999999994</v>
       </c>
+      <c r="CM74">
+        <v>21317</v>
+      </c>
+      <c r="CN74">
+        <v>0.88534972088004882</v>
+      </c>
     </row>
-    <row r="75" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A75" t="s">
         <v>74</v>
       </c>
@@ -21928,8 +22381,14 @@
       <c r="CL75">
         <v>74.8</v>
       </c>
+      <c r="CM75">
+        <v>4156</v>
+      </c>
+      <c r="CN75">
+        <v>0.6179018286814244</v>
+      </c>
     </row>
-    <row r="76" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A76" t="s">
         <v>75</v>
       </c>
@@ -22200,8 +22659,14 @@
       <c r="CL76">
         <v>59.3</v>
       </c>
+      <c r="CM76">
+        <v>1257</v>
+      </c>
+      <c r="CN76">
+        <v>0.82895783611774065</v>
+      </c>
     </row>
-    <row r="77" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A77" t="s">
         <v>76</v>
       </c>
@@ -22472,8 +22937,14 @@
       <c r="CL77">
         <v>64</v>
       </c>
+      <c r="CM77">
+        <v>10515</v>
+      </c>
+      <c r="CN77">
+        <v>0.78925344745601522</v>
+      </c>
     </row>
-    <row r="78" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>77</v>
       </c>
@@ -22744,8 +23215,14 @@
       <c r="CL78">
         <v>72.8</v>
       </c>
+      <c r="CM78">
+        <v>2050</v>
+      </c>
+      <c r="CN78">
+        <v>0.79268292682926833</v>
+      </c>
     </row>
-    <row r="79" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>78</v>
       </c>
@@ -23016,8 +23493,14 @@
       <c r="CL79">
         <v>69.7</v>
       </c>
+      <c r="CM79">
+        <v>653</v>
+      </c>
+      <c r="CN79">
+        <v>0.72128637059724354</v>
+      </c>
     </row>
-    <row r="80" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>79</v>
       </c>
@@ -23288,8 +23771,14 @@
       <c r="CL80">
         <v>44.7</v>
       </c>
+      <c r="CM80">
+        <v>5594</v>
+      </c>
+      <c r="CN80">
+        <v>0.78852341794780123</v>
+      </c>
     </row>
-    <row r="81" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>80</v>
       </c>
@@ -23560,8 +24049,14 @@
       <c r="CL81">
         <v>69.400000000000006</v>
       </c>
+      <c r="CM81">
+        <v>3287</v>
+      </c>
+      <c r="CN81">
+        <v>0.8119866139336781</v>
+      </c>
     </row>
-    <row r="82" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>81</v>
       </c>
@@ -23832,8 +24327,14 @@
       <c r="CL82">
         <v>69</v>
       </c>
+      <c r="CM82">
+        <v>4853</v>
+      </c>
+      <c r="CN82">
+        <v>0.7739542550999382</v>
+      </c>
     </row>
-    <row r="83" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>82</v>
       </c>
@@ -24104,8 +24605,14 @@
       <c r="CL83">
         <v>52.2</v>
       </c>
+      <c r="CM83">
+        <v>6008</v>
+      </c>
+      <c r="CN83">
+        <v>0.82123834886817582</v>
+      </c>
     </row>
-    <row r="84" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>83</v>
       </c>
@@ -24376,8 +24883,14 @@
       <c r="CL84">
         <v>79.099999999999994</v>
       </c>
+      <c r="CM84">
+        <v>129816</v>
+      </c>
+      <c r="CN84">
+        <v>0.82244099340605159</v>
+      </c>
     </row>
-    <row r="85" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>84</v>
       </c>
@@ -24648,8 +25161,14 @@
       <c r="CL85">
         <v>67.7</v>
       </c>
+      <c r="CM85">
+        <v>1025</v>
+      </c>
+      <c r="CN85">
+        <v>0.75219512195121951</v>
+      </c>
     </row>
-    <row r="86" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>85</v>
       </c>
@@ -24920,8 +25439,14 @@
       <c r="CL86">
         <v>78.400000000000006</v>
       </c>
+      <c r="CM86">
+        <v>4886</v>
+      </c>
+      <c r="CN86">
+        <v>0.77261563651248466</v>
+      </c>
     </row>
-    <row r="87" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>86</v>
       </c>
@@ -25192,8 +25717,14 @@
       <c r="CL87">
         <v>72.599999999999994</v>
       </c>
+      <c r="CM87">
+        <v>1251</v>
+      </c>
+      <c r="CN87">
+        <v>0.8840927258193445</v>
+      </c>
     </row>
-    <row r="88" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A88" t="s">
         <v>87</v>
       </c>
@@ -25464,8 +25995,14 @@
       <c r="CL88">
         <v>93.4</v>
       </c>
+      <c r="CM88">
+        <v>4985</v>
+      </c>
+      <c r="CN88">
+        <v>0.86359077231695081</v>
+      </c>
     </row>
-    <row r="89" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A89" t="s">
         <v>88</v>
       </c>
@@ -25736,8 +26273,14 @@
       <c r="CL89">
         <v>81.7</v>
       </c>
+      <c r="CM89">
+        <v>1390</v>
+      </c>
+      <c r="CN89">
+        <v>0.8</v>
+      </c>
     </row>
-    <row r="90" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A90" t="s">
         <v>89</v>
       </c>
@@ -26008,8 +26551,14 @@
       <c r="CL90">
         <v>80.099999999999994</v>
       </c>
+      <c r="CM90">
+        <v>823</v>
+      </c>
+      <c r="CN90">
+        <v>0.69137302551640345</v>
+      </c>
     </row>
-    <row r="91" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A91" t="s">
         <v>90</v>
       </c>
@@ -26280,8 +26829,14 @@
       <c r="CL91">
         <v>64.2</v>
       </c>
+      <c r="CM91">
+        <v>1227</v>
+      </c>
+      <c r="CN91">
+        <v>0.81581092094539531</v>
+      </c>
     </row>
-    <row r="92" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A92" t="s">
         <v>91</v>
       </c>
@@ -26552,8 +27107,14 @@
       <c r="CL92">
         <v>66.7</v>
       </c>
+      <c r="CM92">
+        <v>603</v>
+      </c>
+      <c r="CN92">
+        <v>0.71641791044776115</v>
+      </c>
     </row>
-    <row r="93" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A93" t="s">
         <v>92</v>
       </c>
@@ -26824,8 +27385,14 @@
       <c r="CL93">
         <v>83.1</v>
       </c>
+      <c r="CM93">
+        <v>1939</v>
+      </c>
+      <c r="CN93">
+        <v>0.81536874677668902</v>
+      </c>
     </row>
-    <row r="94" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A94" t="s">
         <v>93</v>
       </c>
@@ -27096,8 +27663,14 @@
       <c r="CL94">
         <v>78.599999999999994</v>
       </c>
+      <c r="CM94">
+        <v>1818</v>
+      </c>
+      <c r="CN94">
+        <v>0.74697469746974698</v>
+      </c>
     </row>
-    <row r="95" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A95" t="s">
         <v>94</v>
       </c>
@@ -27368,8 +27941,14 @@
       <c r="CL95">
         <v>72.2</v>
       </c>
+      <c r="CM95">
+        <v>969</v>
+      </c>
+      <c r="CN95">
+        <v>0.72445820433436536</v>
+      </c>
     </row>
-    <row r="96" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A96" t="s">
         <v>95</v>
       </c>
@@ -27640,8 +28219,14 @@
       <c r="CL96">
         <v>68.400000000000006</v>
       </c>
+      <c r="CM96">
+        <v>52893</v>
+      </c>
+      <c r="CN96">
+        <v>0.82755752178927267</v>
+      </c>
     </row>
-    <row r="97" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A97" t="s">
         <v>96</v>
       </c>
@@ -27912,8 +28497,14 @@
       <c r="CL97">
         <v>58.8</v>
       </c>
+      <c r="CM97">
+        <v>1374</v>
+      </c>
+      <c r="CN97">
+        <v>0.86171761280931591</v>
+      </c>
     </row>
-    <row r="98" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A98" t="s">
         <v>97</v>
       </c>
@@ -28184,8 +28775,14 @@
       <c r="CL98">
         <v>67.599999999999994</v>
       </c>
+      <c r="CM98">
+        <v>5983</v>
+      </c>
+      <c r="CN98">
+        <v>0.86010362694300513</v>
+      </c>
     </row>
-    <row r="99" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A99" t="s">
         <v>98</v>
       </c>
@@ -28456,8 +29053,14 @@
       <c r="CL99">
         <v>80.599999999999994</v>
       </c>
+      <c r="CM99">
+        <v>2856</v>
+      </c>
+      <c r="CN99">
+        <v>0.85784313725490191</v>
+      </c>
     </row>
-    <row r="100" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A100" t="s">
         <v>99</v>
       </c>
@@ -28728,8 +29331,14 @@
       <c r="CL100">
         <v>78.400000000000006</v>
       </c>
+      <c r="CM100">
+        <v>3390</v>
+      </c>
+      <c r="CN100">
+        <v>0.74631268436578169</v>
+      </c>
     </row>
-    <row r="101" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A101" t="s">
         <v>100</v>
       </c>
@@ -29000,8 +29609,14 @@
       <c r="CL101">
         <v>67.599999999999994</v>
       </c>
+      <c r="CM101">
+        <v>1522</v>
+      </c>
+      <c r="CN101">
+        <v>0.85676741130091982</v>
+      </c>
     </row>
-    <row r="102" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A102" t="s">
         <v>101</v>
       </c>
@@ -29272,8 +29887,14 @@
       <c r="CL102">
         <v>68.5</v>
       </c>
+      <c r="CM102">
+        <v>2427</v>
+      </c>
+      <c r="CN102">
+        <v>0.87474248042851255</v>
+      </c>
     </row>
-    <row r="103" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A103" t="s">
         <v>102</v>
       </c>
@@ -29544,8 +30165,14 @@
       <c r="CL103">
         <v>76.2</v>
       </c>
+      <c r="CM103">
+        <v>2026</v>
+      </c>
+      <c r="CN103">
+        <v>0.79615004935834155</v>
+      </c>
     </row>
-    <row r="104" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A104" t="s">
         <v>103</v>
       </c>
@@ -29816,8 +30443,14 @@
       <c r="CL104">
         <v>74.099999999999994</v>
       </c>
+      <c r="CM104">
+        <v>1199</v>
+      </c>
+      <c r="CN104">
+        <v>0.76146788990825687</v>
+      </c>
     </row>
-    <row r="105" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A105" t="s">
         <v>104</v>
       </c>
@@ -30088,8 +30721,14 @@
       <c r="CL105">
         <v>74.8</v>
       </c>
+      <c r="CM105">
+        <v>1156</v>
+      </c>
+      <c r="CN105">
+        <v>0.74134948096885811</v>
+      </c>
     </row>
-    <row r="106" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A106" t="s">
         <v>105</v>
       </c>
@@ -30360,8 +30999,14 @@
       <c r="CL106">
         <v>69.2</v>
       </c>
+      <c r="CM106">
+        <v>1715</v>
+      </c>
+      <c r="CN106">
+        <v>0.76793002915451891</v>
+      </c>
     </row>
-    <row r="107" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A107" t="s">
         <v>106</v>
       </c>
@@ -30632,8 +31277,14 @@
       <c r="CL107">
         <v>80.599999999999994</v>
       </c>
+      <c r="CM107">
+        <v>1403</v>
+      </c>
+      <c r="CN107">
+        <v>0.73342836778332143</v>
+      </c>
     </row>
-    <row r="108" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A108" t="s">
         <v>107</v>
       </c>
@@ -30904,8 +31555,14 @@
       <c r="CL108">
         <v>77.400000000000006</v>
       </c>
+      <c r="CM108">
+        <v>1821</v>
+      </c>
+      <c r="CN108">
+        <v>0.80230642504118621</v>
+      </c>
     </row>
-    <row r="109" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A109" t="s">
         <v>108</v>
       </c>
@@ -31176,8 +31833,14 @@
       <c r="CL109">
         <v>89.3</v>
       </c>
+      <c r="CM109">
+        <v>3376</v>
+      </c>
+      <c r="CN109">
+        <v>0.60545023696682465</v>
+      </c>
     </row>
-    <row r="110" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A110" t="s">
         <v>109</v>
       </c>
@@ -31448,8 +32111,14 @@
       <c r="CL110">
         <v>66.099999999999994</v>
       </c>
+      <c r="CM110">
+        <v>1671</v>
+      </c>
+      <c r="CN110">
+        <v>0.78096947935368044</v>
+      </c>
     </row>
-    <row r="111" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A111" t="s">
         <v>110</v>
       </c>
@@ -31720,8 +32389,14 @@
       <c r="CL111">
         <v>84.6</v>
       </c>
+      <c r="CM111">
+        <v>7899</v>
+      </c>
+      <c r="CN111">
+        <v>0.85770350677300922</v>
+      </c>
     </row>
-    <row r="112" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A112" t="s">
         <v>111</v>
       </c>
@@ -31992,8 +32667,14 @@
       <c r="CL112">
         <v>70.599999999999994</v>
       </c>
+      <c r="CM112">
+        <v>1301</v>
+      </c>
+      <c r="CN112">
+        <v>0.84780937740199847</v>
+      </c>
     </row>
-    <row r="113" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A113" t="s">
         <v>112</v>
       </c>
@@ -32264,8 +32945,14 @@
       <c r="CL113">
         <v>71.099999999999994</v>
       </c>
+      <c r="CM113">
+        <v>1661</v>
+      </c>
+      <c r="CN113">
+        <v>0.8892233594220349</v>
+      </c>
     </row>
-    <row r="114" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A114" t="s">
         <v>113</v>
       </c>
@@ -32536,8 +33223,14 @@
       <c r="CL114">
         <v>86.6</v>
       </c>
+      <c r="CM114">
+        <v>965</v>
+      </c>
+      <c r="CN114">
+        <v>0.81554404145077719</v>
+      </c>
     </row>
-    <row r="115" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A115" t="s">
         <v>114</v>
       </c>
@@ -32808,8 +33501,14 @@
       <c r="CL115">
         <v>68</v>
       </c>
+      <c r="CM115">
+        <v>13409</v>
+      </c>
+      <c r="CN115">
+        <v>0.83182936833470056</v>
+      </c>
     </row>
-    <row r="116" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A116" t="s">
         <v>115</v>
       </c>
@@ -33080,8 +33779,14 @@
       <c r="CL116">
         <v>75.2</v>
       </c>
+      <c r="CM116">
+        <v>14041</v>
+      </c>
+      <c r="CN116">
+        <v>0.8449540631009187</v>
+      </c>
     </row>
-    <row r="117" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A117" t="s">
         <v>116</v>
       </c>
@@ -33352,8 +34057,14 @@
       <c r="CL117">
         <v>76.900000000000006</v>
       </c>
+      <c r="CM117">
+        <v>510</v>
+      </c>
+      <c r="CN117">
+        <v>0.86862745098039218</v>
+      </c>
     </row>
-    <row r="118" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A118" t="s">
         <v>117</v>
       </c>
@@ -33624,8 +34335,14 @@
       <c r="CL118">
         <v>69.599999999999994</v>
       </c>
+      <c r="CM118">
+        <v>1482</v>
+      </c>
+      <c r="CN118">
+        <v>0.82253711201079627</v>
+      </c>
     </row>
-    <row r="119" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A119" t="s">
         <v>118</v>
       </c>
@@ -33896,8 +34613,14 @@
       <c r="CL119">
         <v>75.400000000000006</v>
       </c>
+      <c r="CM119">
+        <v>5203</v>
+      </c>
+      <c r="CN119">
+        <v>0.76551989236978668</v>
+      </c>
     </row>
-    <row r="120" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A120" t="s">
         <v>119</v>
       </c>
@@ -34168,8 +34891,14 @@
       <c r="CL120">
         <v>71.3</v>
       </c>
+      <c r="CM120">
+        <v>238</v>
+      </c>
+      <c r="CN120">
+        <v>0.55882352941176472</v>
+      </c>
     </row>
-    <row r="121" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A121" t="s">
         <v>120</v>
       </c>
@@ -34440,8 +35169,14 @@
       <c r="CL121">
         <v>33.200000000000003</v>
       </c>
+      <c r="CM121">
+        <v>2912</v>
+      </c>
+      <c r="CN121">
+        <v>0.77026098901098905</v>
+      </c>
     </row>
-    <row r="122" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A122" t="s">
         <v>121</v>
       </c>
@@ -34712,8 +35447,14 @@
       <c r="CL122">
         <v>63.8</v>
       </c>
+      <c r="CM122">
+        <v>10493</v>
+      </c>
+      <c r="CN122">
+        <v>0.64366720670923472</v>
+      </c>
     </row>
-    <row r="123" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A123" t="s">
         <v>122</v>
       </c>
@@ -34984,8 +35725,14 @@
       <c r="CL123">
         <v>53.3</v>
       </c>
+      <c r="CM123">
+        <v>2666</v>
+      </c>
+      <c r="CN123">
+        <v>0.76106526631657911</v>
+      </c>
     </row>
-    <row r="124" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A124" t="s">
         <v>123</v>
       </c>
@@ -35256,8 +36003,14 @@
       <c r="CL124">
         <v>77.099999999999994</v>
       </c>
+      <c r="CM124">
+        <v>1992</v>
+      </c>
+      <c r="CN124">
+        <v>0.57530120481927716</v>
+      </c>
     </row>
-    <row r="125" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A125" t="s">
         <v>124</v>
       </c>
@@ -35528,8 +36281,14 @@
       <c r="CL125">
         <v>63.9</v>
       </c>
+      <c r="CM125">
+        <v>1087</v>
+      </c>
+      <c r="CN125">
+        <v>0.60533578656853726</v>
+      </c>
     </row>
-    <row r="126" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A126" t="s">
         <v>125</v>
       </c>
@@ -35800,8 +36559,14 @@
       <c r="CL126">
         <v>54.2</v>
       </c>
+      <c r="CM126">
+        <v>1034</v>
+      </c>
+      <c r="CN126">
+        <v>0.78046421663442944</v>
+      </c>
     </row>
-    <row r="127" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A127" t="s">
         <v>126</v>
       </c>
@@ -36072,8 +36837,14 @@
       <c r="CL127">
         <v>69.400000000000006</v>
       </c>
+      <c r="CM127">
+        <v>1823</v>
+      </c>
+      <c r="CN127">
+        <v>0.79978058145913333</v>
+      </c>
     </row>
-    <row r="128" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A128" t="s">
         <v>127</v>
       </c>
@@ -36344,8 +37115,14 @@
       <c r="CL128">
         <v>69.2</v>
       </c>
+      <c r="CM128">
+        <v>2349</v>
+      </c>
+      <c r="CN128">
+        <v>0.84716900808854834</v>
+      </c>
     </row>
-    <row r="129" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A129" t="s">
         <v>128</v>
       </c>
@@ -36616,8 +37393,14 @@
       <c r="CL129">
         <v>88.4</v>
       </c>
+      <c r="CM129">
+        <v>6717</v>
+      </c>
+      <c r="CN129">
+        <v>0.82879261575107932</v>
+      </c>
     </row>
-    <row r="130" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A130" t="s">
         <v>129</v>
       </c>
@@ -36888,8 +37671,14 @@
       <c r="CL130">
         <v>67</v>
       </c>
+      <c r="CM130">
+        <v>2070</v>
+      </c>
+      <c r="CN130">
+        <v>0.82270531400966185</v>
+      </c>
     </row>
-    <row r="131" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A131" t="s">
         <v>130</v>
       </c>
@@ -37160,8 +37949,14 @@
       <c r="CL131">
         <v>72.900000000000006</v>
       </c>
+      <c r="CM131">
+        <v>1381</v>
+      </c>
+      <c r="CN131">
+        <v>0.80448950036205646</v>
+      </c>
     </row>
-    <row r="132" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A132" t="s">
         <v>131</v>
       </c>
@@ -37432,8 +38227,14 @@
       <c r="CL132">
         <v>88.5</v>
       </c>
+      <c r="CM132">
+        <v>2568</v>
+      </c>
+      <c r="CN132">
+        <v>0.84852024922118385</v>
+      </c>
     </row>
-    <row r="133" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A133" t="s">
         <v>132</v>
       </c>
@@ -37704,8 +38505,14 @@
       <c r="CL133">
         <v>74.7</v>
       </c>
+      <c r="CM133">
+        <v>10107</v>
+      </c>
+      <c r="CN133">
+        <v>0.82111407935094494</v>
+      </c>
     </row>
-    <row r="134" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A134" t="s">
         <v>133</v>
       </c>
@@ -37976,8 +38783,14 @@
       <c r="CL134">
         <v>65.8</v>
       </c>
+      <c r="CM134">
+        <v>2488</v>
+      </c>
+      <c r="CN134">
+        <v>0.75281350482315113</v>
+      </c>
     </row>
-    <row r="135" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A135" t="s">
         <v>134</v>
       </c>
@@ -38248,8 +39061,14 @@
       <c r="CL135">
         <v>61.6</v>
       </c>
+      <c r="CM135">
+        <v>3053</v>
+      </c>
+      <c r="CN135">
+        <v>0.83164100884376024</v>
+      </c>
     </row>
-    <row r="136" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A136" t="s">
         <v>135</v>
       </c>
@@ -38520,8 +39339,14 @@
       <c r="CL136">
         <v>75.8</v>
       </c>
+      <c r="CM136">
+        <v>1878</v>
+      </c>
+      <c r="CN136">
+        <v>0.78700745473908418</v>
+      </c>
     </row>
-    <row r="137" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A137" t="s">
         <v>136</v>
       </c>
@@ -38792,8 +39617,14 @@
       <c r="CL137">
         <v>72.3</v>
       </c>
+      <c r="CM137">
+        <v>2217</v>
+      </c>
+      <c r="CN137">
+        <v>0.79070816418583667</v>
+      </c>
     </row>
-    <row r="138" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A138" t="s">
         <v>137</v>
       </c>
@@ -39064,8 +39895,14 @@
       <c r="CL138">
         <v>64.599999999999994</v>
       </c>
+      <c r="CM138">
+        <v>2266</v>
+      </c>
+      <c r="CN138">
+        <v>0.83406884377758161</v>
+      </c>
     </row>
-    <row r="139" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A139" t="s">
         <v>138</v>
       </c>
@@ -39336,8 +40173,14 @@
       <c r="CL139">
         <v>76.900000000000006</v>
       </c>
+      <c r="CM139">
+        <v>7439</v>
+      </c>
+      <c r="CN139">
+        <v>0.85334050275574669</v>
+      </c>
     </row>
-    <row r="140" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A140" t="s">
         <v>139</v>
       </c>
@@ -39608,8 +40451,14 @@
       <c r="CL140">
         <v>75</v>
       </c>
+      <c r="CM140">
+        <v>4651</v>
+      </c>
+      <c r="CN140">
+        <v>0.89120619221672759</v>
+      </c>
     </row>
-    <row r="141" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A141" t="s">
         <v>140</v>
       </c>
@@ -39880,8 +40729,14 @@
       <c r="CL141">
         <v>76.099999999999994</v>
       </c>
+      <c r="CM141">
+        <v>476</v>
+      </c>
+      <c r="CN141">
+        <v>0.8214285714285714</v>
+      </c>
     </row>
-    <row r="142" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A142" t="s">
         <v>141</v>
       </c>
@@ -40152,8 +41007,14 @@
       <c r="CL142">
         <v>63</v>
       </c>
+      <c r="CM142">
+        <v>831</v>
+      </c>
+      <c r="CN142">
+        <v>0.8038507821901324</v>
+      </c>
     </row>
-    <row r="143" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A143" t="s">
         <v>142</v>
       </c>
@@ -40424,8 +41285,14 @@
       <c r="CL143">
         <v>71.400000000000006</v>
       </c>
+      <c r="CM143">
+        <v>1596</v>
+      </c>
+      <c r="CN143">
+        <v>0.83583959899749372</v>
+      </c>
     </row>
-    <row r="144" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A144" t="s">
         <v>143</v>
       </c>
@@ -40696,8 +41563,14 @@
       <c r="CL144">
         <v>75.099999999999994</v>
       </c>
+      <c r="CM144">
+        <v>3418</v>
+      </c>
+      <c r="CN144">
+        <v>0.82533645406670564</v>
+      </c>
     </row>
-    <row r="145" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A145" t="s">
         <v>144</v>
       </c>
@@ -40968,8 +41841,14 @@
       <c r="CL145">
         <v>69</v>
       </c>
+      <c r="CM145">
+        <v>554</v>
+      </c>
+      <c r="CN145">
+        <v>0.68231046931407946</v>
+      </c>
     </row>
-    <row r="146" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A146" t="s">
         <v>145</v>
       </c>
@@ -41240,8 +42119,14 @@
       <c r="CL146">
         <v>78.900000000000006</v>
       </c>
+      <c r="CM146">
+        <v>4377</v>
+      </c>
+      <c r="CN146">
+        <v>0.78958190541466755</v>
+      </c>
     </row>
-    <row r="147" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A147" t="s">
         <v>146</v>
       </c>
@@ -41512,8 +42397,14 @@
       <c r="CL147">
         <v>75.3</v>
       </c>
+      <c r="CM147">
+        <v>1198</v>
+      </c>
+      <c r="CN147">
+        <v>0.77796327212020033</v>
+      </c>
     </row>
-    <row r="148" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A148" t="s">
         <v>147</v>
       </c>
@@ -41784,8 +42675,14 @@
       <c r="CL148">
         <v>50.5</v>
       </c>
+      <c r="CM148">
+        <v>1127</v>
+      </c>
+      <c r="CN148">
+        <v>0.82076308784383323</v>
+      </c>
     </row>
-    <row r="149" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A149" t="s">
         <v>148</v>
       </c>
@@ -42056,8 +42953,14 @@
       <c r="CL149">
         <v>62.9</v>
       </c>
+      <c r="CM149">
+        <v>3174</v>
+      </c>
+      <c r="CN149">
+        <v>0.8412098298676749</v>
+      </c>
     </row>
-    <row r="150" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A150" t="s">
         <v>149</v>
       </c>
@@ -42328,8 +43231,14 @@
       <c r="CL150">
         <v>71.3</v>
       </c>
+      <c r="CM150">
+        <v>1706</v>
+      </c>
+      <c r="CN150">
+        <v>0.83001172332942552</v>
+      </c>
     </row>
-    <row r="151" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A151" t="s">
         <v>150</v>
       </c>
@@ -42600,8 +43509,14 @@
       <c r="CL151">
         <v>68.3</v>
       </c>
+      <c r="CM151">
+        <v>1796</v>
+      </c>
+      <c r="CN151">
+        <v>0.7048997772828508</v>
+      </c>
     </row>
-    <row r="152" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A152" t="s">
         <v>151</v>
       </c>
@@ -42872,8 +43787,14 @@
       <c r="CL152">
         <v>63.3</v>
       </c>
+      <c r="CM152">
+        <v>7348</v>
+      </c>
+      <c r="CN152">
+        <v>0.76769188894937401</v>
+      </c>
     </row>
-    <row r="153" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A153" t="s">
         <v>152</v>
       </c>
@@ -43144,8 +44065,14 @@
       <c r="CL153">
         <v>70.2</v>
       </c>
+      <c r="CM153">
+        <v>5943</v>
+      </c>
+      <c r="CN153">
+        <v>0.79538953390543499</v>
+      </c>
     </row>
-    <row r="154" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A154" t="s">
         <v>153</v>
       </c>
@@ -43416,8 +44343,14 @@
       <c r="CL154">
         <v>64.3</v>
       </c>
+      <c r="CM154">
+        <v>6176</v>
+      </c>
+      <c r="CN154">
+        <v>0.852979274611399</v>
+      </c>
     </row>
-    <row r="155" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A155" t="s">
         <v>154</v>
       </c>
@@ -43688,8 +44621,14 @@
       <c r="CL155">
         <v>80.599999999999994</v>
       </c>
+      <c r="CM155">
+        <v>10252</v>
+      </c>
+      <c r="CN155">
+        <v>0.82588763168162305</v>
+      </c>
     </row>
-    <row r="156" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A156" t="s">
         <v>155</v>
       </c>
@@ -43960,8 +44899,14 @@
       <c r="CL156">
         <v>75.7</v>
       </c>
+      <c r="CM156">
+        <v>5708</v>
+      </c>
+      <c r="CN156">
+        <v>0.83759635599159077</v>
+      </c>
     </row>
-    <row r="157" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A157" t="s">
         <v>156</v>
       </c>
@@ -44232,8 +45177,14 @@
       <c r="CL157">
         <v>76.7</v>
       </c>
+      <c r="CM157">
+        <v>914</v>
+      </c>
+      <c r="CN157">
+        <v>0.7286652078774617</v>
+      </c>
     </row>
-    <row r="158" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A158" t="s">
         <v>157</v>
       </c>
@@ -44504,8 +45455,14 @@
       <c r="CL158">
         <v>83.2</v>
       </c>
+      <c r="CM158">
+        <v>248</v>
+      </c>
+      <c r="CN158">
+        <v>0.63709677419354838</v>
+      </c>
     </row>
-    <row r="159" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A159" t="s">
         <v>158</v>
       </c>
@@ -44776,8 +45733,14 @@
       <c r="CL159">
         <v>81.7</v>
       </c>
+      <c r="CM159">
+        <v>801</v>
+      </c>
+      <c r="CN159">
+        <v>0.80149812734082393</v>
+      </c>
     </row>
-    <row r="160" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A160" t="s">
         <v>159</v>
       </c>
@@ -45048,8 +46011,14 @@
       <c r="CL160">
         <v>61</v>
       </c>
+      <c r="CM160">
+        <v>1499</v>
+      </c>
+      <c r="CN160">
+        <v>0.83455637091394264</v>
+      </c>
     </row>
-    <row r="161" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A161" t="s">
         <v>160</v>
       </c>
@@ -45320,8 +46289,14 @@
       <c r="CL161">
         <v>74.2</v>
       </c>
+      <c r="CM161">
+        <v>1397</v>
+      </c>
+      <c r="CN161">
+        <v>0.83679312813171081</v>
+      </c>
     </row>
-    <row r="162" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A162" t="s">
         <v>161</v>
       </c>
@@ -45592,8 +46567,14 @@
       <c r="CL162">
         <v>83.2</v>
       </c>
+      <c r="CM162">
+        <v>883</v>
+      </c>
+      <c r="CN162">
+        <v>0.77916194790486981</v>
+      </c>
     </row>
-    <row r="163" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A163" t="s">
         <v>162</v>
       </c>
@@ -45864,8 +46845,14 @@
       <c r="CL163">
         <v>67.900000000000006</v>
       </c>
+      <c r="CM163">
+        <v>822</v>
+      </c>
+      <c r="CN163">
+        <v>0.81021897810218979</v>
+      </c>
     </row>
-    <row r="164" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A164" t="s">
         <v>163</v>
       </c>
@@ -46136,8 +47123,14 @@
       <c r="CL164">
         <v>54.9</v>
       </c>
+      <c r="CM164">
+        <v>442</v>
+      </c>
+      <c r="CN164">
+        <v>0.79411764705882348</v>
+      </c>
     </row>
-    <row r="165" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A165" t="s">
         <v>164</v>
       </c>
@@ -46408,8 +47401,14 @@
       <c r="CL165">
         <v>67.900000000000006</v>
       </c>
+      <c r="CM165">
+        <v>1275</v>
+      </c>
+      <c r="CN165">
+        <v>0.71607843137254901</v>
+      </c>
     </row>
-    <row r="166" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A166" t="s">
         <v>165</v>
       </c>
@@ -46680,8 +47679,14 @@
       <c r="CL166">
         <v>73.3</v>
       </c>
+      <c r="CM166">
+        <v>775</v>
+      </c>
+      <c r="CN166">
+        <v>0.7870967741935484</v>
+      </c>
     </row>
-    <row r="167" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="167" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A167" t="s">
         <v>166</v>
       </c>
@@ -46952,8 +47957,14 @@
       <c r="CL167">
         <v>77.3</v>
       </c>
+      <c r="CM167">
+        <v>904</v>
+      </c>
+      <c r="CN167">
+        <v>0.73119469026548678</v>
+      </c>
     </row>
-    <row r="168" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="168" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A168" t="s">
         <v>167</v>
       </c>
@@ -47224,8 +48235,14 @@
       <c r="CL168">
         <v>65.7</v>
       </c>
+      <c r="CM168">
+        <v>752</v>
+      </c>
+      <c r="CN168">
+        <v>0.67420212765957444</v>
+      </c>
     </row>
-    <row r="169" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="169" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A169" t="s">
         <v>168</v>
       </c>
@@ -47496,8 +48513,14 @@
       <c r="CL169">
         <v>43.3</v>
       </c>
+      <c r="CM169">
+        <v>2494</v>
+      </c>
+      <c r="CN169">
+        <v>0.85846030473135526</v>
+      </c>
     </row>
-    <row r="170" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="170" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A170" t="s">
         <v>169</v>
       </c>
@@ -47768,8 +48791,14 @@
       <c r="CL170">
         <v>68.2</v>
       </c>
+      <c r="CM170">
+        <v>2814</v>
+      </c>
+      <c r="CN170">
+        <v>0.88841506751954513</v>
+      </c>
     </row>
-    <row r="171" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="171" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A171" t="s">
         <v>170</v>
       </c>
@@ -48040,8 +49069,14 @@
       <c r="CL171">
         <v>89.4</v>
       </c>
+      <c r="CM171">
+        <v>3281</v>
+      </c>
+      <c r="CN171">
+        <v>0.82657726302956414</v>
+      </c>
     </row>
-    <row r="172" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="172" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A172" t="s">
         <v>171</v>
       </c>
@@ -48312,8 +49347,14 @@
       <c r="CL172">
         <v>64.7</v>
       </c>
+      <c r="CM172">
+        <v>2638</v>
+      </c>
+      <c r="CN172">
+        <v>0.78658074298711145</v>
+      </c>
     </row>
-    <row r="173" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="173" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A173" t="s">
         <v>172</v>
       </c>
@@ -48584,8 +49625,14 @@
       <c r="CL173">
         <v>76.099999999999994</v>
       </c>
+      <c r="CM173">
+        <v>7504</v>
+      </c>
+      <c r="CN173">
+        <v>0.79677505330490406</v>
+      </c>
     </row>
-    <row r="174" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="174" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A174" t="s">
         <v>173</v>
       </c>
@@ -48856,8 +49903,14 @@
       <c r="CL174">
         <v>78.8</v>
       </c>
+      <c r="CM174">
+        <v>1170</v>
+      </c>
+      <c r="CN174">
+        <v>0.69401709401709399</v>
+      </c>
     </row>
-    <row r="175" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="175" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A175" t="s">
         <v>174</v>
       </c>
@@ -49128,8 +50181,14 @@
       <c r="CL175">
         <v>71.099999999999994</v>
       </c>
+      <c r="CM175">
+        <v>1369</v>
+      </c>
+      <c r="CN175">
+        <v>0.69539810080350617</v>
+      </c>
     </row>
-    <row r="176" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="176" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A176" t="s">
         <v>175</v>
       </c>
@@ -49400,8 +50459,14 @@
       <c r="CL176">
         <v>76.099999999999994</v>
       </c>
+      <c r="CM176">
+        <v>8364</v>
+      </c>
+      <c r="CN176">
+        <v>0.86358201817312286</v>
+      </c>
     </row>
-    <row r="177" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="177" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A177" t="s">
         <v>176</v>
       </c>
@@ -49672,8 +50737,14 @@
       <c r="CL177">
         <v>80.7</v>
       </c>
+      <c r="CM177">
+        <v>4098</v>
+      </c>
+      <c r="CN177">
+        <v>0.84016593460224498</v>
+      </c>
     </row>
-    <row r="178" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="178" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A178" t="s">
         <v>177</v>
       </c>
@@ -49944,8 +51015,14 @@
       <c r="CL178">
         <v>85.9</v>
       </c>
+      <c r="CM178">
+        <v>4269</v>
+      </c>
+      <c r="CN178">
+        <v>0.77465448582806273</v>
+      </c>
     </row>
-    <row r="179" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="179" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A179" t="s">
         <v>178</v>
       </c>
@@ -50216,8 +51293,14 @@
       <c r="CL179">
         <v>83.8</v>
       </c>
+      <c r="CM179">
+        <v>1559</v>
+      </c>
+      <c r="CN179">
+        <v>0.70942912123155866</v>
+      </c>
     </row>
-    <row r="180" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="180" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A180" t="s">
         <v>179</v>
       </c>
@@ -50488,8 +51571,14 @@
       <c r="CL180">
         <v>83.7</v>
       </c>
+      <c r="CM180">
+        <v>1246</v>
+      </c>
+      <c r="CN180">
+        <v>0.80658105939004821</v>
+      </c>
     </row>
-    <row r="181" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="181" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A181" t="s">
         <v>180</v>
       </c>
@@ -50760,8 +51849,14 @@
       <c r="CL181">
         <v>73.900000000000006</v>
       </c>
+      <c r="CM181">
+        <v>2027</v>
+      </c>
+      <c r="CN181">
+        <v>0.76221016280217069</v>
+      </c>
     </row>
-    <row r="182" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="182" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A182" t="s">
         <v>181</v>
       </c>
@@ -51032,8 +52127,14 @@
       <c r="CL182">
         <v>78.900000000000006</v>
       </c>
+      <c r="CM182">
+        <v>3090</v>
+      </c>
+      <c r="CN182">
+        <v>0.85177993527508089</v>
+      </c>
     </row>
-    <row r="183" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="183" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A183" t="s">
         <v>182</v>
       </c>
@@ -51304,8 +52405,14 @@
       <c r="CL183">
         <v>71.5</v>
       </c>
+      <c r="CM183">
+        <v>1683</v>
+      </c>
+      <c r="CN183">
+        <v>0.81937017231134879</v>
+      </c>
     </row>
-    <row r="184" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="184" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A184" t="s">
         <v>183</v>
       </c>
@@ -51576,8 +52683,14 @@
       <c r="CL184">
         <v>65.8</v>
       </c>
+      <c r="CM184">
+        <v>653</v>
+      </c>
+      <c r="CN184">
+        <v>0.75957120980091886</v>
+      </c>
     </row>
-    <row r="185" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="185" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A185" t="s">
         <v>184</v>
       </c>
@@ -51848,8 +52961,14 @@
       <c r="CL185">
         <v>72.900000000000006</v>
       </c>
+      <c r="CM185">
+        <v>1379</v>
+      </c>
+      <c r="CN185">
+        <v>0.87164612037708489</v>
+      </c>
     </row>
-    <row r="186" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="186" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A186" t="s">
         <v>185</v>
       </c>
@@ -52120,8 +53239,14 @@
       <c r="CL186">
         <v>67.900000000000006</v>
       </c>
+      <c r="CM186">
+        <v>5320</v>
+      </c>
+      <c r="CN186">
+        <v>0.73853383458646615</v>
+      </c>
     </row>
-    <row r="187" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="187" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A187" t="s">
         <v>186</v>
       </c>
@@ -52392,8 +53517,14 @@
       <c r="CL187">
         <v>72.7</v>
       </c>
+      <c r="CM187">
+        <v>7573</v>
+      </c>
+      <c r="CN187">
+        <v>0.83890136009507466</v>
+      </c>
     </row>
-    <row r="188" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="188" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A188" t="s">
         <v>187</v>
       </c>
@@ -52664,8 +53795,14 @@
       <c r="CL188">
         <v>59.8</v>
       </c>
+      <c r="CM188">
+        <v>5073</v>
+      </c>
+      <c r="CN188">
+        <v>0.76995860437610886</v>
+      </c>
     </row>
-    <row r="189" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="189" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A189" t="s">
         <v>188</v>
       </c>
@@ -52936,8 +54073,14 @@
       <c r="CL189">
         <v>72.099999999999994</v>
       </c>
+      <c r="CM189">
+        <v>492</v>
+      </c>
+      <c r="CN189">
+        <v>0.82926829268292679</v>
+      </c>
     </row>
-    <row r="190" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="190" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A190" t="s">
         <v>189</v>
       </c>
@@ -53208,8 +54351,14 @@
       <c r="CL190">
         <v>81</v>
       </c>
+      <c r="CM190">
+        <v>1453</v>
+      </c>
+      <c r="CN190">
+        <v>0.85891259463179626</v>
+      </c>
     </row>
-    <row r="191" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="191" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A191" t="s">
         <v>190</v>
       </c>
@@ -53480,8 +54629,14 @@
       <c r="CL191">
         <v>93.7</v>
       </c>
+      <c r="CM191">
+        <v>5889</v>
+      </c>
+      <c r="CN191">
+        <v>0.85073866530820175</v>
+      </c>
     </row>
-    <row r="192" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="192" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A192" t="s">
         <v>191</v>
       </c>
@@ -53752,8 +54907,14 @@
       <c r="CL192">
         <v>66.7</v>
       </c>
+      <c r="CM192">
+        <v>1095</v>
+      </c>
+      <c r="CN192">
+        <v>0.84748858447488584</v>
+      </c>
     </row>
-    <row r="193" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="193" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A193" t="s">
         <v>192</v>
       </c>
@@ -54024,8 +55185,14 @@
       <c r="CL193">
         <v>68</v>
       </c>
+      <c r="CM193">
+        <v>12375</v>
+      </c>
+      <c r="CN193">
+        <v>0.91991919191919191</v>
+      </c>
     </row>
-    <row r="194" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="194" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A194" t="s">
         <v>193</v>
       </c>
@@ -54296,8 +55463,14 @@
       <c r="CL194">
         <v>69.599999999999994</v>
       </c>
+      <c r="CM194">
+        <v>511</v>
+      </c>
+      <c r="CN194">
+        <v>0.80821917808219179</v>
+      </c>
     </row>
-    <row r="195" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="195" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A195" t="s">
         <v>194</v>
       </c>
@@ -54568,8 +55741,14 @@
       <c r="CL195">
         <v>60.5</v>
       </c>
+      <c r="CM195">
+        <v>1885</v>
+      </c>
+      <c r="CN195">
+        <v>0.75066312997347484</v>
+      </c>
     </row>
-    <row r="196" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="196" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A196" t="s">
         <v>195</v>
       </c>
@@ -54840,8 +56019,14 @@
       <c r="CL196">
         <v>84.3</v>
       </c>
+      <c r="CM196">
+        <v>596</v>
+      </c>
+      <c r="CN196">
+        <v>0.72315436241610742</v>
+      </c>
     </row>
-    <row r="197" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="197" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A197" t="s">
         <v>196</v>
       </c>
@@ -55112,8 +56297,14 @@
       <c r="CL197">
         <v>57.7</v>
       </c>
+      <c r="CM197">
+        <v>2575</v>
+      </c>
+      <c r="CN197">
+        <v>0.69475728155339811</v>
+      </c>
     </row>
-    <row r="198" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="198" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A198" t="s">
         <v>197</v>
       </c>
@@ -55384,8 +56575,14 @@
       <c r="CL198">
         <v>63.3</v>
       </c>
+      <c r="CM198">
+        <v>2259</v>
+      </c>
+      <c r="CN198">
+        <v>0.76715360779105801</v>
+      </c>
     </row>
-    <row r="199" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="199" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A199" t="s">
         <v>198</v>
       </c>
@@ -55656,8 +56853,14 @@
       <c r="CL199">
         <v>83.9</v>
       </c>
+      <c r="CM199">
+        <v>863</v>
+      </c>
+      <c r="CN199">
+        <v>0.7404403244495944</v>
+      </c>
     </row>
-    <row r="200" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="200" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A200" t="s">
         <v>199</v>
       </c>
@@ -55928,8 +57131,14 @@
       <c r="CL200">
         <v>84</v>
       </c>
+      <c r="CM200">
+        <v>1640</v>
+      </c>
+      <c r="CN200">
+        <v>0.85792682926829267</v>
+      </c>
     </row>
-    <row r="201" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="201" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A201" t="s">
         <v>200</v>
       </c>
@@ -56200,8 +57409,14 @@
       <c r="CL201">
         <v>102.3</v>
       </c>
+      <c r="CM201">
+        <v>3545</v>
+      </c>
+      <c r="CN201">
+        <v>0.79548660084626233</v>
+      </c>
     </row>
-    <row r="202" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="202" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A202" t="s">
         <v>201</v>
       </c>
@@ -56472,8 +57687,14 @@
       <c r="CL202">
         <v>80.900000000000006</v>
       </c>
+      <c r="CM202">
+        <v>1012</v>
+      </c>
+      <c r="CN202">
+        <v>0.77865612648221338</v>
+      </c>
     </row>
-    <row r="203" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="203" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A203" t="s">
         <v>202</v>
       </c>
@@ -56744,8 +57965,14 @@
       <c r="CL203">
         <v>73.8</v>
       </c>
+      <c r="CM203">
+        <v>6107</v>
+      </c>
+      <c r="CN203">
+        <v>0.87211396757818893</v>
+      </c>
     </row>
-    <row r="204" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="204" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A204" t="s">
         <v>203</v>
       </c>
@@ -57016,8 +58243,14 @@
       <c r="CL204">
         <v>82.9</v>
       </c>
+      <c r="CM204">
+        <v>982</v>
+      </c>
+      <c r="CN204">
+        <v>0.82586558044806513</v>
+      </c>
     </row>
-    <row r="205" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="205" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A205" t="s">
         <v>204</v>
       </c>
@@ -57288,8 +58521,14 @@
       <c r="CL205">
         <v>65.2</v>
       </c>
+      <c r="CM205">
+        <v>6276</v>
+      </c>
+      <c r="CN205">
+        <v>0.84257488846398976</v>
+      </c>
     </row>
-    <row r="206" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="206" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A206" t="s">
         <v>205</v>
       </c>
@@ -57560,8 +58799,14 @@
       <c r="CL206">
         <v>77.8</v>
       </c>
+      <c r="CM206">
+        <v>831</v>
+      </c>
+      <c r="CN206">
+        <v>0.56558363417569191</v>
+      </c>
     </row>
-    <row r="207" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="207" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A207" t="s">
         <v>206</v>
       </c>
@@ -57832,8 +59077,14 @@
       <c r="CL207">
         <v>65.400000000000006</v>
       </c>
+      <c r="CM207">
+        <v>2670</v>
+      </c>
+      <c r="CN207">
+        <v>0.74831460674157302</v>
+      </c>
     </row>
-    <row r="208" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="208" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A208" t="s">
         <v>207</v>
       </c>
@@ -58104,8 +59355,14 @@
       <c r="CL208">
         <v>76</v>
       </c>
+      <c r="CM208">
+        <v>8590</v>
+      </c>
+      <c r="CN208">
+        <v>0.82980209545983707</v>
+      </c>
     </row>
-    <row r="209" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="209" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A209" t="s">
         <v>208</v>
       </c>
@@ -58376,8 +59633,14 @@
       <c r="CL209">
         <v>74.400000000000006</v>
       </c>
+      <c r="CM209">
+        <v>2228</v>
+      </c>
+      <c r="CN209">
+        <v>0.82181328545780974</v>
+      </c>
     </row>
-    <row r="210" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="210" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A210" t="s">
         <v>209</v>
       </c>
@@ -58648,8 +59911,14 @@
       <c r="CL210">
         <v>87.6</v>
       </c>
+      <c r="CM210">
+        <v>562</v>
+      </c>
+      <c r="CN210">
+        <v>0.69395017793594305</v>
+      </c>
     </row>
-    <row r="211" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="211" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A211" t="s">
         <v>210</v>
       </c>
@@ -58920,8 +60189,14 @@
       <c r="CL211">
         <v>61.9</v>
       </c>
+      <c r="CM211">
+        <v>1727</v>
+      </c>
+      <c r="CN211">
+        <v>0.83497394325419805</v>
+      </c>
     </row>
-    <row r="212" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="212" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A212" t="s">
         <v>211</v>
       </c>
@@ -59192,8 +60467,14 @@
       <c r="CL212">
         <v>87.6</v>
       </c>
+      <c r="CM212">
+        <v>1591</v>
+      </c>
+      <c r="CN212">
+        <v>0.85229415461973601</v>
+      </c>
     </row>
-    <row r="213" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="213" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A213" t="s">
         <v>212</v>
       </c>
@@ -59464,8 +60745,14 @@
       <c r="CL213">
         <v>73.3</v>
       </c>
+      <c r="CM213">
+        <v>2122</v>
+      </c>
+      <c r="CN213">
+        <v>0.67624882186616397</v>
+      </c>
     </row>
-    <row r="214" spans="1:90" x14ac:dyDescent="0.2">
+    <row r="214" spans="1:92" x14ac:dyDescent="0.2">
       <c r="A214" t="s">
         <v>213</v>
       </c>
@@ -59739,6 +61026,7 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
   </tableParts>

</xml_diff>

<commit_message>
Solved GINI indeks problem
</commit_message>
<xml_diff>
--- a/Skupna tabela občine.xlsx
+++ b/Skupna tabela občine.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Desktop/Slovenija/Razširjeni kazalniki/streamlit_turisticne_regije_app_v4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{57967CCE-6C5D-0B42-B71A-5BDE1DBB06AE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE2AEED2-5374-3D44-9976-6B011A65A8D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="500" windowWidth="41720" windowHeight="27000" xr2:uid="{855CFD84-EAB2-0A43-A92D-394EE615CEA5}"/>
+    <workbookView xWindow="4020" yWindow="1680" windowWidth="41720" windowHeight="27000" xr2:uid="{855CFD84-EAB2-0A43-A92D-394EE615CEA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Skupna Tabela" sheetId="1" r:id="rId1"/>
@@ -1846,7 +1846,8 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="23.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="4" width="23.5" customWidth="1"/>
+    <col min="2" max="3" width="23.5" customWidth="1"/>
+    <col min="4" max="4" width="26.5" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="33.33203125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="24" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="27.6640625" bestFit="1" customWidth="1"/>

</xml_diff>

<commit_message>
Modified indeks view and GINI indeks display
</commit_message>
<xml_diff>
--- a/Skupna tabela občine.xlsx
+++ b/Skupna tabela občine.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Desktop/Slovenija/Razširjeni kazalniki/streamlit_turisticne_regije_app_v4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F9F5DBDC-0618-EF47-9648-5404E3CEEFAB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DBE14D-E92F-2F4A-8FD6-D741CF5AE026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="31220" yWindow="11140" windowWidth="54620" windowHeight="29900" xr2:uid="{855CFD84-EAB2-0A43-A92D-394EE615CEA5}"/>
+    <workbookView xWindow="22180" yWindow="14160" windowWidth="54620" windowHeight="29900" xr2:uid="{855CFD84-EAB2-0A43-A92D-394EE615CEA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Skupna Tabela" sheetId="1" r:id="rId1"/>
@@ -1400,69 +1400,6 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
@@ -1502,6 +1439,36 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
@@ -1529,7 +1496,40 @@
       <numFmt numFmtId="165" formatCode="0.0%"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -1582,22 +1582,22 @@
     <tableColumn id="106" xr3:uid="{F7FF3683-D64C-B84C-B130-995DD9ED829C}" name="Prenočitve turistov SKUPAJ - 2019"/>
     <tableColumn id="107" xr3:uid="{DFFD75B6-E4A3-0C44-9D48-17B3516A305A}" name="Prenočitve turistov Domači - 2019"/>
     <tableColumn id="108" xr3:uid="{584DB04E-60D9-1744-B6A1-6952195DC361}" name="Prenočitve turistov Tuji - 2019"/>
-    <tableColumn id="7" xr3:uid="{E209E213-8FD4-4C47-B297-1F887AE8D7A7}" name="Prenočitve turistov SKUPAJ - 2024" dataDxfId="84" totalsRowDxfId="54"/>
-    <tableColumn id="8" xr3:uid="{2911BC09-A9DE-DC43-94D4-9C9E6E23A668}" name="Prenočitve turistov Domači - 2024" dataDxfId="83" totalsRowDxfId="53"/>
-    <tableColumn id="9" xr3:uid="{F2E07E25-D318-EF4C-9D58-4F9D024FA8A8}" name="Prenočitve turistov Tuji - 2024" dataDxfId="82" totalsRowDxfId="52"/>
-    <tableColumn id="122" xr3:uid="{552065FC-30CB-E140-83A3-C3991B55A8C6}" name="Prenočitve turistov SKUPAJ - 2025" dataDxfId="81" totalsRowDxfId="51"/>
-    <tableColumn id="123" xr3:uid="{AA739D98-B21D-8C4B-8209-6847B58DF8F4}" name="Prenočitve turistov Domači - 2025" dataDxfId="80" totalsRowDxfId="50"/>
-    <tableColumn id="124" xr3:uid="{0D52A3F1-C861-A84F-A614-D77C5FA49216}" name="Prenočitve turistov Tuji - 2025" dataDxfId="79" totalsRowDxfId="49"/>
-    <tableColumn id="105" xr3:uid="{3F73618F-8B9D-9C40-9ABE-1663CD0B4B36}" name="Prenočitve - povprečno število prenočitev na mesec" dataDxfId="78" totalsRowDxfId="48"/>
-    <tableColumn id="109" xr3:uid="{B1220855-9F1D-CF43-9E92-775EB008AA16}" name="Delež tujih prenočitev - 2019" dataDxfId="77" totalsRowDxfId="47"/>
+    <tableColumn id="7" xr3:uid="{E209E213-8FD4-4C47-B297-1F887AE8D7A7}" name="Prenočitve turistov SKUPAJ - 2024" dataDxfId="84" totalsRowDxfId="83"/>
+    <tableColumn id="8" xr3:uid="{2911BC09-A9DE-DC43-94D4-9C9E6E23A668}" name="Prenočitve turistov Domači - 2024" dataDxfId="82" totalsRowDxfId="81"/>
+    <tableColumn id="9" xr3:uid="{F2E07E25-D318-EF4C-9D58-4F9D024FA8A8}" name="Prenočitve turistov Tuji - 2024" dataDxfId="80" totalsRowDxfId="79"/>
+    <tableColumn id="122" xr3:uid="{552065FC-30CB-E140-83A3-C3991B55A8C6}" name="Prenočitve turistov SKUPAJ - 2025" dataDxfId="78" totalsRowDxfId="77"/>
+    <tableColumn id="123" xr3:uid="{AA739D98-B21D-8C4B-8209-6847B58DF8F4}" name="Prenočitve turistov Domači - 2025" dataDxfId="76" totalsRowDxfId="75"/>
+    <tableColumn id="124" xr3:uid="{0D52A3F1-C861-A84F-A614-D77C5FA49216}" name="Prenočitve turistov Tuji - 2025" dataDxfId="74" totalsRowDxfId="73"/>
+    <tableColumn id="105" xr3:uid="{3F73618F-8B9D-9C40-9ABE-1663CD0B4B36}" name="Prenočitve - povprečno število prenočitev na mesec" dataDxfId="72" totalsRowDxfId="71"/>
+    <tableColumn id="109" xr3:uid="{B1220855-9F1D-CF43-9E92-775EB008AA16}" name="Delež tujih prenočitev - 2019" dataDxfId="70" totalsRowDxfId="69"/>
     <tableColumn id="10" xr3:uid="{AE7EC853-0402-A44C-9F12-18D82AF38827}" name="Delež tujih prenočitev - 2024"/>
     <tableColumn id="125" xr3:uid="{8BC79AC6-F78F-4B4D-9748-B88B6AFF69EE}" name="Delež tujih prenočitev - 2025"/>
     <tableColumn id="110" xr3:uid="{A139B468-44D6-C04C-9966-6DB28C506A45}" name="Rast števila prenočitev 2024/2019 - SKUPAJ"/>
     <tableColumn id="111" xr3:uid="{9040517C-15E6-8C4D-8D7F-E856E27F299C}" name="Rast števila prenočitev 2024/2019 - Domači"/>
     <tableColumn id="112" xr3:uid="{9A1AC9F7-3946-384A-8284-60731B1A7003}" name="Rast števila prenočitev 2024/2019 - Tuji"/>
-    <tableColumn id="126" xr3:uid="{37DB623B-8FCA-2E46-BB4A-C8A36B9D3AEE}" name="Rast števila prenočitev 2025/2019 - SKUPAJ" dataDxfId="76" totalsRowDxfId="46"/>
-    <tableColumn id="127" xr3:uid="{FB1CE38A-E750-9246-972D-AB5C38B8E853}" name="Rast števila prenočitev 2025/2019 - Domači" dataDxfId="75" totalsRowDxfId="45"/>
-    <tableColumn id="128" xr3:uid="{C06A9023-037E-AE4C-AF11-D1DBF757480E}" name="Rast števila prenočitev 2025/2019 - Tuji" dataDxfId="74" totalsRowDxfId="44"/>
+    <tableColumn id="126" xr3:uid="{37DB623B-8FCA-2E46-BB4A-C8A36B9D3AEE}" name="Rast števila prenočitev 2025/2019 - SKUPAJ" dataDxfId="68" totalsRowDxfId="67"/>
+    <tableColumn id="127" xr3:uid="{FB1CE38A-E750-9246-972D-AB5C38B8E853}" name="Rast števila prenočitev 2025/2019 - Domači" dataDxfId="66" totalsRowDxfId="65"/>
+    <tableColumn id="128" xr3:uid="{C06A9023-037E-AE4C-AF11-D1DBF757480E}" name="Rast števila prenočitev 2025/2019 - Tuji" dataDxfId="64" totalsRowDxfId="63"/>
     <tableColumn id="100" xr3:uid="{646738F1-12E5-3D42-B08F-732CB4BD71FB}" name="Delež vseh prenočitev - Domači trg - 2024"/>
     <tableColumn id="101" xr3:uid="{E13F778E-7B5E-764D-A93E-CE2E6F497E0A}" name="Delež vseh prenočitev - DACH trgi - 2024"/>
     <tableColumn id="97" xr3:uid="{4353E62C-3E00-A742-97A0-09F93BE31459}" name="Delež vseh prenočitev - Italijanski trg - 2024"/>
@@ -1614,42 +1614,42 @@
     <tableColumn id="134" xr3:uid="{47D138F1-3468-0446-A0A8-1298EA2CC048}" name="Delež vseh prenočitev - Prekomorski trgi (ZDA, VB, CAN, AU, Azija) - 2025"/>
     <tableColumn id="135" xr3:uid="{99963EE1-0660-E74E-B6D4-6DADD5F900F4}" name="Delež vseh prenočitev - Trgi JV Evrope - 2025"/>
     <tableColumn id="136" xr3:uid="{C21D36A1-E635-E346-9F0E-242FFBC2D5F9}" name="Delež vseh prenočitev - Vsi drugi tuji trgi - 2025"/>
-    <tableColumn id="11" xr3:uid="{5CF30DCA-BA0F-D047-9308-6222A89F2E07}" name="Prihodi turistov SKUPAJ - 2024" dataDxfId="73" totalsRowDxfId="43"/>
-    <tableColumn id="12" xr3:uid="{2608AA17-F184-2D44-B158-EC683F751D56}" name="Prihodi turistov Domači - 2024" dataDxfId="72" totalsRowDxfId="42"/>
-    <tableColumn id="13" xr3:uid="{D040950F-FE38-AF40-AC39-E818CABE1FE1}" name="Prihodi turistov Tuji - 2024" dataDxfId="71" totalsRowDxfId="41"/>
-    <tableColumn id="114" xr3:uid="{79DBE021-6724-BA4B-A6CC-BF8D5E62986D}" name="Prihodi turistov SKUPAJ - 2025" dataDxfId="70" totalsRowDxfId="40"/>
-    <tableColumn id="115" xr3:uid="{7330AE28-8ABF-1442-912F-D54E4863351F}" name="Prihodi turistov Domači - 2025" dataDxfId="69" totalsRowDxfId="39"/>
-    <tableColumn id="116" xr3:uid="{677B102C-DD5D-C542-98A6-030FC27E5DCE}" name="Prihodi turistov Tuji - 2025" dataDxfId="68" totalsRowDxfId="38"/>
-    <tableColumn id="92" xr3:uid="{260CB2C1-DC34-5F48-81C1-0035A515C7E8}" name="GINI Indeks - sezonskost prenočitev - 2024" dataDxfId="67" totalsRowDxfId="37"/>
-    <tableColumn id="113" xr3:uid="{6F600461-C50A-4040-BD92-B01925DC3C2B}" name="Gibanje GINI Indeksa prenoč. 2024/2019" dataDxfId="66" totalsRowDxfId="36"/>
-    <tableColumn id="120" xr3:uid="{78864389-753D-0644-96EE-43E33DC457C5}" name="GINI Indeks - sezonskost prenočitev - 2025" dataDxfId="65" totalsRowDxfId="35"/>
-    <tableColumn id="121" xr3:uid="{EB237473-7927-E543-9439-92CA8EF4944C}" name="Gibanje GINI Indeksa prenoč. 2025/2019" dataDxfId="64" totalsRowDxfId="34"/>
+    <tableColumn id="11" xr3:uid="{5CF30DCA-BA0F-D047-9308-6222A89F2E07}" name="Prihodi turistov SKUPAJ - 2024" dataDxfId="62" totalsRowDxfId="61"/>
+    <tableColumn id="12" xr3:uid="{2608AA17-F184-2D44-B158-EC683F751D56}" name="Prihodi turistov Domači - 2024" dataDxfId="60" totalsRowDxfId="59"/>
+    <tableColumn id="13" xr3:uid="{D040950F-FE38-AF40-AC39-E818CABE1FE1}" name="Prihodi turistov Tuji - 2024" dataDxfId="58" totalsRowDxfId="57"/>
+    <tableColumn id="114" xr3:uid="{79DBE021-6724-BA4B-A6CC-BF8D5E62986D}" name="Prihodi turistov SKUPAJ - 2025" dataDxfId="56" totalsRowDxfId="55"/>
+    <tableColumn id="115" xr3:uid="{7330AE28-8ABF-1442-912F-D54E4863351F}" name="Prihodi turistov Domači - 2025" dataDxfId="54" totalsRowDxfId="53"/>
+    <tableColumn id="116" xr3:uid="{677B102C-DD5D-C542-98A6-030FC27E5DCE}" name="Prihodi turistov Tuji - 2025" dataDxfId="52" totalsRowDxfId="51"/>
+    <tableColumn id="92" xr3:uid="{260CB2C1-DC34-5F48-81C1-0035A515C7E8}" name="GINI Indeks - sezonskost prenočitev - 2024" dataDxfId="50" totalsRowDxfId="49"/>
+    <tableColumn id="113" xr3:uid="{6F600461-C50A-4040-BD92-B01925DC3C2B}" name="Gibanje GINI Indeksa prenoč. 2024/2019" dataDxfId="48" totalsRowDxfId="47"/>
+    <tableColumn id="120" xr3:uid="{78864389-753D-0644-96EE-43E33DC457C5}" name="GINI Indeks - sezonskost prenočitev - 2025" dataDxfId="46" totalsRowDxfId="45"/>
+    <tableColumn id="121" xr3:uid="{EB237473-7927-E543-9439-92CA8EF4944C}" name="Gibanje GINI Indeksa prenoč. 2025/2019" dataDxfId="44" totalsRowDxfId="43"/>
     <tableColumn id="14" xr3:uid="{494C63A2-19AC-0544-861F-B7FA12714240}" name="PDB turistov SKUPAJ - 2024"/>
     <tableColumn id="15" xr3:uid="{A743FB1C-E3E3-8340-BA42-61AD9082C50D}" name="PDB turistov Domači - 2024"/>
     <tableColumn id="16" xr3:uid="{D6397E34-AE62-1B40-8641-B68E90F526C0}" name="PDB turistov Tuji - 2024"/>
     <tableColumn id="117" xr3:uid="{6885EC95-5659-F04B-A251-AE53BDE48149}" name="PDB turistov SKUPAJ - 2025"/>
     <tableColumn id="118" xr3:uid="{4E7DDFB8-17E3-2C4C-AC60-14DA7C782C4D}" name="PDB turistov Domači - 2025"/>
     <tableColumn id="119" xr3:uid="{91E8E2BD-823C-4543-991A-D421CEB98935}" name="PDB turistov Tuji - 2025"/>
-    <tableColumn id="17" xr3:uid="{FF46E309-259F-F74C-B4E3-7DF480EC498E}" name="Nastanitvene kapacitete - Nedeljive enote" totalsRowDxfId="33"/>
-    <tableColumn id="18" xr3:uid="{DFA7A743-7B9B-AC4B-B555-AB008106AD20}" name="Nastanitvene kapacitete - vsa ležišča" totalsRowDxfId="32"/>
-    <tableColumn id="19" xr3:uid="{978F1FBB-9333-EE42-8F86-066AF03E32F3}" name="Nastanitvene kapacitete - stalna ležišča" totalsRowDxfId="31"/>
-    <tableColumn id="20" xr3:uid="{36A5B684-693C-D046-A589-28E1F1CB9AD8}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote)_x0009_- Hoteli in podobni obrati" dataDxfId="63" totalsRowDxfId="30"/>
-    <tableColumn id="21" xr3:uid="{2B702555-9FD7-D940-90E2-CF22763449FC}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote)_x0009_- Kampi" dataDxfId="62" totalsRowDxfId="29"/>
-    <tableColumn id="22" xr3:uid="{B2C76693-F53B-BB47-B0BB-91CDFB3515C1}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote) - Druge vrste kapacitet" dataDxfId="61" totalsRowDxfId="28"/>
-    <tableColumn id="23" xr3:uid="{4DBA3760-7B2D-614B-8D1E-57BF8CACAD66}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Hoteli in podobni obrati" dataDxfId="60" totalsRowDxfId="27"/>
-    <tableColumn id="24" xr3:uid="{B83E8E03-6D6E-4749-935D-B72B0FDB49EF}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Kampi" dataDxfId="59" totalsRowDxfId="26"/>
-    <tableColumn id="25" xr3:uid="{14BC2615-1A3E-6548-803D-A6EE273713C4}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Druge vrste kapacitet" dataDxfId="58" totalsRowDxfId="25"/>
+    <tableColumn id="17" xr3:uid="{FF46E309-259F-F74C-B4E3-7DF480EC498E}" name="Nastanitvene kapacitete - Nedeljive enote" totalsRowDxfId="42"/>
+    <tableColumn id="18" xr3:uid="{DFA7A743-7B9B-AC4B-B555-AB008106AD20}" name="Nastanitvene kapacitete - vsa ležišča" totalsRowDxfId="41"/>
+    <tableColumn id="19" xr3:uid="{978F1FBB-9333-EE42-8F86-066AF03E32F3}" name="Nastanitvene kapacitete - stalna ležišča" totalsRowDxfId="40"/>
+    <tableColumn id="20" xr3:uid="{36A5B684-693C-D046-A589-28E1F1CB9AD8}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote)_x0009_- Hoteli in podobni obrati" dataDxfId="39" totalsRowDxfId="38"/>
+    <tableColumn id="21" xr3:uid="{2B702555-9FD7-D940-90E2-CF22763449FC}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote)_x0009_- Kampi" dataDxfId="37" totalsRowDxfId="36"/>
+    <tableColumn id="22" xr3:uid="{B2C76693-F53B-BB47-B0BB-91CDFB3515C1}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote) - Druge vrste kapacitet" dataDxfId="35" totalsRowDxfId="34"/>
+    <tableColumn id="23" xr3:uid="{4DBA3760-7B2D-614B-8D1E-57BF8CACAD66}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Hoteli in podobni obrati" dataDxfId="33" totalsRowDxfId="32"/>
+    <tableColumn id="24" xr3:uid="{B83E8E03-6D6E-4749-935D-B72B0FDB49EF}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Kampi" dataDxfId="31" totalsRowDxfId="30"/>
+    <tableColumn id="25" xr3:uid="{14BC2615-1A3E-6548-803D-A6EE273713C4}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Druge vrste kapacitet" dataDxfId="29" totalsRowDxfId="28"/>
     <tableColumn id="26" xr3:uid="{6B98A6DD-4A64-EE45-AE54-458C05388214}" name="Delež stalnih ležišč v Hotelih ipd."/>
     <tableColumn id="27" xr3:uid="{CC3F87E6-B3CD-E841-BCED-E5C77DFA385B}" name="Povprečna letna zasedenost staln. ležišč"/>
     <tableColumn id="28" xr3:uid="{36E12EEC-F431-7640-B38F-3F28A52A27A2}" name="Ocenjena povp. Letna zased. sob (nedeljivih enot)"/>
     <tableColumn id="29" xr3:uid="{E32E1653-4218-8144-AE1B-7DA0234BDD6B}" name="Pritisk turizma na družbeni prostor (število stalnih ležišč / 100 prebivalcev)"/>
     <tableColumn id="30" xr3:uid="{6235832E-2F71-6247-9BC2-BB497EF940F1}" name="Gostota turizma"/>
     <tableColumn id="31" xr3:uid="{6059D037-013F-3443-92BE-556256221BB9}" name="Intenzivnost turizma (število nočitev na dan / 100 prebivalcev)"/>
-    <tableColumn id="32" xr3:uid="{0EC9E9BB-E7DF-8F40-8DAC-C329014153B6}" name="Delovno aktivni v  turizmu (OECD/WTO)" totalsRowDxfId="24"/>
-    <tableColumn id="33" xr3:uid="{70783B5E-3FC1-DD44-9C4B-F29ABE2F730A}" name="Število zaposl. in samozaposl. v aktivnih podjetjih v Gostinstvu (I)" totalsRowDxfId="23"/>
-    <tableColumn id="34" xr3:uid="{55BC080C-8A66-C04E-A1E9-A6D4133CCFE0}" name="Zaposleni v Gostinstvu (I) v registr.podjetjih in s.p." dataDxfId="57" totalsRowDxfId="22"/>
-    <tableColumn id="35" xr3:uid="{88DF1418-F448-F64B-AB10-E2E30ADD50CE}" name="Zaposleni v nastan.dejav. (I55) v registr.podjetjih in s.p." dataDxfId="56" totalsRowDxfId="21"/>
-    <tableColumn id="36" xr3:uid="{135A837A-5EB5-2546-AB5F-35C76A605B6C}" name="Vsi delovni aktivni na območju" dataDxfId="55" totalsRowDxfId="20"/>
+    <tableColumn id="32" xr3:uid="{0EC9E9BB-E7DF-8F40-8DAC-C329014153B6}" name="Delovno aktivni v  turizmu (OECD/WTO)" totalsRowDxfId="27"/>
+    <tableColumn id="33" xr3:uid="{70783B5E-3FC1-DD44-9C4B-F29ABE2F730A}" name="Število zaposl. in samozaposl. v aktivnih podjetjih v Gostinstvu (I)" totalsRowDxfId="26"/>
+    <tableColumn id="34" xr3:uid="{55BC080C-8A66-C04E-A1E9-A6D4133CCFE0}" name="Zaposleni v Gostinstvu (I) v registr.podjetjih in s.p." dataDxfId="25" totalsRowDxfId="24"/>
+    <tableColumn id="35" xr3:uid="{88DF1418-F448-F64B-AB10-E2E30ADD50CE}" name="Zaposleni v nastan.dejav. (I55) v registr.podjetjih in s.p." dataDxfId="23" totalsRowDxfId="22"/>
+    <tableColumn id="36" xr3:uid="{135A837A-5EB5-2546-AB5F-35C76A605B6C}" name="Vsi delovni aktivni na območju" dataDxfId="21" totalsRowDxfId="20"/>
     <tableColumn id="37" xr3:uid="{52A7F38A-5C90-964D-B065-B17C7BA263D5}" name="Delež delovno aktivnih v turizmu (OECD/WTO)" totalsRowDxfId="19"/>
     <tableColumn id="38" xr3:uid="{C0F240E5-648C-7342-B26C-C8B4E0C3F6B4}" name="Število vseh vrst podjetij na območju" totalsRowDxfId="18"/>
     <tableColumn id="39" xr3:uid="{36A2CDB3-CA3D-9043-ADE8-DD7F31F3FE73}" name="Prihodek (v 1000 EUR) vseh podjetij na območju" totalsRowDxfId="17"/>

</xml_diff>

<commit_message>
Minor indicator name changes
</commit_message>
<xml_diff>
--- a/Skupna tabela občine.xlsx
+++ b/Skupna tabela občine.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/peter/Desktop/Slovenija/Razširjeni kazalniki/streamlit_turisticne_regije_app_v4/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59DBE14D-E92F-2F4A-8FD6-D741CF5AE026}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{035E900F-19A7-504E-ACA0-F742238BB4BD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="22180" yWindow="14160" windowWidth="54620" windowHeight="29900" xr2:uid="{855CFD84-EAB2-0A43-A92D-394EE615CEA5}"/>
+    <workbookView xWindow="11500" yWindow="13040" windowWidth="54620" windowHeight="29900" xr2:uid="{855CFD84-EAB2-0A43-A92D-394EE615CEA5}"/>
   </bookViews>
   <sheets>
     <sheet name="Skupna Tabela" sheetId="1" r:id="rId1"/>
@@ -731,9 +731,6 @@
     <t>Gostota turizma</t>
   </si>
   <si>
-    <t>Delovno aktivni v  turizmu (OECD/WTO)</t>
-  </si>
-  <si>
     <t>Zaposleni v Gostinstvu (I) v registr.podjetjih in s.p.</t>
   </si>
   <si>
@@ -1172,9 +1169,6 @@
     <t>Delež vseh prenočitev - Domači trg - 2024</t>
   </si>
   <si>
-    <t>Delež vseh prenočitev - DACH trgi - 2024</t>
-  </si>
-  <si>
     <t>Delež vseh prenočitev - Italijanski trg - 2024</t>
   </si>
   <si>
@@ -1188,9 +1182,6 @@
   </si>
   <si>
     <t>Delež vseh prenočitev - Vsi drugi tuji trgi - 2024</t>
-  </si>
-  <si>
-    <t>Delež vseh prenočitev - DACH trgi - 2025</t>
   </si>
   <si>
     <t>Delež vseh prenočitev - Italijanski trg - 2025</t>
@@ -1212,6 +1203,15 @@
   </si>
   <si>
     <t>Delež vseh prenočitev - Vzh.evropski trgi (PL,CZ,HU,SK,LIT,LTV,EST,RU,UKR) - 2024</t>
+  </si>
+  <si>
+    <t>Delež vseh prenočitev - DACH trgi (nemško govoreči trgi: D, A in CH) - 2024</t>
+  </si>
+  <si>
+    <t>Delež vseh prenočitev - DACH trgi (nemško govoreči trgi: D, A in CH) - 2025</t>
+  </si>
+  <si>
+    <t>Delovno aktivno prebivalstvo v turizmu (OECD/WTO)</t>
   </si>
 </sst>
 </file>
@@ -1400,6 +1400,69 @@
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="2" formatCode="0.00"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="0.0%"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="0.000"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="1" formatCode="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
@@ -1439,36 +1502,6 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
@@ -1496,40 +1529,7 @@
       <numFmt numFmtId="165" formatCode="0.0%"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="165" formatCode="0.0%"/>
-    </dxf>
-    <dxf>
       <numFmt numFmtId="164" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="164" formatCode="0.000"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="1" formatCode="0"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="1" formatCode="0"/>
@@ -1582,24 +1582,24 @@
     <tableColumn id="106" xr3:uid="{F7FF3683-D64C-B84C-B130-995DD9ED829C}" name="Prenočitve turistov SKUPAJ - 2019"/>
     <tableColumn id="107" xr3:uid="{DFFD75B6-E4A3-0C44-9D48-17B3516A305A}" name="Prenočitve turistov Domači - 2019"/>
     <tableColumn id="108" xr3:uid="{584DB04E-60D9-1744-B6A1-6952195DC361}" name="Prenočitve turistov Tuji - 2019"/>
-    <tableColumn id="7" xr3:uid="{E209E213-8FD4-4C47-B297-1F887AE8D7A7}" name="Prenočitve turistov SKUPAJ - 2024" dataDxfId="84" totalsRowDxfId="83"/>
-    <tableColumn id="8" xr3:uid="{2911BC09-A9DE-DC43-94D4-9C9E6E23A668}" name="Prenočitve turistov Domači - 2024" dataDxfId="82" totalsRowDxfId="81"/>
-    <tableColumn id="9" xr3:uid="{F2E07E25-D318-EF4C-9D58-4F9D024FA8A8}" name="Prenočitve turistov Tuji - 2024" dataDxfId="80" totalsRowDxfId="79"/>
-    <tableColumn id="122" xr3:uid="{552065FC-30CB-E140-83A3-C3991B55A8C6}" name="Prenočitve turistov SKUPAJ - 2025" dataDxfId="78" totalsRowDxfId="77"/>
-    <tableColumn id="123" xr3:uid="{AA739D98-B21D-8C4B-8209-6847B58DF8F4}" name="Prenočitve turistov Domači - 2025" dataDxfId="76" totalsRowDxfId="75"/>
-    <tableColumn id="124" xr3:uid="{0D52A3F1-C861-A84F-A614-D77C5FA49216}" name="Prenočitve turistov Tuji - 2025" dataDxfId="74" totalsRowDxfId="73"/>
-    <tableColumn id="105" xr3:uid="{3F73618F-8B9D-9C40-9ABE-1663CD0B4B36}" name="Prenočitve - povprečno število prenočitev na mesec" dataDxfId="72" totalsRowDxfId="71"/>
-    <tableColumn id="109" xr3:uid="{B1220855-9F1D-CF43-9E92-775EB008AA16}" name="Delež tujih prenočitev - 2019" dataDxfId="70" totalsRowDxfId="69"/>
+    <tableColumn id="7" xr3:uid="{E209E213-8FD4-4C47-B297-1F887AE8D7A7}" name="Prenočitve turistov SKUPAJ - 2024" dataDxfId="84" totalsRowDxfId="54"/>
+    <tableColumn id="8" xr3:uid="{2911BC09-A9DE-DC43-94D4-9C9E6E23A668}" name="Prenočitve turistov Domači - 2024" dataDxfId="83" totalsRowDxfId="53"/>
+    <tableColumn id="9" xr3:uid="{F2E07E25-D318-EF4C-9D58-4F9D024FA8A8}" name="Prenočitve turistov Tuji - 2024" dataDxfId="82" totalsRowDxfId="52"/>
+    <tableColumn id="122" xr3:uid="{552065FC-30CB-E140-83A3-C3991B55A8C6}" name="Prenočitve turistov SKUPAJ - 2025" dataDxfId="81" totalsRowDxfId="51"/>
+    <tableColumn id="123" xr3:uid="{AA739D98-B21D-8C4B-8209-6847B58DF8F4}" name="Prenočitve turistov Domači - 2025" dataDxfId="80" totalsRowDxfId="50"/>
+    <tableColumn id="124" xr3:uid="{0D52A3F1-C861-A84F-A614-D77C5FA49216}" name="Prenočitve turistov Tuji - 2025" dataDxfId="79" totalsRowDxfId="49"/>
+    <tableColumn id="105" xr3:uid="{3F73618F-8B9D-9C40-9ABE-1663CD0B4B36}" name="Prenočitve - povprečno število prenočitev na mesec" dataDxfId="78" totalsRowDxfId="48"/>
+    <tableColumn id="109" xr3:uid="{B1220855-9F1D-CF43-9E92-775EB008AA16}" name="Delež tujih prenočitev - 2019" dataDxfId="77" totalsRowDxfId="47"/>
     <tableColumn id="10" xr3:uid="{AE7EC853-0402-A44C-9F12-18D82AF38827}" name="Delež tujih prenočitev - 2024"/>
     <tableColumn id="125" xr3:uid="{8BC79AC6-F78F-4B4D-9748-B88B6AFF69EE}" name="Delež tujih prenočitev - 2025"/>
     <tableColumn id="110" xr3:uid="{A139B468-44D6-C04C-9966-6DB28C506A45}" name="Rast števila prenočitev 2024/2019 - SKUPAJ"/>
     <tableColumn id="111" xr3:uid="{9040517C-15E6-8C4D-8D7F-E856E27F299C}" name="Rast števila prenočitev 2024/2019 - Domači"/>
     <tableColumn id="112" xr3:uid="{9A1AC9F7-3946-384A-8284-60731B1A7003}" name="Rast števila prenočitev 2024/2019 - Tuji"/>
-    <tableColumn id="126" xr3:uid="{37DB623B-8FCA-2E46-BB4A-C8A36B9D3AEE}" name="Rast števila prenočitev 2025/2019 - SKUPAJ" dataDxfId="68" totalsRowDxfId="67"/>
-    <tableColumn id="127" xr3:uid="{FB1CE38A-E750-9246-972D-AB5C38B8E853}" name="Rast števila prenočitev 2025/2019 - Domači" dataDxfId="66" totalsRowDxfId="65"/>
-    <tableColumn id="128" xr3:uid="{C06A9023-037E-AE4C-AF11-D1DBF757480E}" name="Rast števila prenočitev 2025/2019 - Tuji" dataDxfId="64" totalsRowDxfId="63"/>
+    <tableColumn id="126" xr3:uid="{37DB623B-8FCA-2E46-BB4A-C8A36B9D3AEE}" name="Rast števila prenočitev 2025/2019 - SKUPAJ" dataDxfId="76" totalsRowDxfId="46"/>
+    <tableColumn id="127" xr3:uid="{FB1CE38A-E750-9246-972D-AB5C38B8E853}" name="Rast števila prenočitev 2025/2019 - Domači" dataDxfId="75" totalsRowDxfId="45"/>
+    <tableColumn id="128" xr3:uid="{C06A9023-037E-AE4C-AF11-D1DBF757480E}" name="Rast števila prenočitev 2025/2019 - Tuji" dataDxfId="74" totalsRowDxfId="44"/>
     <tableColumn id="100" xr3:uid="{646738F1-12E5-3D42-B08F-732CB4BD71FB}" name="Delež vseh prenočitev - Domači trg - 2024"/>
-    <tableColumn id="101" xr3:uid="{E13F778E-7B5E-764D-A93E-CE2E6F497E0A}" name="Delež vseh prenočitev - DACH trgi - 2024"/>
+    <tableColumn id="101" xr3:uid="{E13F778E-7B5E-764D-A93E-CE2E6F497E0A}" name="Delež vseh prenočitev - DACH trgi (nemško govoreči trgi: D, A in CH) - 2024"/>
     <tableColumn id="97" xr3:uid="{4353E62C-3E00-A742-97A0-09F93BE31459}" name="Delež vseh prenočitev - Italijanski trg - 2024"/>
     <tableColumn id="98" xr3:uid="{610ECDE2-6D04-A047-91E5-67167D9D99DB}" name="Delež vseh prenočitev - Vzh.evropski trgi (PL,CZ,HU,SK,LIT,LTV,EST,RU,UKR) - 2024"/>
     <tableColumn id="99" xr3:uid="{CD8B1967-9DD5-D64C-8F1F-161A789F5F39}" name="Delež vseh prenočitev - Drugi zah.in sev. evropski trgi (ES,P, F,Benelux, Skandinavske države) - 2024"/>
@@ -1607,49 +1607,49 @@
     <tableColumn id="95" xr3:uid="{D5614879-03D8-BE4D-8BB9-B1493690172E}" name="Delež vseh prenočitev - Trgi JV Evrope - 2024"/>
     <tableColumn id="94" xr3:uid="{5E5059F9-5ABE-A940-B1FB-98129F4C2C53}" name="Delež vseh prenočitev - Vsi drugi tuji trgi - 2024"/>
     <tableColumn id="129" xr3:uid="{E27E0654-A1C7-554D-B611-6461B0A40D2C}" name="Delež vseh prenočitev - Domači trg - 2025"/>
-    <tableColumn id="130" xr3:uid="{4545FC34-2172-0A4A-BE8D-4B9E0765B913}" name="Delež vseh prenočitev - DACH trgi - 2025"/>
+    <tableColumn id="130" xr3:uid="{4545FC34-2172-0A4A-BE8D-4B9E0765B913}" name="Delež vseh prenočitev - DACH trgi (nemško govoreči trgi: D, A in CH) - 2025"/>
     <tableColumn id="131" xr3:uid="{4929DA25-B637-2E44-A07F-E42459929194}" name="Delež vseh prenočitev - Italijanski trg - 2025"/>
     <tableColumn id="132" xr3:uid="{4FC91462-2081-1248-824D-7F98A0EE4F46}" name="Delež vseh prenočitev - Vzh.evropski trgi (PL,CZ,HU,SK,LIT,LTV,EST,RU,UKR) - 2025"/>
     <tableColumn id="133" xr3:uid="{293709AE-30D5-4548-9C79-951416DE2864}" name="Delež vseh prenočitev - Drugi zah.in sev. evropski trgi (ES,P, F,Benelux, Skandinavske države) - 2025"/>
     <tableColumn id="134" xr3:uid="{47D138F1-3468-0446-A0A8-1298EA2CC048}" name="Delež vseh prenočitev - Prekomorski trgi (ZDA, VB, CAN, AU, Azija) - 2025"/>
     <tableColumn id="135" xr3:uid="{99963EE1-0660-E74E-B6D4-6DADD5F900F4}" name="Delež vseh prenočitev - Trgi JV Evrope - 2025"/>
     <tableColumn id="136" xr3:uid="{C21D36A1-E635-E346-9F0E-242FFBC2D5F9}" name="Delež vseh prenočitev - Vsi drugi tuji trgi - 2025"/>
-    <tableColumn id="11" xr3:uid="{5CF30DCA-BA0F-D047-9308-6222A89F2E07}" name="Prihodi turistov SKUPAJ - 2024" dataDxfId="62" totalsRowDxfId="61"/>
-    <tableColumn id="12" xr3:uid="{2608AA17-F184-2D44-B158-EC683F751D56}" name="Prihodi turistov Domači - 2024" dataDxfId="60" totalsRowDxfId="59"/>
-    <tableColumn id="13" xr3:uid="{D040950F-FE38-AF40-AC39-E818CABE1FE1}" name="Prihodi turistov Tuji - 2024" dataDxfId="58" totalsRowDxfId="57"/>
-    <tableColumn id="114" xr3:uid="{79DBE021-6724-BA4B-A6CC-BF8D5E62986D}" name="Prihodi turistov SKUPAJ - 2025" dataDxfId="56" totalsRowDxfId="55"/>
-    <tableColumn id="115" xr3:uid="{7330AE28-8ABF-1442-912F-D54E4863351F}" name="Prihodi turistov Domači - 2025" dataDxfId="54" totalsRowDxfId="53"/>
-    <tableColumn id="116" xr3:uid="{677B102C-DD5D-C542-98A6-030FC27E5DCE}" name="Prihodi turistov Tuji - 2025" dataDxfId="52" totalsRowDxfId="51"/>
-    <tableColumn id="92" xr3:uid="{260CB2C1-DC34-5F48-81C1-0035A515C7E8}" name="GINI Indeks - sezonskost prenočitev - 2024" dataDxfId="50" totalsRowDxfId="49"/>
-    <tableColumn id="113" xr3:uid="{6F600461-C50A-4040-BD92-B01925DC3C2B}" name="Gibanje GINI Indeksa prenoč. 2024/2019" dataDxfId="48" totalsRowDxfId="47"/>
-    <tableColumn id="120" xr3:uid="{78864389-753D-0644-96EE-43E33DC457C5}" name="GINI Indeks - sezonskost prenočitev - 2025" dataDxfId="46" totalsRowDxfId="45"/>
-    <tableColumn id="121" xr3:uid="{EB237473-7927-E543-9439-92CA8EF4944C}" name="Gibanje GINI Indeksa prenoč. 2025/2019" dataDxfId="44" totalsRowDxfId="43"/>
+    <tableColumn id="11" xr3:uid="{5CF30DCA-BA0F-D047-9308-6222A89F2E07}" name="Prihodi turistov SKUPAJ - 2024" dataDxfId="73" totalsRowDxfId="43"/>
+    <tableColumn id="12" xr3:uid="{2608AA17-F184-2D44-B158-EC683F751D56}" name="Prihodi turistov Domači - 2024" dataDxfId="72" totalsRowDxfId="42"/>
+    <tableColumn id="13" xr3:uid="{D040950F-FE38-AF40-AC39-E818CABE1FE1}" name="Prihodi turistov Tuji - 2024" dataDxfId="71" totalsRowDxfId="41"/>
+    <tableColumn id="114" xr3:uid="{79DBE021-6724-BA4B-A6CC-BF8D5E62986D}" name="Prihodi turistov SKUPAJ - 2025" dataDxfId="70" totalsRowDxfId="40"/>
+    <tableColumn id="115" xr3:uid="{7330AE28-8ABF-1442-912F-D54E4863351F}" name="Prihodi turistov Domači - 2025" dataDxfId="69" totalsRowDxfId="39"/>
+    <tableColumn id="116" xr3:uid="{677B102C-DD5D-C542-98A6-030FC27E5DCE}" name="Prihodi turistov Tuji - 2025" dataDxfId="68" totalsRowDxfId="38"/>
+    <tableColumn id="92" xr3:uid="{260CB2C1-DC34-5F48-81C1-0035A515C7E8}" name="GINI Indeks - sezonskost prenočitev - 2024" dataDxfId="67" totalsRowDxfId="37"/>
+    <tableColumn id="113" xr3:uid="{6F600461-C50A-4040-BD92-B01925DC3C2B}" name="Gibanje GINI Indeksa prenoč. 2024/2019" dataDxfId="66" totalsRowDxfId="36"/>
+    <tableColumn id="120" xr3:uid="{78864389-753D-0644-96EE-43E33DC457C5}" name="GINI Indeks - sezonskost prenočitev - 2025" dataDxfId="65" totalsRowDxfId="35"/>
+    <tableColumn id="121" xr3:uid="{EB237473-7927-E543-9439-92CA8EF4944C}" name="Gibanje GINI Indeksa prenoč. 2025/2019" dataDxfId="64" totalsRowDxfId="34"/>
     <tableColumn id="14" xr3:uid="{494C63A2-19AC-0544-861F-B7FA12714240}" name="PDB turistov SKUPAJ - 2024"/>
     <tableColumn id="15" xr3:uid="{A743FB1C-E3E3-8340-BA42-61AD9082C50D}" name="PDB turistov Domači - 2024"/>
     <tableColumn id="16" xr3:uid="{D6397E34-AE62-1B40-8641-B68E90F526C0}" name="PDB turistov Tuji - 2024"/>
     <tableColumn id="117" xr3:uid="{6885EC95-5659-F04B-A251-AE53BDE48149}" name="PDB turistov SKUPAJ - 2025"/>
     <tableColumn id="118" xr3:uid="{4E7DDFB8-17E3-2C4C-AC60-14DA7C782C4D}" name="PDB turistov Domači - 2025"/>
     <tableColumn id="119" xr3:uid="{91E8E2BD-823C-4543-991A-D421CEB98935}" name="PDB turistov Tuji - 2025"/>
-    <tableColumn id="17" xr3:uid="{FF46E309-259F-F74C-B4E3-7DF480EC498E}" name="Nastanitvene kapacitete - Nedeljive enote" totalsRowDxfId="42"/>
-    <tableColumn id="18" xr3:uid="{DFA7A743-7B9B-AC4B-B555-AB008106AD20}" name="Nastanitvene kapacitete - vsa ležišča" totalsRowDxfId="41"/>
-    <tableColumn id="19" xr3:uid="{978F1FBB-9333-EE42-8F86-066AF03E32F3}" name="Nastanitvene kapacitete - stalna ležišča" totalsRowDxfId="40"/>
-    <tableColumn id="20" xr3:uid="{36A5B684-693C-D046-A589-28E1F1CB9AD8}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote)_x0009_- Hoteli in podobni obrati" dataDxfId="39" totalsRowDxfId="38"/>
-    <tableColumn id="21" xr3:uid="{2B702555-9FD7-D940-90E2-CF22763449FC}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote)_x0009_- Kampi" dataDxfId="37" totalsRowDxfId="36"/>
-    <tableColumn id="22" xr3:uid="{B2C76693-F53B-BB47-B0BB-91CDFB3515C1}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote) - Druge vrste kapacitet" dataDxfId="35" totalsRowDxfId="34"/>
-    <tableColumn id="23" xr3:uid="{4DBA3760-7B2D-614B-8D1E-57BF8CACAD66}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Hoteli in podobni obrati" dataDxfId="33" totalsRowDxfId="32"/>
-    <tableColumn id="24" xr3:uid="{B83E8E03-6D6E-4749-935D-B72B0FDB49EF}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Kampi" dataDxfId="31" totalsRowDxfId="30"/>
-    <tableColumn id="25" xr3:uid="{14BC2615-1A3E-6548-803D-A6EE273713C4}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Druge vrste kapacitet" dataDxfId="29" totalsRowDxfId="28"/>
+    <tableColumn id="17" xr3:uid="{FF46E309-259F-F74C-B4E3-7DF480EC498E}" name="Nastanitvene kapacitete - Nedeljive enote" totalsRowDxfId="33"/>
+    <tableColumn id="18" xr3:uid="{DFA7A743-7B9B-AC4B-B555-AB008106AD20}" name="Nastanitvene kapacitete - vsa ležišča" totalsRowDxfId="32"/>
+    <tableColumn id="19" xr3:uid="{978F1FBB-9333-EE42-8F86-066AF03E32F3}" name="Nastanitvene kapacitete - stalna ležišča" totalsRowDxfId="31"/>
+    <tableColumn id="20" xr3:uid="{36A5B684-693C-D046-A589-28E1F1CB9AD8}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote)_x0009_- Hoteli in podobni obrati" dataDxfId="63" totalsRowDxfId="30"/>
+    <tableColumn id="21" xr3:uid="{2B702555-9FD7-D940-90E2-CF22763449FC}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote)_x0009_- Kampi" dataDxfId="62" totalsRowDxfId="29"/>
+    <tableColumn id="22" xr3:uid="{B2C76693-F53B-BB47-B0BB-91CDFB3515C1}" name="Struktura nastanitvenih kapacitet - Sobe (nedeljive enote) - Druge vrste kapacitet" dataDxfId="61" totalsRowDxfId="28"/>
+    <tableColumn id="23" xr3:uid="{4DBA3760-7B2D-614B-8D1E-57BF8CACAD66}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Hoteli in podobni obrati" dataDxfId="60" totalsRowDxfId="27"/>
+    <tableColumn id="24" xr3:uid="{B83E8E03-6D6E-4749-935D-B72B0FDB49EF}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Kampi" dataDxfId="59" totalsRowDxfId="26"/>
+    <tableColumn id="25" xr3:uid="{14BC2615-1A3E-6548-803D-A6EE273713C4}" name="Struktura nastanitvenih kapacitet - Stalna ležišča - Druge vrste kapacitet" dataDxfId="58" totalsRowDxfId="25"/>
     <tableColumn id="26" xr3:uid="{6B98A6DD-4A64-EE45-AE54-458C05388214}" name="Delež stalnih ležišč v Hotelih ipd."/>
     <tableColumn id="27" xr3:uid="{CC3F87E6-B3CD-E841-BCED-E5C77DFA385B}" name="Povprečna letna zasedenost staln. ležišč"/>
     <tableColumn id="28" xr3:uid="{36E12EEC-F431-7640-B38F-3F28A52A27A2}" name="Ocenjena povp. Letna zased. sob (nedeljivih enot)"/>
     <tableColumn id="29" xr3:uid="{E32E1653-4218-8144-AE1B-7DA0234BDD6B}" name="Pritisk turizma na družbeni prostor (število stalnih ležišč / 100 prebivalcev)"/>
     <tableColumn id="30" xr3:uid="{6235832E-2F71-6247-9BC2-BB497EF940F1}" name="Gostota turizma"/>
     <tableColumn id="31" xr3:uid="{6059D037-013F-3443-92BE-556256221BB9}" name="Intenzivnost turizma (število nočitev na dan / 100 prebivalcev)"/>
-    <tableColumn id="32" xr3:uid="{0EC9E9BB-E7DF-8F40-8DAC-C329014153B6}" name="Delovno aktivni v  turizmu (OECD/WTO)" totalsRowDxfId="27"/>
-    <tableColumn id="33" xr3:uid="{70783B5E-3FC1-DD44-9C4B-F29ABE2F730A}" name="Število zaposl. in samozaposl. v aktivnih podjetjih v Gostinstvu (I)" totalsRowDxfId="26"/>
-    <tableColumn id="34" xr3:uid="{55BC080C-8A66-C04E-A1E9-A6D4133CCFE0}" name="Zaposleni v Gostinstvu (I) v registr.podjetjih in s.p." dataDxfId="25" totalsRowDxfId="24"/>
-    <tableColumn id="35" xr3:uid="{88DF1418-F448-F64B-AB10-E2E30ADD50CE}" name="Zaposleni v nastan.dejav. (I55) v registr.podjetjih in s.p." dataDxfId="23" totalsRowDxfId="22"/>
-    <tableColumn id="36" xr3:uid="{135A837A-5EB5-2546-AB5F-35C76A605B6C}" name="Vsi delovni aktivni na območju" dataDxfId="21" totalsRowDxfId="20"/>
+    <tableColumn id="32" xr3:uid="{0EC9E9BB-E7DF-8F40-8DAC-C329014153B6}" name="Delovno aktivno prebivalstvo v turizmu (OECD/WTO)" totalsRowDxfId="24"/>
+    <tableColumn id="33" xr3:uid="{70783B5E-3FC1-DD44-9C4B-F29ABE2F730A}" name="Število zaposl. in samozaposl. v aktivnih podjetjih v Gostinstvu (I)" totalsRowDxfId="23"/>
+    <tableColumn id="34" xr3:uid="{55BC080C-8A66-C04E-A1E9-A6D4133CCFE0}" name="Zaposleni v Gostinstvu (I) v registr.podjetjih in s.p." dataDxfId="57" totalsRowDxfId="22"/>
+    <tableColumn id="35" xr3:uid="{88DF1418-F448-F64B-AB10-E2E30ADD50CE}" name="Zaposleni v nastan.dejav. (I55) v registr.podjetjih in s.p." dataDxfId="56" totalsRowDxfId="21"/>
+    <tableColumn id="36" xr3:uid="{135A837A-5EB5-2546-AB5F-35C76A605B6C}" name="Vsi delovni aktivni na območju" dataDxfId="55" totalsRowDxfId="20"/>
     <tableColumn id="37" xr3:uid="{52A7F38A-5C90-964D-B065-B17C7BA263D5}" name="Delež delovno aktivnih v turizmu (OECD/WTO)" totalsRowDxfId="19"/>
     <tableColumn id="38" xr3:uid="{C0F240E5-648C-7342-B26C-C8B4E0C3F6B4}" name="Število vseh vrst podjetij na območju" totalsRowDxfId="18"/>
     <tableColumn id="39" xr3:uid="{36A2CDB3-CA3D-9043-ADE8-DD7F31F3FE73}" name="Prihodek (v 1000 EUR) vseh podjetij na območju" totalsRowDxfId="17"/>
@@ -2126,13 +2126,13 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
       <c r="D1" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="E1" t="s">
-        <v>326</v>
+        <v>325</v>
       </c>
       <c r="F1" t="s">
         <v>214</v>
@@ -2141,7 +2141,7 @@
         <v>225</v>
       </c>
       <c r="H1" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="I1" t="s">
         <v>224</v>
@@ -2150,184 +2150,184 @@
         <v>226</v>
       </c>
       <c r="K1" t="s">
+        <v>341</v>
+      </c>
+      <c r="L1" t="s">
+        <v>343</v>
+      </c>
+      <c r="M1" t="s">
+        <v>344</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="O1" s="1" t="s">
         <v>342</v>
       </c>
-      <c r="L1" t="s">
-        <v>344</v>
-      </c>
-      <c r="M1" t="s">
+      <c r="P1" s="1" t="s">
         <v>345</v>
       </c>
-      <c r="N1" s="1" t="s">
-        <v>341</v>
-      </c>
-      <c r="O1" s="1" t="s">
-        <v>343</v>
-      </c>
-      <c r="P1" s="1" t="s">
+      <c r="Q1" s="1" t="s">
+        <v>369</v>
+      </c>
+      <c r="R1" s="1" t="s">
+        <v>370</v>
+      </c>
+      <c r="S1" s="1" t="s">
+        <v>368</v>
+      </c>
+      <c r="T1" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="U1" s="3" t="s">
+        <v>347</v>
+      </c>
+      <c r="V1" t="s">
         <v>346</v>
       </c>
-      <c r="Q1" s="1" t="s">
-        <v>370</v>
-      </c>
-      <c r="R1" s="1" t="s">
+      <c r="W1" t="s">
         <v>371</v>
       </c>
-      <c r="S1" s="1" t="s">
-        <v>369</v>
-      </c>
-      <c r="T1" s="1" t="s">
+      <c r="X1" t="s">
+        <v>348</v>
+      </c>
+      <c r="Y1" t="s">
+        <v>350</v>
+      </c>
+      <c r="Z1" t="s">
+        <v>349</v>
+      </c>
+      <c r="AA1" s="4" t="s">
+        <v>372</v>
+      </c>
+      <c r="AB1" s="4" t="s">
+        <v>373</v>
+      </c>
+      <c r="AC1" s="4" t="s">
+        <v>374</v>
+      </c>
+      <c r="AD1" t="s">
+        <v>376</v>
+      </c>
+      <c r="AE1" t="s">
+        <v>389</v>
+      </c>
+      <c r="AF1" t="s">
+        <v>377</v>
+      </c>
+      <c r="AG1" t="s">
+        <v>388</v>
+      </c>
+      <c r="AH1" t="s">
+        <v>378</v>
+      </c>
+      <c r="AI1" t="s">
+        <v>379</v>
+      </c>
+      <c r="AJ1" t="s">
+        <v>380</v>
+      </c>
+      <c r="AK1" t="s">
+        <v>381</v>
+      </c>
+      <c r="AL1" t="s">
+        <v>375</v>
+      </c>
+      <c r="AM1" t="s">
+        <v>390</v>
+      </c>
+      <c r="AN1" t="s">
+        <v>382</v>
+      </c>
+      <c r="AO1" t="s">
+        <v>383</v>
+      </c>
+      <c r="AP1" t="s">
+        <v>384</v>
+      </c>
+      <c r="AQ1" t="s">
+        <v>385</v>
+      </c>
+      <c r="AR1" t="s">
+        <v>386</v>
+      </c>
+      <c r="AS1" t="s">
+        <v>387</v>
+      </c>
+      <c r="AT1" s="1" t="s">
         <v>354</v>
       </c>
-      <c r="U1" s="3" t="s">
-        <v>348</v>
-      </c>
-      <c r="V1" t="s">
-        <v>347</v>
-      </c>
-      <c r="W1" t="s">
-        <v>372</v>
-      </c>
-      <c r="X1" t="s">
-        <v>349</v>
-      </c>
-      <c r="Y1" t="s">
+      <c r="AU1" s="1" t="s">
+        <v>355</v>
+      </c>
+      <c r="AV1" s="1" t="s">
+        <v>356</v>
+      </c>
+      <c r="AW1" s="1" t="s">
+        <v>358</v>
+      </c>
+      <c r="AX1" s="1" t="s">
+        <v>359</v>
+      </c>
+      <c r="AY1" s="1" t="s">
+        <v>357</v>
+      </c>
+      <c r="AZ1" s="2" t="s">
+        <v>352</v>
+      </c>
+      <c r="BA1" s="2" t="s">
         <v>351</v>
       </c>
-      <c r="Z1" t="s">
-        <v>350</v>
-      </c>
-      <c r="AA1" s="4" t="s">
-        <v>373</v>
-      </c>
-      <c r="AB1" s="4" t="s">
-        <v>374</v>
-      </c>
-      <c r="AC1" s="4" t="s">
-        <v>375</v>
-      </c>
-      <c r="AD1" t="s">
-        <v>377</v>
-      </c>
-      <c r="AE1" t="s">
-        <v>378</v>
-      </c>
-      <c r="AF1" t="s">
-        <v>379</v>
-      </c>
-      <c r="AG1" t="s">
-        <v>391</v>
-      </c>
-      <c r="AH1" t="s">
-        <v>380</v>
-      </c>
-      <c r="AI1" t="s">
-        <v>381</v>
-      </c>
-      <c r="AJ1" t="s">
-        <v>382</v>
-      </c>
-      <c r="AK1" t="s">
-        <v>383</v>
-      </c>
-      <c r="AL1" t="s">
-        <v>376</v>
-      </c>
-      <c r="AM1" t="s">
-        <v>384</v>
-      </c>
-      <c r="AN1" t="s">
-        <v>385</v>
-      </c>
-      <c r="AO1" t="s">
-        <v>386</v>
-      </c>
-      <c r="AP1" t="s">
-        <v>387</v>
-      </c>
-      <c r="AQ1" t="s">
-        <v>388</v>
-      </c>
-      <c r="AR1" t="s">
-        <v>389</v>
-      </c>
-      <c r="AS1" t="s">
-        <v>390</v>
-      </c>
-      <c r="AT1" s="1" t="s">
-        <v>355</v>
-      </c>
-      <c r="AU1" s="1" t="s">
-        <v>356</v>
-      </c>
-      <c r="AV1" s="1" t="s">
-        <v>357</v>
-      </c>
-      <c r="AW1" s="1" t="s">
-        <v>359</v>
-      </c>
-      <c r="AX1" s="1" t="s">
+      <c r="BB1" s="2" t="s">
         <v>360</v>
       </c>
-      <c r="AY1" s="1" t="s">
-        <v>358</v>
-      </c>
-      <c r="AZ1" s="2" t="s">
-        <v>353</v>
-      </c>
-      <c r="BA1" s="2" t="s">
-        <v>352</v>
-      </c>
-      <c r="BB1" s="2" t="s">
+      <c r="BC1" s="2" t="s">
         <v>361</v>
       </c>
-      <c r="BC1" s="2" t="s">
+      <c r="BD1" t="s">
         <v>362</v>
       </c>
-      <c r="BD1" t="s">
+      <c r="BE1" t="s">
         <v>363</v>
       </c>
-      <c r="BE1" t="s">
+      <c r="BF1" t="s">
         <v>364</v>
       </c>
-      <c r="BF1" t="s">
+      <c r="BG1" t="s">
         <v>365</v>
       </c>
-      <c r="BG1" t="s">
+      <c r="BH1" t="s">
         <v>366</v>
       </c>
-      <c r="BH1" t="s">
+      <c r="BI1" t="s">
         <v>367</v>
       </c>
-      <c r="BI1" t="s">
-        <v>368</v>
-      </c>
       <c r="BJ1" t="s">
+        <v>280</v>
+      </c>
+      <c r="BK1" t="s">
         <v>281</v>
       </c>
-      <c r="BK1" t="s">
+      <c r="BL1" t="s">
         <v>282</v>
       </c>
-      <c r="BL1" t="s">
+      <c r="BM1" s="1" t="s">
         <v>283</v>
       </c>
-      <c r="BM1" s="1" t="s">
+      <c r="BN1" s="1" t="s">
         <v>284</v>
       </c>
-      <c r="BN1" s="1" t="s">
+      <c r="BO1" s="1" t="s">
         <v>285</v>
       </c>
-      <c r="BO1" s="1" t="s">
+      <c r="BP1" s="1" t="s">
         <v>286</v>
       </c>
-      <c r="BP1" s="1" t="s">
+      <c r="BQ1" s="1" t="s">
         <v>287</v>
       </c>
-      <c r="BQ1" s="1" t="s">
+      <c r="BR1" s="1" t="s">
         <v>288</v>
-      </c>
-      <c r="BR1" s="1" t="s">
-        <v>289</v>
       </c>
       <c r="BS1" t="s">
         <v>227</v>
@@ -2339,196 +2339,196 @@
         <v>229</v>
       </c>
       <c r="BV1" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="BW1" t="s">
         <v>230</v>
       </c>
       <c r="BX1" t="s">
+        <v>294</v>
+      </c>
+      <c r="BY1" t="s">
+        <v>391</v>
+      </c>
+      <c r="BZ1" t="s">
+        <v>290</v>
+      </c>
+      <c r="CA1" s="1" t="s">
+        <v>231</v>
+      </c>
+      <c r="CB1" s="1" t="s">
         <v>295</v>
       </c>
-      <c r="BY1" t="s">
-        <v>231</v>
-      </c>
-      <c r="BZ1" t="s">
+      <c r="CC1" s="1" t="s">
+        <v>232</v>
+      </c>
+      <c r="CD1" t="s">
+        <v>233</v>
+      </c>
+      <c r="CE1" t="s">
+        <v>234</v>
+      </c>
+      <c r="CF1" t="s">
+        <v>235</v>
+      </c>
+      <c r="CG1" t="s">
+        <v>236</v>
+      </c>
+      <c r="CH1" t="s">
+        <v>237</v>
+      </c>
+      <c r="CI1" t="s">
+        <v>238</v>
+      </c>
+      <c r="CJ1" t="s">
+        <v>239</v>
+      </c>
+      <c r="CK1" t="s">
+        <v>240</v>
+      </c>
+      <c r="CL1" t="s">
+        <v>241</v>
+      </c>
+      <c r="CM1" t="s">
+        <v>242</v>
+      </c>
+      <c r="CN1" t="s">
+        <v>243</v>
+      </c>
+      <c r="CO1" t="s">
+        <v>244</v>
+      </c>
+      <c r="CP1" t="s">
+        <v>245</v>
+      </c>
+      <c r="CQ1" t="s">
+        <v>246</v>
+      </c>
+      <c r="CR1" t="s">
+        <v>247</v>
+      </c>
+      <c r="CS1" t="s">
+        <v>248</v>
+      </c>
+      <c r="CT1" t="s">
+        <v>249</v>
+      </c>
+      <c r="CU1" t="s">
+        <v>250</v>
+      </c>
+      <c r="CV1" t="s">
         <v>291</v>
       </c>
-      <c r="CA1" s="1" t="s">
-        <v>232</v>
-      </c>
-      <c r="CB1" s="1" t="s">
+      <c r="CW1" t="s">
+        <v>251</v>
+      </c>
+      <c r="CX1" t="s">
+        <v>252</v>
+      </c>
+      <c r="CY1" t="s">
+        <v>253</v>
+      </c>
+      <c r="CZ1" t="s">
+        <v>254</v>
+      </c>
+      <c r="DA1" t="s">
+        <v>255</v>
+      </c>
+      <c r="DB1" t="s">
+        <v>256</v>
+      </c>
+      <c r="DC1" t="s">
+        <v>257</v>
+      </c>
+      <c r="DD1" t="s">
+        <v>292</v>
+      </c>
+      <c r="DE1" t="s">
+        <v>258</v>
+      </c>
+      <c r="DF1" t="s">
+        <v>259</v>
+      </c>
+      <c r="DG1" t="s">
+        <v>260</v>
+      </c>
+      <c r="DH1" t="s">
+        <v>261</v>
+      </c>
+      <c r="DI1" t="s">
+        <v>262</v>
+      </c>
+      <c r="DJ1" t="s">
+        <v>263</v>
+      </c>
+      <c r="DK1" t="s">
+        <v>264</v>
+      </c>
+      <c r="DL1" t="s">
+        <v>265</v>
+      </c>
+      <c r="DM1" t="s">
         <v>296</v>
       </c>
-      <c r="CC1" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="CD1" t="s">
-        <v>234</v>
-      </c>
-      <c r="CE1" t="s">
-        <v>235</v>
-      </c>
-      <c r="CF1" t="s">
-        <v>236</v>
-      </c>
-      <c r="CG1" t="s">
-        <v>237</v>
-      </c>
-      <c r="CH1" t="s">
-        <v>238</v>
-      </c>
-      <c r="CI1" t="s">
-        <v>239</v>
-      </c>
-      <c r="CJ1" t="s">
-        <v>240</v>
-      </c>
-      <c r="CK1" t="s">
-        <v>241</v>
-      </c>
-      <c r="CL1" t="s">
-        <v>242</v>
-      </c>
-      <c r="CM1" t="s">
-        <v>243</v>
-      </c>
-      <c r="CN1" t="s">
-        <v>244</v>
-      </c>
-      <c r="CO1" t="s">
-        <v>245</v>
-      </c>
-      <c r="CP1" t="s">
-        <v>246</v>
-      </c>
-      <c r="CQ1" t="s">
-        <v>247</v>
-      </c>
-      <c r="CR1" t="s">
-        <v>248</v>
-      </c>
-      <c r="CS1" t="s">
-        <v>249</v>
-      </c>
-      <c r="CT1" t="s">
-        <v>250</v>
-      </c>
-      <c r="CU1" t="s">
-        <v>251</v>
-      </c>
-      <c r="CV1" t="s">
-        <v>292</v>
-      </c>
-      <c r="CW1" t="s">
-        <v>252</v>
-      </c>
-      <c r="CX1" t="s">
-        <v>253</v>
-      </c>
-      <c r="CY1" t="s">
-        <v>254</v>
-      </c>
-      <c r="CZ1" t="s">
-        <v>255</v>
-      </c>
-      <c r="DA1" t="s">
-        <v>256</v>
-      </c>
-      <c r="DB1" t="s">
-        <v>257</v>
-      </c>
-      <c r="DC1" t="s">
-        <v>258</v>
-      </c>
-      <c r="DD1" t="s">
-        <v>293</v>
-      </c>
-      <c r="DE1" t="s">
-        <v>259</v>
-      </c>
-      <c r="DF1" t="s">
-        <v>260</v>
-      </c>
-      <c r="DG1" t="s">
-        <v>261</v>
-      </c>
-      <c r="DH1" t="s">
-        <v>262</v>
-      </c>
-      <c r="DI1" t="s">
-        <v>263</v>
-      </c>
-      <c r="DJ1" t="s">
-        <v>264</v>
-      </c>
-      <c r="DK1" t="s">
-        <v>265</v>
-      </c>
-      <c r="DL1" t="s">
+      <c r="DN1" t="s">
+        <v>298</v>
+      </c>
+      <c r="DO1" t="s">
+        <v>297</v>
+      </c>
+      <c r="DP1" t="s">
         <v>266</v>
       </c>
-      <c r="DM1" t="s">
-        <v>297</v>
-      </c>
-      <c r="DN1" t="s">
+      <c r="DQ1" t="s">
+        <v>267</v>
+      </c>
+      <c r="DR1" t="s">
+        <v>268</v>
+      </c>
+      <c r="DS1" t="s">
+        <v>269</v>
+      </c>
+      <c r="DT1" t="s">
+        <v>270</v>
+      </c>
+      <c r="DU1" t="s">
+        <v>271</v>
+      </c>
+      <c r="DV1" t="s">
+        <v>272</v>
+      </c>
+      <c r="DW1" t="s">
+        <v>273</v>
+      </c>
+      <c r="DX1" t="s">
+        <v>274</v>
+      </c>
+      <c r="DY1" t="s">
+        <v>275</v>
+      </c>
+      <c r="DZ1" t="s">
         <v>299</v>
       </c>
-      <c r="DO1" t="s">
-        <v>298</v>
-      </c>
-      <c r="DP1" t="s">
-        <v>267</v>
-      </c>
-      <c r="DQ1" t="s">
-        <v>268</v>
-      </c>
-      <c r="DR1" t="s">
-        <v>269</v>
-      </c>
-      <c r="DS1" t="s">
-        <v>270</v>
-      </c>
-      <c r="DT1" t="s">
-        <v>271</v>
-      </c>
-      <c r="DU1" t="s">
-        <v>272</v>
-      </c>
-      <c r="DV1" t="s">
-        <v>273</v>
-      </c>
-      <c r="DW1" t="s">
-        <v>274</v>
-      </c>
-      <c r="DX1" t="s">
-        <v>275</v>
-      </c>
-      <c r="DY1" t="s">
+      <c r="EA1" t="s">
         <v>276</v>
       </c>
-      <c r="DZ1" t="s">
+      <c r="EB1" t="s">
         <v>300</v>
       </c>
-      <c r="EA1" t="s">
+      <c r="EC1" t="s">
         <v>277</v>
       </c>
-      <c r="EB1" t="s">
+      <c r="ED1" t="s">
+        <v>278</v>
+      </c>
+      <c r="EE1" t="s">
+        <v>279</v>
+      </c>
+      <c r="EF1" t="s">
+        <v>302</v>
+      </c>
+      <c r="EG1" t="s">
         <v>301</v>
-      </c>
-      <c r="EC1" t="s">
-        <v>278</v>
-      </c>
-      <c r="ED1" t="s">
-        <v>279</v>
-      </c>
-      <c r="EE1" t="s">
-        <v>280</v>
-      </c>
-      <c r="EF1" t="s">
-        <v>303</v>
-      </c>
-      <c r="EG1" t="s">
-        <v>302</v>
       </c>
     </row>
     <row r="2" spans="1:137" x14ac:dyDescent="0.2">
@@ -2937,13 +2937,13 @@
         <v>1</v>
       </c>
       <c r="C3" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D3" t="s">
         <v>218</v>
       </c>
       <c r="E3" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F3" t="s">
         <v>215</v>
@@ -3350,13 +3350,13 @@
         <v>1</v>
       </c>
       <c r="C4" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D4" t="s">
         <v>218</v>
       </c>
       <c r="E4" t="s">
-        <v>309</v>
+        <v>308</v>
       </c>
       <c r="F4" t="s">
         <v>216</v>
@@ -3763,7 +3763,7 @@
         <v>1</v>
       </c>
       <c r="C5" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D5" t="s">
         <v>218</v>
@@ -4170,7 +4170,7 @@
         <v>1</v>
       </c>
       <c r="C6" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D6" t="s">
         <v>218</v>
@@ -4577,13 +4577,13 @@
         <v>1</v>
       </c>
       <c r="C7" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D7" t="s">
         <v>218</v>
       </c>
       <c r="E7" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F7" t="s">
         <v>219</v>
@@ -4990,16 +4990,16 @@
         <v>1</v>
       </c>
       <c r="C8" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D8" t="s">
         <v>218</v>
       </c>
       <c r="E8" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F8" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G8">
         <v>31</v>
@@ -5403,7 +5403,7 @@
         <v>1</v>
       </c>
       <c r="C9" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D9" t="s">
         <v>218</v>
@@ -5412,7 +5412,7 @@
         <v>8</v>
       </c>
       <c r="F9" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G9">
         <v>72</v>
@@ -5816,13 +5816,13 @@
         <v>1</v>
       </c>
       <c r="C10" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D10" t="s">
         <v>218</v>
       </c>
       <c r="E10" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F10" t="s">
         <v>215</v>
@@ -6223,7 +6223,7 @@
         <v>1</v>
       </c>
       <c r="C11" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D11" t="s">
         <v>218</v>
@@ -6232,7 +6232,7 @@
         <v>10</v>
       </c>
       <c r="F11" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G11">
         <v>334</v>
@@ -6636,7 +6636,7 @@
         <v>1</v>
       </c>
       <c r="C12" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D12" t="s">
         <v>218</v>
@@ -7043,16 +7043,16 @@
         <v>1</v>
       </c>
       <c r="C13" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D13" t="s">
         <v>218</v>
       </c>
       <c r="E13" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F13" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G13">
         <v>367</v>
@@ -7456,10 +7456,10 @@
         <v>1</v>
       </c>
       <c r="C14" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D14" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E14" t="s">
         <v>218</v>
@@ -7863,7 +7863,7 @@
         <v>1</v>
       </c>
       <c r="C15" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D15" t="s">
         <v>218</v>
@@ -8276,7 +8276,7 @@
         <v>1</v>
       </c>
       <c r="C16" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D16" t="s">
         <v>218</v>
@@ -8689,16 +8689,16 @@
         <v>1</v>
       </c>
       <c r="C17" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D17" t="s">
         <v>218</v>
       </c>
       <c r="E17" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F17" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G17">
         <v>268</v>
@@ -9102,7 +9102,7 @@
         <v>1</v>
       </c>
       <c r="C18" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D18" t="s">
         <v>218</v>
@@ -9509,7 +9509,7 @@
         <v>1</v>
       </c>
       <c r="C19" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D19" t="s">
         <v>218</v>
@@ -9922,16 +9922,16 @@
         <v>1</v>
       </c>
       <c r="C20" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D20" t="s">
         <v>218</v>
       </c>
       <c r="E20" t="s">
-        <v>314</v>
+        <v>313</v>
       </c>
       <c r="F20" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G20">
         <v>78</v>
@@ -10335,13 +10335,13 @@
         <v>1</v>
       </c>
       <c r="C21" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D21" t="s">
         <v>218</v>
       </c>
       <c r="E21" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F21" t="s">
         <v>215</v>
@@ -10748,7 +10748,7 @@
         <v>1</v>
       </c>
       <c r="C22" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D22" t="s">
         <v>218</v>
@@ -10757,7 +10757,7 @@
         <v>21</v>
       </c>
       <c r="F22" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G22">
         <v>132</v>
@@ -11161,13 +11161,13 @@
         <v>1</v>
       </c>
       <c r="C23" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D23" t="s">
         <v>218</v>
       </c>
       <c r="E23" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F23" t="s">
         <v>219</v>
@@ -11568,10 +11568,10 @@
         <v>1</v>
       </c>
       <c r="C24" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D24" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E24" t="s">
         <v>218</v>
@@ -11975,7 +11975,7 @@
         <v>1</v>
       </c>
       <c r="C25" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D25" t="s">
         <v>218</v>
@@ -12382,13 +12382,13 @@
         <v>1</v>
       </c>
       <c r="C26" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D26" t="s">
         <v>218</v>
       </c>
       <c r="E26" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F26" t="s">
         <v>222</v>
@@ -12789,16 +12789,16 @@
         <v>1</v>
       </c>
       <c r="C27" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D27" t="s">
         <v>218</v>
       </c>
       <c r="E27" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F27" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G27">
         <v>340</v>
@@ -13202,7 +13202,7 @@
         <v>1</v>
       </c>
       <c r="C28" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D28" t="s">
         <v>218</v>
@@ -13609,13 +13609,13 @@
         <v>1</v>
       </c>
       <c r="C29" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D29" t="s">
         <v>218</v>
       </c>
       <c r="E29" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F29" t="s">
         <v>215</v>
@@ -14022,10 +14022,10 @@
         <v>1</v>
       </c>
       <c r="C30" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D30" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E30" t="s">
         <v>218</v>
@@ -14432,7 +14432,7 @@
         <v>1</v>
       </c>
       <c r="C31" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D31" t="s">
         <v>218</v>
@@ -14845,7 +14845,7 @@
         <v>1</v>
       </c>
       <c r="C32" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D32" t="s">
         <v>218</v>
@@ -15258,7 +15258,7 @@
         <v>1</v>
       </c>
       <c r="C33" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D33" t="s">
         <v>218</v>
@@ -15665,7 +15665,7 @@
         <v>1</v>
       </c>
       <c r="C34" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D34" t="s">
         <v>218</v>
@@ -16078,7 +16078,7 @@
         <v>1</v>
       </c>
       <c r="C35" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D35" t="s">
         <v>218</v>
@@ -16491,16 +16491,16 @@
         <v>1</v>
       </c>
       <c r="C36" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D36" t="s">
         <v>218</v>
       </c>
       <c r="E36" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F36" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G36">
         <v>110</v>
@@ -16904,7 +16904,7 @@
         <v>1</v>
       </c>
       <c r="C37" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D37" t="s">
         <v>218</v>
@@ -17317,7 +17317,7 @@
         <v>1</v>
       </c>
       <c r="C38" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D38" t="s">
         <v>218</v>
@@ -17724,13 +17724,13 @@
         <v>1</v>
       </c>
       <c r="C39" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D39" t="s">
         <v>218</v>
       </c>
       <c r="E39" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F39" t="s">
         <v>222</v>
@@ -18137,13 +18137,13 @@
         <v>1</v>
       </c>
       <c r="C40" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D40" t="s">
         <v>218</v>
       </c>
       <c r="E40" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F40" t="s">
         <v>219</v>
@@ -18550,7 +18550,7 @@
         <v>1</v>
       </c>
       <c r="C41" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D41" t="s">
         <v>218</v>
@@ -18559,7 +18559,7 @@
         <v>176</v>
       </c>
       <c r="F41" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G41">
         <v>153</v>
@@ -18963,7 +18963,7 @@
         <v>1</v>
       </c>
       <c r="C42" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D42" t="s">
         <v>218</v>
@@ -19367,16 +19367,16 @@
         <v>1</v>
       </c>
       <c r="C43" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D43" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E43" t="s">
         <v>218</v>
       </c>
       <c r="F43" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G43">
         <v>116</v>
@@ -19780,7 +19780,7 @@
         <v>1</v>
       </c>
       <c r="C44" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D44" t="s">
         <v>218</v>
@@ -20193,13 +20193,13 @@
         <v>1</v>
       </c>
       <c r="C45" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D45" t="s">
         <v>218</v>
       </c>
       <c r="E45" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F45" t="s">
         <v>222</v>
@@ -20606,7 +20606,7 @@
         <v>1</v>
       </c>
       <c r="C46" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D46" t="s">
         <v>218</v>
@@ -21019,7 +21019,7 @@
         <v>1</v>
       </c>
       <c r="C47" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D47" t="s">
         <v>218</v>
@@ -21426,7 +21426,7 @@
         <v>1</v>
       </c>
       <c r="C48" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D48" t="s">
         <v>218</v>
@@ -21839,7 +21839,7 @@
         <v>1</v>
       </c>
       <c r="C49" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D49" t="s">
         <v>218</v>
@@ -22252,13 +22252,13 @@
         <v>1</v>
       </c>
       <c r="C50" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D50" t="s">
         <v>218</v>
       </c>
       <c r="E50" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F50" t="s">
         <v>219</v>
@@ -22665,7 +22665,7 @@
         <v>1</v>
       </c>
       <c r="C51" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D51" t="s">
         <v>218</v>
@@ -23072,7 +23072,7 @@
         <v>1</v>
       </c>
       <c r="C52" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D52" t="s">
         <v>218</v>
@@ -23479,10 +23479,10 @@
         <v>1</v>
       </c>
       <c r="C53" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D53" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E53" t="s">
         <v>218</v>
@@ -23886,13 +23886,13 @@
         <v>1</v>
       </c>
       <c r="C54" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D54" t="s">
         <v>218</v>
       </c>
       <c r="E54" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F54" t="s">
         <v>215</v>
@@ -24299,7 +24299,7 @@
         <v>1</v>
       </c>
       <c r="C55" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D55" t="s">
         <v>218</v>
@@ -24308,7 +24308,7 @@
         <v>54</v>
       </c>
       <c r="F55" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G55">
         <v>293</v>
@@ -24712,7 +24712,7 @@
         <v>1</v>
       </c>
       <c r="C56" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D56" t="s">
         <v>218</v>
@@ -25125,13 +25125,13 @@
         <v>1</v>
       </c>
       <c r="C57" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D57" t="s">
         <v>218</v>
       </c>
       <c r="E57" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F57" t="s">
         <v>215</v>
@@ -25538,7 +25538,7 @@
         <v>1</v>
       </c>
       <c r="C58" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D58" t="s">
         <v>218</v>
@@ -25951,13 +25951,13 @@
         <v>1</v>
       </c>
       <c r="C59" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D59" t="s">
         <v>218</v>
       </c>
       <c r="E59" t="s">
-        <v>320</v>
+        <v>319</v>
       </c>
       <c r="F59" t="s">
         <v>216</v>
@@ -26364,16 +26364,16 @@
         <v>1</v>
       </c>
       <c r="C60" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D60" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E60" t="s">
         <v>218</v>
       </c>
       <c r="F60" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G60">
         <v>76</v>
@@ -26777,16 +26777,16 @@
         <v>1</v>
       </c>
       <c r="C61" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D61" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E61" t="s">
         <v>218</v>
       </c>
       <c r="F61" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G61">
         <v>69</v>
@@ -27190,7 +27190,7 @@
         <v>1</v>
       </c>
       <c r="C62" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D62" t="s">
         <v>218</v>
@@ -27597,7 +27597,7 @@
         <v>1</v>
       </c>
       <c r="C63" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D63" t="s">
         <v>218</v>
@@ -28010,16 +28010,16 @@
         <v>1</v>
       </c>
       <c r="C64" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D64" t="s">
         <v>218</v>
       </c>
       <c r="E64" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F64" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G64">
         <v>147</v>
@@ -28423,7 +28423,7 @@
         <v>1</v>
       </c>
       <c r="C65" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D65" t="s">
         <v>218</v>
@@ -28830,16 +28830,16 @@
         <v>1</v>
       </c>
       <c r="C66" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D66" t="s">
         <v>218</v>
       </c>
       <c r="E66" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F66" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G66">
         <v>193</v>
@@ -29243,7 +29243,7 @@
         <v>1</v>
       </c>
       <c r="C67" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D67" t="s">
         <v>218</v>
@@ -29650,16 +29650,16 @@
         <v>1</v>
       </c>
       <c r="C68" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D68" t="s">
         <v>218</v>
       </c>
       <c r="E68" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F68" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G68">
         <v>556</v>
@@ -30063,13 +30063,13 @@
         <v>1</v>
       </c>
       <c r="C69" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D69" t="s">
         <v>218</v>
       </c>
       <c r="E69" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F69" t="s">
         <v>215</v>
@@ -30476,7 +30476,7 @@
         <v>1</v>
       </c>
       <c r="C70" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D70" t="s">
         <v>218</v>
@@ -30889,13 +30889,13 @@
         <v>1</v>
       </c>
       <c r="C71" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D71" t="s">
         <v>218</v>
       </c>
       <c r="E71" t="s">
-        <v>322</v>
+        <v>321</v>
       </c>
       <c r="F71" t="s">
         <v>216</v>
@@ -31302,16 +31302,16 @@
         <v>1</v>
       </c>
       <c r="C72" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D72" t="s">
         <v>218</v>
       </c>
       <c r="E72" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F72" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G72">
         <v>58</v>
@@ -31709,16 +31709,16 @@
         <v>1</v>
       </c>
       <c r="C73" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D73" t="s">
         <v>218</v>
       </c>
       <c r="E73" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F73" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G73">
         <v>56</v>
@@ -32122,7 +32122,7 @@
         <v>1</v>
       </c>
       <c r="C74" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D74" t="s">
         <v>218</v>
@@ -32535,7 +32535,7 @@
         <v>1</v>
       </c>
       <c r="C75" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D75" t="s">
         <v>218</v>
@@ -32544,7 +32544,7 @@
         <v>74</v>
       </c>
       <c r="F75" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G75">
         <v>151</v>
@@ -32948,7 +32948,7 @@
         <v>1</v>
       </c>
       <c r="C76" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D76" t="s">
         <v>218</v>
@@ -32957,7 +32957,7 @@
         <v>75</v>
       </c>
       <c r="F76" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G76">
         <v>256</v>
@@ -33361,7 +33361,7 @@
         <v>1</v>
       </c>
       <c r="C77" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D77" t="s">
         <v>218</v>
@@ -33774,16 +33774,16 @@
         <v>1</v>
       </c>
       <c r="C78" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D78" t="s">
         <v>218</v>
       </c>
       <c r="E78" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F78" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G78">
         <v>287</v>
@@ -34187,13 +34187,13 @@
         <v>1</v>
       </c>
       <c r="C79" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D79" t="s">
         <v>218</v>
       </c>
       <c r="E79" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F79" t="s">
         <v>219</v>
@@ -34600,7 +34600,7 @@
         <v>1</v>
       </c>
       <c r="C80" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D80" t="s">
         <v>218</v>
@@ -35013,7 +35013,7 @@
         <v>1</v>
       </c>
       <c r="C81" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D81" t="s">
         <v>218</v>
@@ -35426,13 +35426,13 @@
         <v>1</v>
       </c>
       <c r="C82" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D82" t="s">
         <v>218</v>
       </c>
       <c r="E82" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F82" t="s">
         <v>219</v>
@@ -35839,7 +35839,7 @@
         <v>1</v>
       </c>
       <c r="C83" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D83" t="s">
         <v>218</v>
@@ -36252,10 +36252,10 @@
         <v>1</v>
       </c>
       <c r="C84" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D84" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E84" t="s">
         <v>218</v>
@@ -36665,7 +36665,7 @@
         <v>1</v>
       </c>
       <c r="C85" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D85" t="s">
         <v>218</v>
@@ -37078,13 +37078,13 @@
         <v>1</v>
       </c>
       <c r="C86" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D86" t="s">
         <v>218</v>
       </c>
       <c r="E86" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F86" t="s">
         <v>222</v>
@@ -37491,7 +37491,7 @@
         <v>1</v>
       </c>
       <c r="C87" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D87" t="s">
         <v>218</v>
@@ -37904,7 +37904,7 @@
         <v>1</v>
       </c>
       <c r="C88" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D88" t="s">
         <v>218</v>
@@ -38317,7 +38317,7 @@
         <v>1</v>
       </c>
       <c r="C89" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D89" t="s">
         <v>218</v>
@@ -38730,13 +38730,13 @@
         <v>1</v>
       </c>
       <c r="C90" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D90" t="s">
         <v>218</v>
       </c>
       <c r="E90" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F90" t="s">
         <v>215</v>
@@ -39143,16 +39143,16 @@
         <v>1</v>
       </c>
       <c r="C91" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D91" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E91" t="s">
         <v>218</v>
       </c>
       <c r="F91" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G91">
         <v>135</v>
@@ -39556,13 +39556,13 @@
         <v>1</v>
       </c>
       <c r="C92" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D92" t="s">
         <v>218</v>
       </c>
       <c r="E92" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F92" t="s">
         <v>219</v>
@@ -39963,13 +39963,13 @@
         <v>1</v>
       </c>
       <c r="C93" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D93" t="s">
         <v>218</v>
       </c>
       <c r="E93" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F93" t="s">
         <v>222</v>
@@ -40370,7 +40370,7 @@
         <v>1</v>
       </c>
       <c r="C94" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D94" t="s">
         <v>218</v>
@@ -40783,10 +40783,10 @@
         <v>1</v>
       </c>
       <c r="C95" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D95" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E95" t="s">
         <v>218</v>
@@ -41190,13 +41190,13 @@
         <v>1</v>
       </c>
       <c r="C96" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D96" t="s">
         <v>218</v>
       </c>
       <c r="E96" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F96" t="s">
         <v>219</v>
@@ -41603,13 +41603,13 @@
         <v>1</v>
       </c>
       <c r="C97" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D97" t="s">
         <v>218</v>
       </c>
       <c r="E97" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F97" t="s">
         <v>219</v>
@@ -42016,7 +42016,7 @@
         <v>1</v>
       </c>
       <c r="C98" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D98" t="s">
         <v>218</v>
@@ -42423,7 +42423,7 @@
         <v>1</v>
       </c>
       <c r="C99" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D99" t="s">
         <v>218</v>
@@ -42836,7 +42836,7 @@
         <v>1</v>
       </c>
       <c r="C100" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D100" t="s">
         <v>218</v>
@@ -43249,16 +43249,16 @@
         <v>1</v>
       </c>
       <c r="C101" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D101" t="s">
         <v>218</v>
       </c>
       <c r="E101" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F101" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G101">
         <v>109</v>
@@ -43662,13 +43662,13 @@
         <v>1</v>
       </c>
       <c r="C102" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D102" t="s">
         <v>218</v>
       </c>
       <c r="E102" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F102" t="s">
         <v>222</v>
@@ -44075,13 +44075,13 @@
         <v>1</v>
       </c>
       <c r="C103" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D103" t="s">
         <v>218</v>
       </c>
       <c r="E103" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F103" t="s">
         <v>219</v>
@@ -44488,13 +44488,13 @@
         <v>1</v>
       </c>
       <c r="C104" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D104" t="s">
         <v>218</v>
       </c>
       <c r="E104" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F104" t="s">
         <v>215</v>
@@ -44895,16 +44895,16 @@
         <v>1</v>
       </c>
       <c r="C105" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D105" t="s">
         <v>218</v>
       </c>
       <c r="E105" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F105" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G105">
         <v>31</v>
@@ -45302,16 +45302,16 @@
         <v>1</v>
       </c>
       <c r="C106" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D106" t="s">
         <v>218</v>
       </c>
       <c r="E106" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F106" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G106">
         <v>48</v>
@@ -45709,13 +45709,13 @@
         <v>1</v>
       </c>
       <c r="C107" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D107" t="s">
         <v>218</v>
       </c>
       <c r="E107" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F107" t="s">
         <v>222</v>
@@ -46116,16 +46116,16 @@
         <v>1</v>
       </c>
       <c r="C108" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D108" t="s">
         <v>218</v>
       </c>
       <c r="E108" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F108" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G108">
         <v>73</v>
@@ -46523,7 +46523,7 @@
         <v>1</v>
       </c>
       <c r="C109" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D109" t="s">
         <v>218</v>
@@ -46930,7 +46930,7 @@
         <v>1</v>
       </c>
       <c r="C110" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D110" t="s">
         <v>218</v>
@@ -47343,13 +47343,13 @@
         <v>1</v>
       </c>
       <c r="C111" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D111" t="s">
         <v>218</v>
       </c>
       <c r="E111" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F111" t="s">
         <v>222</v>
@@ -47756,7 +47756,7 @@
         <v>1</v>
       </c>
       <c r="C112" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D112" t="s">
         <v>218</v>
@@ -48169,13 +48169,13 @@
         <v>1</v>
       </c>
       <c r="C113" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D113" t="s">
         <v>218</v>
       </c>
       <c r="E113" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F113" t="s">
         <v>222</v>
@@ -48582,7 +48582,7 @@
         <v>1</v>
       </c>
       <c r="C114" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D114" t="s">
         <v>218</v>
@@ -48591,7 +48591,7 @@
         <v>218</v>
       </c>
       <c r="F114" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G114">
         <v>28</v>
@@ -48989,13 +48989,13 @@
         <v>1</v>
       </c>
       <c r="C115" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D115" t="s">
         <v>218</v>
       </c>
       <c r="E115" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F115" t="s">
         <v>222</v>
@@ -49402,13 +49402,13 @@
         <v>1</v>
       </c>
       <c r="C116" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D116" t="s">
         <v>218</v>
       </c>
       <c r="E116" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F116" t="s">
         <v>215</v>
@@ -49815,16 +49815,16 @@
         <v>1</v>
       </c>
       <c r="C117" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D117" t="s">
         <v>218</v>
       </c>
       <c r="E117" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F117" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G117">
         <v>236</v>
@@ -50228,7 +50228,7 @@
         <v>1</v>
       </c>
       <c r="C118" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D118" t="s">
         <v>218</v>
@@ -50635,13 +50635,13 @@
         <v>1</v>
       </c>
       <c r="C119" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D119" t="s">
         <v>218</v>
       </c>
       <c r="E119" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F119" t="s">
         <v>219</v>
@@ -51048,10 +51048,10 @@
         <v>1</v>
       </c>
       <c r="C120" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D120" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E120" t="s">
         <v>218</v>
@@ -51461,16 +51461,16 @@
         <v>1</v>
       </c>
       <c r="C121" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D121" t="s">
         <v>218</v>
       </c>
       <c r="E121" t="s">
-        <v>321</v>
+        <v>320</v>
       </c>
       <c r="F121" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G121">
         <v>36</v>
@@ -51874,13 +51874,13 @@
         <v>1</v>
       </c>
       <c r="C122" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D122" t="s">
         <v>218</v>
       </c>
       <c r="E122" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F122" t="s">
         <v>219</v>
@@ -52287,13 +52287,13 @@
         <v>1</v>
       </c>
       <c r="C123" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D123" t="s">
         <v>218</v>
       </c>
       <c r="E123" t="s">
-        <v>324</v>
+        <v>323</v>
       </c>
       <c r="F123" t="s">
         <v>216</v>
@@ -52700,13 +52700,13 @@
         <v>1</v>
       </c>
       <c r="C124" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D124" t="s">
         <v>218</v>
       </c>
       <c r="E124" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F124" t="s">
         <v>215</v>
@@ -53113,7 +53113,7 @@
         <v>1</v>
       </c>
       <c r="C125" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D125" t="s">
         <v>218</v>
@@ -53526,10 +53526,10 @@
         <v>1</v>
       </c>
       <c r="C126" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D126" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E126" t="s">
         <v>218</v>
@@ -53939,13 +53939,13 @@
         <v>1</v>
       </c>
       <c r="C127" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D127" t="s">
         <v>218</v>
       </c>
       <c r="E127" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F127" t="s">
         <v>222</v>
@@ -54346,13 +54346,13 @@
         <v>1</v>
       </c>
       <c r="C128" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D128" t="s">
         <v>218</v>
       </c>
       <c r="E128" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F128" t="s">
         <v>219</v>
@@ -54753,10 +54753,10 @@
         <v>1</v>
       </c>
       <c r="C129" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D129" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E129" t="s">
         <v>218</v>
@@ -55166,13 +55166,13 @@
         <v>1</v>
       </c>
       <c r="C130" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D130" t="s">
         <v>218</v>
       </c>
       <c r="E130" t="s">
-        <v>312</v>
+        <v>311</v>
       </c>
       <c r="F130" t="s">
         <v>215</v>
@@ -55579,10 +55579,10 @@
         <v>1</v>
       </c>
       <c r="C131" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D131" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E131" t="s">
         <v>218</v>
@@ -55992,16 +55992,16 @@
         <v>1</v>
       </c>
       <c r="C132" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D132" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E132" t="s">
         <v>218</v>
       </c>
       <c r="F132" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G132">
         <v>87</v>
@@ -56399,13 +56399,13 @@
         <v>1</v>
       </c>
       <c r="C133" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D133" t="s">
         <v>218</v>
       </c>
       <c r="E133" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F133" t="s">
         <v>222</v>
@@ -56806,7 +56806,7 @@
         <v>1</v>
       </c>
       <c r="C134" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D134" t="s">
         <v>218</v>
@@ -57219,7 +57219,7 @@
         <v>1</v>
       </c>
       <c r="C135" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D135" t="s">
         <v>218</v>
@@ -57632,13 +57632,13 @@
         <v>1</v>
       </c>
       <c r="C136" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D136" t="s">
         <v>218</v>
       </c>
       <c r="E136" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F136" t="s">
         <v>219</v>
@@ -58039,16 +58039,16 @@
         <v>1</v>
       </c>
       <c r="C137" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D137" t="s">
         <v>218</v>
       </c>
       <c r="E137" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F137" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G137">
         <v>52</v>
@@ -58446,7 +58446,7 @@
         <v>1</v>
       </c>
       <c r="C138" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D138" t="s">
         <v>218</v>
@@ -58859,13 +58859,13 @@
         <v>1</v>
       </c>
       <c r="C139" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D139" t="s">
         <v>218</v>
       </c>
       <c r="E139" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F139" t="s">
         <v>222</v>
@@ -59272,7 +59272,7 @@
         <v>1</v>
       </c>
       <c r="C140" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D140" t="s">
         <v>218</v>
@@ -59281,7 +59281,7 @@
         <v>139</v>
       </c>
       <c r="F140" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G140">
         <v>119</v>
@@ -59685,13 +59685,13 @@
         <v>1</v>
       </c>
       <c r="C141" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D141" t="s">
         <v>218</v>
       </c>
       <c r="E141" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F141" t="s">
         <v>222</v>
@@ -60098,7 +60098,7 @@
         <v>1</v>
       </c>
       <c r="C142" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D142" t="s">
         <v>218</v>
@@ -60511,13 +60511,13 @@
         <v>1</v>
       </c>
       <c r="C143" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D143" t="s">
         <v>218</v>
       </c>
       <c r="E143" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F143" t="s">
         <v>222</v>
@@ -60924,13 +60924,13 @@
         <v>1</v>
       </c>
       <c r="C144" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D144" t="s">
         <v>218</v>
       </c>
       <c r="E144" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F144" t="s">
         <v>215</v>
@@ -61337,16 +61337,16 @@
         <v>1</v>
       </c>
       <c r="C145" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D145" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E145" t="s">
         <v>218</v>
       </c>
       <c r="F145" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G145">
         <v>154</v>
@@ -61750,13 +61750,13 @@
         <v>1</v>
       </c>
       <c r="C146" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D146" t="s">
         <v>218</v>
       </c>
       <c r="E146" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F146" t="s">
         <v>222</v>
@@ -62163,7 +62163,7 @@
         <v>1</v>
       </c>
       <c r="C147" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D147" t="s">
         <v>218</v>
@@ -62576,7 +62576,7 @@
         <v>1</v>
       </c>
       <c r="C148" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D148" t="s">
         <v>218</v>
@@ -62989,7 +62989,7 @@
         <v>1</v>
       </c>
       <c r="C149" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D149" t="s">
         <v>218</v>
@@ -63402,13 +63402,13 @@
         <v>1</v>
       </c>
       <c r="C150" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D150" t="s">
         <v>218</v>
       </c>
       <c r="E150" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F150" t="s">
         <v>219</v>
@@ -63815,13 +63815,13 @@
         <v>1</v>
       </c>
       <c r="C151" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D151" t="s">
         <v>218</v>
       </c>
       <c r="E151" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F151" t="s">
         <v>219</v>
@@ -64222,16 +64222,16 @@
         <v>1</v>
       </c>
       <c r="C152" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D152" t="s">
         <v>218</v>
       </c>
       <c r="E152" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="F152" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G152">
         <v>147</v>
@@ -64635,16 +64635,16 @@
         <v>1</v>
       </c>
       <c r="C153" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D153" t="s">
         <v>218</v>
       </c>
       <c r="E153" t="s">
-        <v>311</v>
+        <v>310</v>
       </c>
       <c r="F153" t="s">
-        <v>304</v>
+        <v>303</v>
       </c>
       <c r="G153">
         <v>272</v>
@@ -65048,13 +65048,13 @@
         <v>1</v>
       </c>
       <c r="C154" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D154" t="s">
         <v>218</v>
       </c>
       <c r="E154" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
       <c r="F154" t="s">
         <v>215</v>
@@ -65461,13 +65461,13 @@
         <v>1</v>
       </c>
       <c r="C155" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D155" t="s">
         <v>218</v>
       </c>
       <c r="E155" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F155" t="s">
         <v>222</v>
@@ -65874,13 +65874,13 @@
         <v>1</v>
       </c>
       <c r="C156" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D156" t="s">
         <v>218</v>
       </c>
       <c r="E156" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F156" t="s">
         <v>219</v>
@@ -66287,13 +66287,13 @@
         <v>1</v>
       </c>
       <c r="C157" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D157" t="s">
         <v>218</v>
       </c>
       <c r="E157" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F157" t="s">
         <v>219</v>
@@ -66700,16 +66700,16 @@
         <v>1</v>
       </c>
       <c r="C158" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D158" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E158" t="s">
         <v>218</v>
       </c>
       <c r="F158" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G158">
         <v>49</v>
@@ -67107,13 +67107,13 @@
         <v>1</v>
       </c>
       <c r="C159" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D159" t="s">
         <v>218</v>
       </c>
       <c r="E159" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F159" t="s">
         <v>222</v>
@@ -67520,10 +67520,10 @@
         <v>1</v>
       </c>
       <c r="C160" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D160" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E160" t="s">
         <v>218</v>
@@ -67927,13 +67927,13 @@
         <v>1</v>
       </c>
       <c r="C161" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D161" t="s">
         <v>218</v>
       </c>
       <c r="E161" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F161" t="s">
         <v>219</v>
@@ -68340,16 +68340,16 @@
         <v>1</v>
       </c>
       <c r="C162" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D162" t="s">
         <v>218</v>
       </c>
       <c r="E162" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F162" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G162">
         <v>29</v>
@@ -68753,13 +68753,13 @@
         <v>1</v>
       </c>
       <c r="C163" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D163" t="s">
         <v>218</v>
       </c>
       <c r="E163" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F163" t="s">
         <v>219</v>
@@ -69166,13 +69166,13 @@
         <v>1</v>
       </c>
       <c r="C164" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D164" t="s">
         <v>218</v>
       </c>
       <c r="E164" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F164" t="s">
         <v>219</v>
@@ -69573,7 +69573,7 @@
         <v>1</v>
       </c>
       <c r="C165" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D165" t="s">
         <v>218</v>
@@ -69980,7 +69980,7 @@
         <v>1</v>
       </c>
       <c r="C166" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D166" t="s">
         <v>218</v>
@@ -70387,13 +70387,13 @@
         <v>1</v>
       </c>
       <c r="C167" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D167" t="s">
         <v>218</v>
       </c>
       <c r="E167" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F167" t="s">
         <v>219</v>
@@ -70800,10 +70800,10 @@
         <v>1</v>
       </c>
       <c r="C168" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D168" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="E168" t="s">
         <v>218</v>
@@ -71207,7 +71207,7 @@
         <v>1</v>
       </c>
       <c r="C169" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D169" t="s">
         <v>218</v>
@@ -71614,13 +71614,13 @@
         <v>1</v>
       </c>
       <c r="C170" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D170" t="s">
         <v>218</v>
       </c>
       <c r="E170" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F170" t="s">
         <v>215</v>
@@ -72027,7 +72027,7 @@
         <v>1</v>
       </c>
       <c r="C171" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D171" t="s">
         <v>218</v>
@@ -72036,7 +72036,7 @@
         <v>218</v>
       </c>
       <c r="F171" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G171">
         <v>40</v>
@@ -72440,13 +72440,13 @@
         <v>1</v>
       </c>
       <c r="C172" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D172" t="s">
         <v>218</v>
       </c>
       <c r="E172" t="s">
-        <v>310</v>
+        <v>309</v>
       </c>
       <c r="F172" t="s">
         <v>219</v>
@@ -72853,16 +72853,16 @@
         <v>1</v>
       </c>
       <c r="C173" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D173" t="s">
         <v>218</v>
       </c>
       <c r="E173" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F173" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G173">
         <v>96</v>
@@ -73260,10 +73260,10 @@
         <v>1</v>
       </c>
       <c r="C174" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D174" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E174" t="s">
         <v>218</v>
@@ -73673,16 +73673,16 @@
         <v>1</v>
       </c>
       <c r="C175" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D175" t="s">
         <v>218</v>
       </c>
       <c r="E175" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F175" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G175">
         <v>49</v>
@@ -74080,16 +74080,16 @@
         <v>1</v>
       </c>
       <c r="C176" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D176" t="s">
         <v>218</v>
       </c>
       <c r="E176" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F176" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G176">
         <v>61</v>
@@ -74487,7 +74487,7 @@
         <v>1</v>
       </c>
       <c r="C177" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D177" t="s">
         <v>218</v>
@@ -74496,7 +74496,7 @@
         <v>176</v>
       </c>
       <c r="F177" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G177">
         <v>146</v>
@@ -74900,7 +74900,7 @@
         <v>1</v>
       </c>
       <c r="C178" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D178" t="s">
         <v>218</v>
@@ -75313,10 +75313,10 @@
         <v>1</v>
       </c>
       <c r="C179" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D179" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E179" t="s">
         <v>218</v>
@@ -75726,16 +75726,16 @@
         <v>1</v>
       </c>
       <c r="C180" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D180" t="s">
         <v>218</v>
       </c>
       <c r="E180" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F180" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G180">
         <v>34</v>
@@ -76139,13 +76139,13 @@
         <v>1</v>
       </c>
       <c r="C181" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D181" t="s">
         <v>218</v>
       </c>
       <c r="E181" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="F181" t="s">
         <v>222</v>
@@ -76552,7 +76552,7 @@
         <v>1</v>
       </c>
       <c r="C182" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D182" t="s">
         <v>218</v>
@@ -76959,13 +76959,13 @@
         <v>1</v>
       </c>
       <c r="C183" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D183" t="s">
         <v>218</v>
       </c>
       <c r="E183" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F183" t="s">
         <v>222</v>
@@ -77372,10 +77372,10 @@
         <v>1</v>
       </c>
       <c r="C184" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D184" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E184" t="s">
         <v>218</v>
@@ -77779,10 +77779,10 @@
         <v>1</v>
       </c>
       <c r="C185" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D185" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E185" t="s">
         <v>218</v>
@@ -78186,7 +78186,7 @@
         <v>1</v>
       </c>
       <c r="C186" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D186" t="s">
         <v>218</v>
@@ -78593,16 +78593,16 @@
         <v>1</v>
       </c>
       <c r="C187" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D187" t="s">
         <v>218</v>
       </c>
       <c r="E187" t="s">
-        <v>313</v>
+        <v>312</v>
       </c>
       <c r="F187" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G187">
         <v>382</v>
@@ -79006,10 +79006,10 @@
         <v>1</v>
       </c>
       <c r="C188" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D188" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E188" t="s">
         <v>218</v>
@@ -79419,16 +79419,16 @@
         <v>1</v>
       </c>
       <c r="C189" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D189" t="s">
         <v>218</v>
       </c>
       <c r="E189" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F189" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G189">
         <v>163</v>
@@ -79832,7 +79832,7 @@
         <v>1</v>
       </c>
       <c r="C190" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D190" t="s">
         <v>218</v>
@@ -80239,7 +80239,7 @@
         <v>1</v>
       </c>
       <c r="C191" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D191" t="s">
         <v>218</v>
@@ -80652,16 +80652,16 @@
         <v>1</v>
       </c>
       <c r="C192" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D192" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E192" t="s">
         <v>218</v>
       </c>
       <c r="F192" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G192">
         <v>155</v>
@@ -81059,7 +81059,7 @@
         <v>1</v>
       </c>
       <c r="C193" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D193" t="s">
         <v>218</v>
@@ -81466,13 +81466,13 @@
         <v>1</v>
       </c>
       <c r="C194" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D194" t="s">
         <v>218</v>
       </c>
       <c r="E194" t="s">
-        <v>325</v>
+        <v>324</v>
       </c>
       <c r="F194" t="s">
         <v>222</v>
@@ -81879,7 +81879,7 @@
         <v>1</v>
       </c>
       <c r="C195" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D195" t="s">
         <v>218</v>
@@ -82286,7 +82286,7 @@
         <v>1</v>
       </c>
       <c r="C196" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D196" t="s">
         <v>218</v>
@@ -82699,7 +82699,7 @@
         <v>1</v>
       </c>
       <c r="C197" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D197" t="s">
         <v>218</v>
@@ -83112,10 +83112,10 @@
         <v>1</v>
       </c>
       <c r="C198" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D198" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E198" t="s">
         <v>218</v>
@@ -83525,13 +83525,13 @@
         <v>1</v>
       </c>
       <c r="C199" t="s">
-        <v>337</v>
+        <v>336</v>
       </c>
       <c r="D199" t="s">
         <v>218</v>
       </c>
       <c r="E199" t="s">
-        <v>308</v>
+        <v>307</v>
       </c>
       <c r="F199" t="s">
         <v>215</v>
@@ -83938,13 +83938,13 @@
         <v>1</v>
       </c>
       <c r="C200" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D200" t="s">
         <v>218</v>
       </c>
       <c r="E200" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F200" t="s">
         <v>219</v>
@@ -84345,7 +84345,7 @@
         <v>1</v>
       </c>
       <c r="C201" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D201" t="s">
         <v>218</v>
@@ -84752,10 +84752,10 @@
         <v>1</v>
       </c>
       <c r="C202" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D202" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="E202" t="s">
         <v>218</v>
@@ -85165,10 +85165,10 @@
         <v>1</v>
       </c>
       <c r="C203" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D203" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E203" t="s">
         <v>218</v>
@@ -85578,7 +85578,7 @@
         <v>1</v>
       </c>
       <c r="C204" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D204" t="s">
         <v>218</v>
@@ -85991,13 +85991,13 @@
         <v>1</v>
       </c>
       <c r="C205" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D205" t="s">
         <v>218</v>
       </c>
       <c r="E205" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="F205" t="s">
         <v>222</v>
@@ -86398,10 +86398,10 @@
         <v>1</v>
       </c>
       <c r="C206" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D206" t="s">
-        <v>333</v>
+        <v>332</v>
       </c>
       <c r="E206" t="s">
         <v>218</v>
@@ -86811,10 +86811,10 @@
         <v>1</v>
       </c>
       <c r="C207" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D207" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E207" t="s">
         <v>218</v>
@@ -87224,13 +87224,13 @@
         <v>1</v>
       </c>
       <c r="C208" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D208" t="s">
         <v>218</v>
       </c>
       <c r="E208" t="s">
-        <v>323</v>
+        <v>322</v>
       </c>
       <c r="F208" t="s">
         <v>219</v>
@@ -87637,10 +87637,10 @@
         <v>1</v>
       </c>
       <c r="C209" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D209" t="s">
-        <v>329</v>
+        <v>328</v>
       </c>
       <c r="E209" t="s">
         <v>218</v>
@@ -88050,7 +88050,7 @@
         <v>1</v>
       </c>
       <c r="C210" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D210" t="s">
         <v>218</v>
@@ -88059,7 +88059,7 @@
         <v>176</v>
       </c>
       <c r="F210" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G210">
         <v>164</v>
@@ -88463,10 +88463,10 @@
         <v>1</v>
       </c>
       <c r="C211" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D211" t="s">
-        <v>330</v>
+        <v>329</v>
       </c>
       <c r="E211" t="s">
         <v>218</v>
@@ -88870,7 +88870,7 @@
         <v>1</v>
       </c>
       <c r="C212" t="s">
-        <v>340</v>
+        <v>339</v>
       </c>
       <c r="D212" t="s">
         <v>218</v>
@@ -88879,7 +88879,7 @@
         <v>176</v>
       </c>
       <c r="F212" t="s">
-        <v>306</v>
+        <v>305</v>
       </c>
       <c r="G212">
         <v>49</v>
@@ -89283,16 +89283,16 @@
         <v>1</v>
       </c>
       <c r="C213" t="s">
-        <v>339</v>
+        <v>338</v>
       </c>
       <c r="D213" t="s">
-        <v>332</v>
+        <v>331</v>
       </c>
       <c r="E213" t="s">
         <v>218</v>
       </c>
       <c r="F213" t="s">
-        <v>305</v>
+        <v>304</v>
       </c>
       <c r="G213">
         <v>43</v>
@@ -89690,16 +89690,16 @@
         <v>1</v>
       </c>
       <c r="C214" t="s">
-        <v>338</v>
+        <v>337</v>
       </c>
       <c r="D214" t="s">
         <v>218</v>
       </c>
       <c r="E214" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="F214" t="s">
-        <v>307</v>
+        <v>306</v>
       </c>
       <c r="G214">
         <v>164</v>

</xml_diff>